<commit_message>
Improved dashboard visual design
- Two-column responsive layout + horizontal dividers

- Consistent color palette
</commit_message>
<xml_diff>
--- a/backend/Rwanda/financial-statements-CleanStep.xlsx
+++ b/backend/Rwanda/financial-statements-CleanStep.xlsx
@@ -2506,34 +2506,34 @@
         <v>0</v>
       </c>
       <c r="F37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="19" t="n">
         <v>-45.48</v>
       </c>
-      <c r="G37" s="19" t="n">
+      <c r="H37" s="19" t="n">
         <v>-136.44</v>
       </c>
-      <c r="H37" s="19" t="n">
+      <c r="I37" s="19" t="n">
         <v>-227.4</v>
       </c>
-      <c r="I37" s="19" t="n">
+      <c r="J37" s="19" t="n">
         <v>-318.36</v>
       </c>
-      <c r="J37" s="19" t="n">
+      <c r="K37" s="19" t="n">
         <v>-409.3199999999999</v>
       </c>
-      <c r="K37" s="19" t="n">
+      <c r="L37" s="19" t="n">
         <v>-500.2799999999999</v>
       </c>
-      <c r="L37" s="19" t="n">
+      <c r="M37" s="19" t="n">
         <v>-591.2399999999999</v>
       </c>
-      <c r="M37" s="19" t="n">
+      <c r="N37" s="19" t="n">
         <v>-682.1999999999999</v>
       </c>
-      <c r="N37" s="19" t="n">
+      <c r="O37" s="19" t="n">
         <v>-773.16</v>
-      </c>
-      <c r="O37" s="19" t="n">
-        <v>-864.12</v>
       </c>
     </row>
     <row r="38" ht="15.5" customHeight="1">
@@ -2821,37 +2821,37 @@
         <v>-273.9964236684048</v>
       </c>
       <c r="E43" s="18" t="n">
-        <v>-547.5645208596383</v>
+        <v>-546.9928473368097</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>-28.91237241151316</v>
+        <v>-1015.428796079918</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>-605.3365675262133</v>
+        <v>-787.3729911946183</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>-1253.133747502193</v>
+        <v>-1630.038022722473</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>-1567.49648555585</v>
+        <v>-2234.997104338955</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>-1464.45115053207</v>
+        <v>-2398.19260572833</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>-1253.055247028271</v>
+        <v>-2143.958603865033</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>-1041.642200685596</v>
+        <v>-1781.378320858076</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>-830.2376861422772</v>
+        <v>-1418.78513947524</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>-656.8710359808772</v>
+        <v>-1094.234109810682</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>-633.6845208596383</v>
+        <v>-919.8674596492822</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -2874,37 +2874,37 @@
         <v>-273.9964236684048</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>-547.5645208596383</v>
+        <v>-546.9928473368097</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>-28.91237241151316</v>
+        <v>-1015.428796079918</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>-605.3365675262133</v>
+        <v>-787.3729911946183</v>
       </c>
       <c r="H44" s="18" t="n">
-        <v>-1253.133747502193</v>
+        <v>-1630.038022722473</v>
       </c>
       <c r="I44" s="18" t="n">
-        <v>-1567.49648555585</v>
+        <v>-2234.997104338955</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>-1464.45115053207</v>
+        <v>-2398.19260572833</v>
       </c>
       <c r="K44" s="18" t="n">
-        <v>-1253.055247028271</v>
+        <v>-2143.958603865033</v>
       </c>
       <c r="L44" s="18" t="n">
-        <v>-1041.642200685596</v>
+        <v>-1781.378320858076</v>
       </c>
       <c r="M44" s="18" t="n">
-        <v>-830.2376861422772</v>
+        <v>-1418.78513947524</v>
       </c>
       <c r="N44" s="18" t="n">
-        <v>-656.8710359808772</v>
+        <v>-1094.234109810682</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>-633.6845208596383</v>
+        <v>-919.8674596492822</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -3033,37 +3033,37 @@
         <v>-273.9964236684048</v>
       </c>
       <c r="E47" s="18" t="n">
-        <v>-547.5645208596383</v>
+        <v>-546.9928473368097</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>-28.91237241151316</v>
+        <v>-1015.428796079918</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>-605.3365675262133</v>
+        <v>-787.3729911946183</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>-1253.133747502193</v>
+        <v>-1630.038022722473</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>-1567.49648555585</v>
+        <v>-2234.997104338955</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>-1464.45115053207</v>
+        <v>-2398.19260572833</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>-1253.055247028271</v>
+        <v>-2143.958603865033</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>-1041.642200685596</v>
+        <v>-1781.378320858076</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>-830.2376861422772</v>
+        <v>-1418.78513947524</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>-656.8710359808772</v>
+        <v>-1094.234109810682</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>-633.6845208596383</v>
+        <v>-919.8674596492822</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -3092,31 +3092,31 @@
         <v>-355.0763073598987</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>-888.020502474599</v>
+        <v>-842.540502474599</v>
       </c>
       <c r="H48" s="18" t="n">
-        <v>-1733.685534002453</v>
+        <v>-1642.725534002453</v>
       </c>
       <c r="I48" s="18" t="n">
-        <v>-2341.644615618935</v>
+        <v>-2446.55246717081</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>-2507.84011700831</v>
+        <v>-2904.344312123009</v>
       </c>
       <c r="K48" s="18" t="n">
-        <v>-2256.606115145014</v>
+        <v>-2920.351146672868</v>
       </c>
       <c r="L48" s="18" t="n">
-        <v>-1897.025832138057</v>
+        <v>-2518.932765306414</v>
       </c>
       <c r="M48" s="18" t="n">
+        <v>-2009.172347259296</v>
+      </c>
+      <c r="N48" s="18" t="n">
         <v>-1537.432650755221</v>
       </c>
-      <c r="N48" s="18" t="n">
+      <c r="O48" s="18" t="n">
         <v>-1215.881621090663</v>
-      </c>
-      <c r="O48" s="18" t="n">
-        <v>-1044.514970929263</v>
       </c>
     </row>
     <row r="49" ht="15.5" customHeight="1">
@@ -3251,31 +3251,31 @@
         <v>0</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>-241.3478515518748</v>
+        <v>-195.8678515518748</v>
       </c>
       <c r="H51" s="18" t="n">
-        <v>-819.7720466665751</v>
+        <v>-728.812046666575</v>
       </c>
       <c r="I51" s="18" t="n">
-        <v>-1469.569226642554</v>
+        <v>-1574.477078194429</v>
       </c>
       <c r="J51" s="18" t="n">
-        <v>-1785.931964696211</v>
+        <v>-2182.436159810911</v>
       </c>
       <c r="K51" s="18" t="n">
-        <v>-1684.886629672432</v>
+        <v>-2348.631661200286</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>-1475.490726168633</v>
+        <v>-2097.39765933699</v>
       </c>
       <c r="M51" s="18" t="n">
-        <v>-1266.077679825958</v>
+        <v>-1737.817376330033</v>
       </c>
       <c r="N51" s="18" t="n">
+        <v>-1378.224194947197</v>
+      </c>
+      <c r="O51" s="18" t="n">
         <v>-1056.673165282639</v>
-      </c>
-      <c r="O51" s="18" t="n">
-        <v>-885.3065151212389</v>
       </c>
     </row>
     <row r="52" ht="15.5" customHeight="1">
@@ -3301,34 +3301,34 @@
         <v>3</v>
       </c>
       <c r="F52" s="18" t="n">
-        <v>763</v>
+        <v>6</v>
       </c>
       <c r="G52" s="18" t="n">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="H52" s="18" t="n">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="I52" s="18" t="n">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="J52" s="18" t="n">
-        <v>771</v>
+        <v>776</v>
       </c>
       <c r="K52" s="18" t="n">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="L52" s="18" t="n">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="M52" s="18" t="n">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="N52" s="18" t="n">
-        <v>779</v>
+        <v>788</v>
       </c>
       <c r="O52" s="18" t="n">
-        <v>781</v>
+        <v>791</v>
       </c>
     </row>
     <row r="53" ht="15.5" customHeight="1">
@@ -3407,34 +3407,34 @@
         <v>3</v>
       </c>
       <c r="F54" s="18" t="n">
-        <v>763</v>
+        <v>6</v>
       </c>
       <c r="G54" s="18" t="n">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="H54" s="18" t="n">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="I54" s="18" t="n">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="J54" s="18" t="n">
-        <v>771</v>
+        <v>776</v>
       </c>
       <c r="K54" s="18" t="n">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="L54" s="18" t="n">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="M54" s="18" t="n">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="N54" s="18" t="n">
-        <v>779</v>
+        <v>788</v>
       </c>
       <c r="O54" s="18" t="n">
-        <v>781</v>
+        <v>791</v>
       </c>
     </row>
     <row r="55" ht="15.5" customHeight="1">
@@ -3619,34 +3619,34 @@
         <v>-156.2084558080239</v>
       </c>
       <c r="F58" s="18" t="n">
-        <v>407.9236926401013</v>
+        <v>-349.0763073598987</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>-123.020502474599</v>
+        <v>-75.54050247459895</v>
       </c>
       <c r="H58" s="18" t="n">
-        <v>-966.6855340024533</v>
+        <v>-872.7255340024533</v>
       </c>
       <c r="I58" s="18" t="n">
-        <v>-1572.644615618935</v>
+        <v>-1673.55246717081</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>-1736.84011700831</v>
+        <v>-2128.344312123009</v>
       </c>
       <c r="K58" s="18" t="n">
-        <v>-1483.606115145014</v>
+        <v>-2141.351146672868</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>-1122.025832138057</v>
+        <v>-1736.932765306414</v>
       </c>
       <c r="M58" s="18" t="n">
-        <v>-760.4326507552209</v>
+        <v>-1224.172347259296</v>
       </c>
       <c r="N58" s="18" t="n">
-        <v>-436.8816210906627</v>
+        <v>-749.4326507552209</v>
       </c>
       <c r="O58" s="18" t="n">
-        <v>-263.5149709292627</v>
+        <v>-424.881621090663</v>
       </c>
     </row>
     <row r="59" ht="15.5" customHeight="1">
@@ -3669,37 +3669,37 @@
         <v>-115.7879678603809</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>-391.3560650516143</v>
+        <v>-390.7843915287858</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>-436.8360650516145</v>
+        <v>-666.3524887200192</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>-482.3160650516144</v>
+        <v>-711.8324887200193</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>-286.4482134997397</v>
+        <v>-757.3124887200195</v>
       </c>
       <c r="I59" s="18" t="n">
-        <v>5.148130063085318</v>
+        <v>-561.4446371681447</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>272.3889664762396</v>
+        <v>-269.8482936053206</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>230.550868116743</v>
+        <v>-2.607457192164929</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>80.38363145246058</v>
+        <v>-44.44555555166198</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>-69.80503538705625</v>
+        <v>-194.6127922159437</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>-219.9894148902144</v>
+        <v>-344.8014590554612</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>-370.1695499303755</v>
+        <v>-494.9858385586192</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -4573,34 +4573,34 @@
         <v>-273.9964236684048</v>
       </c>
       <c r="F76" s="18" t="n">
-        <v>-547.5645208596383</v>
+        <v>-546.9928473368097</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>-28.91237241151316</v>
+        <v>-1015.428796079918</v>
       </c>
       <c r="H76" s="18" t="n">
-        <v>-605.3365675262133</v>
+        <v>-787.3729911946183</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>-1253.133747502193</v>
+        <v>-1630.038022722473</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>-1567.49648555585</v>
+        <v>-2234.997104338955</v>
       </c>
       <c r="K76" s="18" t="n">
-        <v>-1464.45115053207</v>
+        <v>-2398.19260572833</v>
       </c>
       <c r="L76" s="18" t="n">
-        <v>-1253.055247028271</v>
+        <v>-2143.958603865033</v>
       </c>
       <c r="M76" s="18" t="n">
-        <v>-1041.642200685596</v>
+        <v>-1781.378320858076</v>
       </c>
       <c r="N76" s="18" t="n">
-        <v>-830.2376861422772</v>
+        <v>-1418.78513947524</v>
       </c>
       <c r="O76" s="18" t="n">
-        <v>-656.8710359808772</v>
+        <v>-1094.234109810682</v>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
@@ -4676,37 +4676,37 @@
         <v>-273.9964236684048</v>
       </c>
       <c r="E78" s="18" t="n">
-        <v>-547.5645208596383</v>
+        <v>-546.9928473368097</v>
       </c>
       <c r="F78" s="18" t="n">
-        <v>-28.91237241151316</v>
+        <v>-1015.428796079918</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>-605.3365675262133</v>
+        <v>-787.3729911946183</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>-1253.133747502193</v>
+        <v>-1630.038022722473</v>
       </c>
       <c r="I78" s="18" t="n">
-        <v>-1567.49648555585</v>
+        <v>-2234.997104338955</v>
       </c>
       <c r="J78" s="18" t="n">
-        <v>-1464.45115053207</v>
+        <v>-2398.19260572833</v>
       </c>
       <c r="K78" s="18" t="n">
-        <v>-1253.055247028271</v>
+        <v>-2143.958603865033</v>
       </c>
       <c r="L78" s="18" t="n">
-        <v>-1041.642200685596</v>
+        <v>-1781.378320858076</v>
       </c>
       <c r="M78" s="18" t="n">
-        <v>-830.2376861422772</v>
+        <v>-1418.78513947524</v>
       </c>
       <c r="N78" s="18" t="n">
-        <v>-656.8710359808772</v>
+        <v>-1094.234109810682</v>
       </c>
       <c r="O78" s="18" t="n">
-        <v>-633.6845208596383</v>
+        <v>-919.8674596492822</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -5657,34 +5657,34 @@
         <v>761.5749464668912</v>
       </c>
       <c r="F96" s="20" t="n">
-        <v>842.2036917224142</v>
+        <v>842.5346606040516</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>-319.9275621043757</v>
+        <v>487.1273843625155</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>-1138.51992716426</v>
+        <v>-966.6002130270998</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>-1788.31710714024</v>
+        <v>-2052.433414500138</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>-2104.679845193897</v>
+        <v>-2660.392496116621</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>-2003.634510170117</v>
+        <v>-2826.587997505996</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>-1794.238606666318</v>
+        <v>-2575.353995642699</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>-1584.825560323643</v>
+        <v>-2215.773712635742</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>-1375.421045780324</v>
+        <v>-1856.180531252906</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>-1127.995559817816</v>
+        <v>-1458.57066578724</v>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
@@ -5866,37 +5866,37 @@
         <v>761.5749464668912</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>842.2036917224142</v>
+        <v>842.5346606040516</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>-319.9275621043757</v>
+        <v>487.1273843625155</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>-1138.51992716426</v>
+        <v>-966.6002130270998</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>-1788.31710714024</v>
+        <v>-2052.433414500138</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>-2104.679845193897</v>
+        <v>-2660.392496116621</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>-2003.634510170117</v>
+        <v>-2826.587997505996</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>-1794.238606666318</v>
+        <v>-2575.353995642699</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>-1584.825560323643</v>
+        <v>-2215.773712635742</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>-1375.421045780324</v>
+        <v>-1856.180531252906</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>-1127.995559817816</v>
+        <v>-1458.57066578724</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>-730.4479070615439</v>
+        <v>-910.8428779908063</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -6296,31 +6296,31 @@
         <v>3</v>
       </c>
       <c r="G108" s="18" t="n">
-        <v>763</v>
+        <v>6</v>
       </c>
       <c r="H108" s="18" t="n">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="I108" s="18" t="n">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="J108" s="18" t="n">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="K108" s="18" t="n">
-        <v>771</v>
+        <v>776</v>
       </c>
       <c r="L108" s="18" t="n">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="M108" s="18" t="n">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="N108" s="18" t="n">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="O108" s="18" t="n">
-        <v>779</v>
+        <v>788</v>
       </c>
     </row>
     <row r="109" ht="15.5" customHeight="1">
@@ -6452,34 +6452,34 @@
         <v>3</v>
       </c>
       <c r="F111" s="18" t="n">
-        <v>763</v>
+        <v>6</v>
       </c>
       <c r="G111" s="18" t="n">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="H111" s="18" t="n">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="I111" s="18" t="n">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="J111" s="18" t="n">
-        <v>771</v>
+        <v>776</v>
       </c>
       <c r="K111" s="18" t="n">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="L111" s="18" t="n">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="M111" s="18" t="n">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="N111" s="18" t="n">
-        <v>779</v>
+        <v>788</v>
       </c>
       <c r="O111" s="18" t="n">
-        <v>781</v>
+        <v>791</v>
       </c>
     </row>
     <row r="112" ht="15.5" customHeight="1">
@@ -8776,7 +8776,7 @@
         <v>4627.282008722714</v>
       </c>
       <c r="O41" s="18" t="n">
-        <v>4206.583225413329</v>
+        <v>4818.436049145901</v>
       </c>
     </row>
     <row r="42" ht="15.5" customHeight="1">
@@ -8829,7 +8829,7 @@
         <v>4627.282008722714</v>
       </c>
       <c r="O42" s="18" t="n">
-        <v>4206.583225413329</v>
+        <v>4818.436049145901</v>
       </c>
     </row>
     <row r="43" ht="15.5" customHeight="1">
@@ -8882,7 +8882,7 @@
         <v>135.9230875941853</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>-145.2932861724019</v>
+        <v>138.003837047472</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -8935,7 +8935,7 @@
         <v>14</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>-269.2971232198739</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -9094,7 +9094,7 @@
         <v>4763.205096316899</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>4061.289939240927</v>
+        <v>4956.439886193373</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -9138,10 +9138,10 @@
         <v>3996.528176865003</v>
       </c>
       <c r="L48" s="18" t="n">
-        <v>4377.04364257835</v>
+        <v>4306.578867276742</v>
       </c>
       <c r="M48" s="18" t="n">
-        <v>4578.386145566312</v>
+        <v>4648.85092086792</v>
       </c>
       <c r="N48" s="18" t="n">
         <v>4811.950101719302</v>
@@ -9297,10 +9297,10 @@
         <v>3648.168091378179</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>4066.992952166611</v>
+        <v>3996.528176865003</v>
       </c>
       <c r="M51" s="18" t="n">
-        <v>4306.578867276742</v>
+        <v>4377.04364257835</v>
       </c>
       <c r="N51" s="18" t="n">
         <v>4578.386145566312</v>
@@ -9668,10 +9668,10 @@
         <v>3938.440612974634</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>4316.873200576842</v>
+        <v>4246.408425275234</v>
       </c>
       <c r="M58" s="18" t="n">
-        <v>4516.133546566795</v>
+        <v>4586.598321868403</v>
       </c>
       <c r="N58" s="18" t="n">
         <v>4745.616055221008</v>
@@ -9721,16 +9721,16 @@
         <v>15.58904109589093</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>-54.87573420571698</v>
+        <v>15.58904109589093</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>15.58904109589184</v>
+        <v>-54.87573420571607</v>
       </c>
       <c r="N59" s="18" t="n">
         <v>17.58904109589184</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>-874.5609058565551</v>
+        <v>20.58904109589093</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -10737,7 +10737,7 @@
         <v>14</v>
       </c>
       <c r="O78" s="18" t="n">
-        <v>-269.2971232198739</v>
+        <v>14</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -11108,7 +11108,7 @@
         <v>4627.282008722714</v>
       </c>
       <c r="O85" s="18" t="n">
-        <v>4206.583225413329</v>
+        <v>4818.436049145901</v>
       </c>
     </row>
     <row r="86" ht="15.5" customHeight="1">
@@ -11706,10 +11706,10 @@
         <v>18459.51422057945</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>21665.85122419476</v>
+        <v>21736.31599949639</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>25152.88362848072</v>
+        <v>25082.41885317909</v>
       </c>
       <c r="N96" s="20" t="n">
         <v>28709.12115268048</v>
@@ -11915,10 +11915,10 @@
         <v>18459.51422057945</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>21665.85122419476</v>
+        <v>21736.31599949639</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>25152.88362848072</v>
+        <v>25082.41885317909</v>
       </c>
       <c r="M100" s="20" t="n">
         <v>28709.12115268048</v>
@@ -11927,7 +11927,7 @@
         <v>32404.99899420075</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>36069.03589658669</v>
+        <v>36240.49420498676</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -14568,34 +14568,34 @@
         <v>-10.584</v>
       </c>
       <c r="F37" s="19" t="n">
-        <v>-15.274</v>
+        <v>-19.594</v>
       </c>
       <c r="G37" s="19" t="n">
-        <v>-20.946</v>
+        <v>-27.186</v>
       </c>
       <c r="H37" s="19" t="n">
-        <v>-27.01933333333334</v>
+        <v>-35.83933333333334</v>
       </c>
       <c r="I37" s="19" t="n">
-        <v>-33.684</v>
+        <v>-45.03400000000001</v>
       </c>
       <c r="J37" s="19" t="n">
-        <v>-40.64733333333334</v>
+        <v>-54.48733333333333</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>-45.93666666666666</v>
+        <v>-62.20666666666668</v>
       </c>
       <c r="L37" s="19" t="n">
-        <v>-49.192</v>
+        <v>-67.84199999999998</v>
       </c>
       <c r="M37" s="19" t="n">
-        <v>-52.03333333333333</v>
+        <v>-71.43333333333334</v>
       </c>
       <c r="N37" s="19" t="n">
-        <v>-54.87066666666666</v>
+        <v>-74.61066666666666</v>
       </c>
       <c r="O37" s="19" t="n">
-        <v>-57.69333333333333</v>
+        <v>-77.76333333333332</v>
       </c>
     </row>
     <row r="38" ht="15.5" customHeight="1">
@@ -14886,34 +14886,34 @@
         <v>0.5519529271896613</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>4.789570936428327</v>
+        <v>4.872312952428326</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>9.721677720917388</v>
+        <v>9.879931955992507</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>16.04774380171231</v>
+        <v>16.35176849320063</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>24.58991837021113</v>
+        <v>25.00580878117003</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>22.78411935783657</v>
+        <v>23.19343442632972</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>20.90041037483058</v>
+        <v>21.29986242962509</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>18.99733483624383</v>
+        <v>19.38856771295618</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>17.3672748084873</v>
+        <v>17.49056247972017</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>15.81043236270174</v>
+        <v>15.86632277366065</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>14.26727646565449</v>
+        <v>14.32152304099695</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -14939,34 +14939,34 @@
         <v>1.064829639518428</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>5.514502443277642</v>
+        <v>5.597244459277642</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>10.65455443324615</v>
+        <v>10.81280866832127</v>
       </c>
       <c r="H44" s="18" t="n">
-        <v>17.18527804828765</v>
+        <v>17.48930273977597</v>
       </c>
       <c r="I44" s="18" t="n">
-        <v>25.92717864418373</v>
+        <v>26.34306905514263</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>24.31699607016533</v>
+        <v>24.72631113865848</v>
       </c>
       <c r="K44" s="18" t="n">
-        <v>22.49493092277579</v>
+        <v>22.8943829775703</v>
       </c>
       <c r="L44" s="18" t="n">
-        <v>20.61980058966849</v>
+        <v>21.01103346638084</v>
       </c>
       <c r="M44" s="18" t="n">
-        <v>19.01686384958319</v>
+        <v>19.14015152081606</v>
       </c>
       <c r="N44" s="18" t="n">
-        <v>17.48714469146886</v>
+        <v>17.54303510242777</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>15.9694682464764</v>
+        <v>16.02371482181886</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -15098,34 +15098,34 @@
         <v>0.7979529271896613</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>5.185570936428327</v>
+        <v>5.268312952428326</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>10.25567772091739</v>
+        <v>10.41393195599251</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>16.69841046837897</v>
+        <v>17.00243515986729</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>25.34591837021113</v>
+        <v>25.76180878117003</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>23.59678602450323</v>
+        <v>24.00610109299638</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>21.72374370816392</v>
+        <v>22.12319576295842</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>19.82533483624383</v>
+        <v>20.21656771295618</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>18.19394147515397</v>
+        <v>18.31722914638684</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>16.62976569603507</v>
+        <v>16.68565610699398</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>15.06394313232115</v>
+        <v>15.11818970766361</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -15154,13 +15154,13 @@
         <v>-1.20696931622679</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>-1.304934392542375</v>
+        <v>-1.932329362843744</v>
       </c>
       <c r="H48" s="18" t="n">
-        <v>-2.339394754096205</v>
+        <v>-2.496756957377249</v>
       </c>
       <c r="I48" s="18" t="n">
-        <v>-4.08956004068785</v>
+        <v>-4.209644938240621</v>
       </c>
       <c r="J48" s="18" t="n">
         <v>-6.311502661143089</v>
@@ -15313,13 +15313,13 @@
         <v>-1.099794986071236</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>-0.9598706457534301</v>
+        <v>-1.5872656160548</v>
       </c>
       <c r="H51" s="18" t="n">
-        <v>-1.52786848908934</v>
+        <v>-1.685230692370385</v>
       </c>
       <c r="I51" s="18" t="n">
-        <v>-2.599606156371443</v>
+        <v>-2.719691053924215</v>
       </c>
       <c r="J51" s="18" t="n">
         <v>-4.46985634051586</v>
@@ -15328,7 +15328,7 @@
         <v>-6.691798960971099</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>-8.866128398362793</v>
+        <v>-8.86612839836279</v>
       </c>
       <c r="M51" s="18" t="n">
         <v>-11.04034493928043</v>
@@ -15684,13 +15684,13 @@
         <v>3.517962190622525</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>8.627942319786392</v>
+        <v>8.000547349485023</v>
       </c>
       <c r="H58" s="18" t="n">
-        <v>14.79813949247914</v>
+        <v>14.64077728919809</v>
       </c>
       <c r="I58" s="18" t="n">
-        <v>23.24770023328475</v>
+        <v>23.12761533573198</v>
       </c>
       <c r="J58" s="18" t="n">
         <v>21.22137405118568</v>
@@ -15734,34 +15734,34 @@
         <v>1.00457490110412</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>1.667608745805802</v>
+        <v>1.750350761805801</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>1.627735401130996</v>
+        <v>2.413384606507485</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>1.900270975899836</v>
+        <v>2.3616578706692</v>
       </c>
       <c r="I59" s="18" t="n">
-        <v>2.098218136926377</v>
+        <v>2.634193445438047</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>2.375411973317551</v>
+        <v>2.784727041810701</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>2.61505525875349</v>
+        <v>3.014507313547998</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>2.862917722271593</v>
+        <v>3.254150598983941</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>3.378725391269176</v>
+        <v>3.502013062502046</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>3.961930320540709</v>
+        <v>4.017820731499619</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>4.534925694265228</v>
+        <v>4.589172269607687</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -16638,31 +16638,31 @@
         <v>1.064829639518428</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>5.514502443277642</v>
+        <v>5.597244459277642</v>
       </c>
       <c r="H76" s="18" t="n">
-        <v>10.65455443324615</v>
+        <v>10.81280866832127</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>17.18527804828765</v>
+        <v>17.48930273977597</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>25.92717864418373</v>
+        <v>26.34306905514263</v>
       </c>
       <c r="K76" s="18" t="n">
-        <v>24.31699607016533</v>
+        <v>24.72631113865848</v>
       </c>
       <c r="L76" s="18" t="n">
-        <v>22.49493092277579</v>
+        <v>22.8943829775703</v>
       </c>
       <c r="M76" s="18" t="n">
-        <v>20.61980058966849</v>
+        <v>21.01103346638084</v>
       </c>
       <c r="N76" s="18" t="n">
-        <v>19.01686384958319</v>
+        <v>19.14015152081606</v>
       </c>
       <c r="O76" s="18" t="n">
-        <v>17.48714469146886</v>
+        <v>17.54303510242777</v>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
@@ -16741,34 +16741,34 @@
         <v>1.064829639518428</v>
       </c>
       <c r="F78" s="18" t="n">
-        <v>5.514502443277642</v>
+        <v>5.597244459277642</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>10.65455443324615</v>
+        <v>10.81280866832127</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>17.18527804828765</v>
+        <v>17.48930273977597</v>
       </c>
       <c r="I78" s="18" t="n">
-        <v>25.92717864418373</v>
+        <v>26.34306905514263</v>
       </c>
       <c r="J78" s="18" t="n">
-        <v>24.31699607016533</v>
+        <v>24.72631113865848</v>
       </c>
       <c r="K78" s="18" t="n">
-        <v>22.49493092277579</v>
+        <v>22.8943829775703</v>
       </c>
       <c r="L78" s="18" t="n">
-        <v>20.61980058966849</v>
+        <v>21.01103346638084</v>
       </c>
       <c r="M78" s="18" t="n">
-        <v>19.01686384958319</v>
+        <v>19.14015152081606</v>
       </c>
       <c r="N78" s="18" t="n">
-        <v>17.48714469146886</v>
+        <v>17.54303510242777</v>
       </c>
       <c r="O78" s="18" t="n">
-        <v>15.9694682464764</v>
+        <v>16.02371482181886</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -17722,13 +17722,13 @@
         <v>1.230311960749614</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>0.7359124553982314</v>
+        <v>1.363307425699603</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>0.2334865053282429</v>
+        <v>0.3908487086092867</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>-0.6981246572313926</v>
+        <v>-0.5780397596786215</v>
       </c>
       <c r="J96" s="20" t="n">
         <v>-2.188078541547799</v>
@@ -17737,13 +17737,13 @@
         <v>-4.029724862175027</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>-5.823757999738711</v>
+        <v>-5.823757999738709</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>-7.61767824082834</v>
+        <v>-7.617678240828338</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>-9.411706258759011</v>
+        <v>-9.411706258759009</v>
       </c>
       <c r="O96" s="20" t="n">
         <v>-11.20591395499266</v>
@@ -17931,13 +17931,13 @@
         <v>1.230311960749614</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>0.7359124553982314</v>
+        <v>1.363307425699603</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>0.2334865053282429</v>
+        <v>0.3908487086092867</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>-0.6981246572313926</v>
+        <v>-0.5780397596786215</v>
       </c>
       <c r="I100" s="20" t="n">
         <v>-2.188078541547799</v>
@@ -17946,19 +17946,19 @@
         <v>-4.029724862175027</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>-5.823757999738711</v>
+        <v>-5.823757999738709</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>-7.61767824082834</v>
+        <v>-7.617678240828338</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>-9.411706258759011</v>
+        <v>-9.411706258759009</v>
       </c>
       <c r="N100" s="20" t="n">
         <v>-11.20591395499266</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>-12.98991504465789</v>
+        <v>-12.98991504465788</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -20620,13 +20620,13 @@
         <v>-102.9455882482798</v>
       </c>
       <c r="M37" s="19" t="n">
-        <v>-211.2762969230018</v>
+        <v>-211.2762969230016</v>
       </c>
       <c r="N37" s="19" t="n">
-        <v>-357.5237612260821</v>
+        <v>-357.5237612260819</v>
       </c>
       <c r="O37" s="19" t="n">
-        <v>-541.6960463870478</v>
+        <v>-541.696046387048</v>
       </c>
     </row>
     <row r="38" ht="15.5" customHeight="1">
@@ -20835,7 +20835,7 @@
         <v>4397.880947567281</v>
       </c>
       <c r="N41" s="18" t="n">
-        <v>4627.282008722716</v>
+        <v>4627.282008722714</v>
       </c>
       <c r="O41" s="18" t="n">
         <v>4818.436049145903</v>
@@ -20888,7 +20888,7 @@
         <v>4397.880947567281</v>
       </c>
       <c r="N42" s="18" t="n">
-        <v>4627.282008722716</v>
+        <v>4627.282008722714</v>
       </c>
       <c r="O42" s="18" t="n">
         <v>4818.436049145903</v>
@@ -20917,34 +20917,34 @@
         <v>1003.391117474072</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>1279.171703532507</v>
+        <v>1278.600030009678</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>1554.947988556262</v>
+        <v>1554.376315033434</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>1830.720037317144</v>
+        <v>1830.148363794316</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>2106.48791372163</v>
+        <v>2105.916240198801</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>2382.251680821688</v>
+        <v>2381.68000729886</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>2657.881540477052</v>
+        <v>2657.309866954223</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>2933.477721258876</v>
+        <v>2932.906047736049</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>3209.073180927569</v>
+        <v>3208.501507404741</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>3484.667931097034</v>
+        <v>3484.096257574205</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>3760.261983221006</v>
+        <v>3759.690309698178</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -20970,34 +20970,34 @@
         <v>973.0429276858573</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>1248.611024877091</v>
+        <v>1248.039351354262</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>1524.179122068324</v>
+        <v>1523.607448545496</v>
       </c>
       <c r="H44" s="18" t="n">
-        <v>1799.747219259557</v>
+        <v>1799.175545736729</v>
       </c>
       <c r="I44" s="18" t="n">
-        <v>2075.315316450791</v>
+        <v>2074.743642927962</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>2350.883413642024</v>
+        <v>2350.311740119196</v>
       </c>
       <c r="K44" s="18" t="n">
-        <v>2626.451510833258</v>
+        <v>2625.879837310429</v>
       </c>
       <c r="L44" s="18" t="n">
-        <v>2902.019608024491</v>
+        <v>2901.447934501663</v>
       </c>
       <c r="M44" s="18" t="n">
-        <v>3177.587705215724</v>
+        <v>3177.016031692896</v>
       </c>
       <c r="N44" s="18" t="n">
-        <v>3453.155802406958</v>
+        <v>3452.584128884129</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>3728.723899598191</v>
+        <v>3728.152226075363</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -21129,34 +21129,34 @@
         <v>2188.934227409571</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>3000.156193255411</v>
+        <v>2999.584519732583</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>3773.12508777403</v>
+        <v>3772.553414251202</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>4507.841110498985</v>
+        <v>4507.269436976157</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>5204.304458750879</v>
+        <v>5203.73278522805</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>5862.477758388485</v>
+        <v>5861.906084865657</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>6482.234589561317</v>
+        <v>6481.662916038488</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>7063.715704532602</v>
+        <v>7063.144031009773</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>7606.95412849485</v>
+        <v>7606.382454972021</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>8111.949939819749</v>
+        <v>8111.378266296919</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>8578.698032366909</v>
+        <v>8578.126358844082</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -21185,31 +21185,31 @@
         <v>1199.810297296057</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>1581.382089146499</v>
+        <v>1581.622781487826</v>
       </c>
       <c r="H48" s="18" t="n">
-        <v>1924.697054228054</v>
+        <v>1924.937777927854</v>
       </c>
       <c r="I48" s="18" t="n">
-        <v>2229.755482662951</v>
+        <v>2229.996205699612</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>2496.527229297121</v>
+        <v>2496.767951677277</v>
       </c>
       <c r="K48" s="18" t="n">
-        <v>2724.755965443383</v>
+        <v>2724.996687173596</v>
       </c>
       <c r="L48" s="18" t="n">
-        <v>2914.675465180135</v>
+        <v>2914.916186266907</v>
       </c>
       <c r="M48" s="18" t="n">
-        <v>3066.351724776917</v>
+        <v>3066.592430323402</v>
       </c>
       <c r="N48" s="18" t="n">
-        <v>3179.784832424792</v>
+        <v>3180.025522661097</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>3254.970666066729</v>
+        <v>3255.211355974531</v>
       </c>
     </row>
     <row r="49" ht="15.5" customHeight="1">
@@ -21344,31 +21344,31 @@
         <v>620.532300738528</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>1040.361149146706</v>
+        <v>1040.601841488033</v>
       </c>
       <c r="H51" s="18" t="n">
-        <v>1421.932909638675</v>
+        <v>1422.173633338475</v>
       </c>
       <c r="I51" s="18" t="n">
-        <v>1765.247875383368</v>
+        <v>1765.488598420029</v>
       </c>
       <c r="J51" s="18" t="n">
-        <v>2070.306304474771</v>
+        <v>2070.547026854927</v>
       </c>
       <c r="K51" s="18" t="n">
-        <v>2337.078051758884</v>
+        <v>2337.318773489097</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>2565.306788548587</v>
+        <v>2565.547509635359</v>
       </c>
       <c r="M51" s="18" t="n">
-        <v>2755.226303825626</v>
+        <v>2755.467009372111</v>
       </c>
       <c r="N51" s="18" t="n">
-        <v>2906.902578732588</v>
+        <v>2907.143268968893</v>
       </c>
       <c r="O51" s="18" t="n">
-        <v>3020.335686708966</v>
+        <v>3020.576376616769</v>
       </c>
     </row>
     <row r="52" ht="15.5" customHeight="1">
@@ -21715,31 +21715,31 @@
         <v>1956.838659736531</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>2338.202263754451</v>
+        <v>2338.442956095779</v>
       </c>
       <c r="H58" s="18" t="n">
-        <v>2681.313277266356</v>
+        <v>2681.554000966157</v>
       </c>
       <c r="I58" s="18" t="n">
-        <v>2986.171926488003</v>
+        <v>2986.412649524663</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>3252.748003213348</v>
+        <v>3252.988725593504</v>
       </c>
       <c r="K58" s="18" t="n">
-        <v>3480.914976895479</v>
+        <v>3481.155698625693</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>3670.80639304164</v>
+        <v>3671.047114128412</v>
       </c>
       <c r="M58" s="18" t="n">
-        <v>3822.455290160962</v>
+        <v>3822.695995707447</v>
       </c>
       <c r="N58" s="18" t="n">
-        <v>3935.861744830607</v>
+        <v>3936.102435066912</v>
       </c>
       <c r="O58" s="18" t="n">
-        <v>4011.021623539805</v>
+        <v>4011.262313447607</v>
       </c>
     </row>
     <row r="59" ht="15.5" customHeight="1">
@@ -21765,34 +21765,34 @@
         <v>651.952619555344</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>1043.31753351888</v>
+        <v>1042.745859996052</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>1434.922824019579</v>
+        <v>1434.110458155424</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>1826.527833232628</v>
+        <v>1825.71543601</v>
       </c>
       <c r="I59" s="18" t="n">
-        <v>2218.132532262877</v>
+        <v>2217.320135703387</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>2609.729755175137</v>
+        <v>2608.917359272154</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>3001.319612665838</v>
+        <v>3000.507217412795</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>3392.909311490962</v>
+        <v>3392.096916881361</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>3784.498838333888</v>
+        <v>3783.686459264574</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>4176.088194989143</v>
+        <v>4175.275831230007</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>4567.676408827104</v>
+        <v>4566.864045396474</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -22669,31 +22669,31 @@
         <v>973.0429276858573</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>1248.611024877091</v>
+        <v>1248.039351354262</v>
       </c>
       <c r="H76" s="18" t="n">
-        <v>1524.179122068324</v>
+        <v>1523.607448545496</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>1799.747219259557</v>
+        <v>1799.175545736729</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>2075.315316450791</v>
+        <v>2074.743642927962</v>
       </c>
       <c r="K76" s="18" t="n">
-        <v>2350.883413642024</v>
+        <v>2350.311740119196</v>
       </c>
       <c r="L76" s="18" t="n">
-        <v>2626.451510833258</v>
+        <v>2625.879837310429</v>
       </c>
       <c r="M76" s="18" t="n">
-        <v>2902.019608024491</v>
+        <v>2901.447934501663</v>
       </c>
       <c r="N76" s="18" t="n">
-        <v>3177.587705215724</v>
+        <v>3177.016031692896</v>
       </c>
       <c r="O76" s="18" t="n">
-        <v>3453.155802406958</v>
+        <v>3452.584128884129</v>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
@@ -22772,34 +22772,34 @@
         <v>973.0429276858573</v>
       </c>
       <c r="F78" s="18" t="n">
-        <v>1248.611024877091</v>
+        <v>1248.039351354262</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>1524.179122068324</v>
+        <v>1523.607448545496</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>1799.747219259557</v>
+        <v>1799.175545736729</v>
       </c>
       <c r="I78" s="18" t="n">
-        <v>2075.315316450791</v>
+        <v>2074.743642927962</v>
       </c>
       <c r="J78" s="18" t="n">
-        <v>2350.883413642024</v>
+        <v>2350.311740119196</v>
       </c>
       <c r="K78" s="18" t="n">
-        <v>2626.451510833258</v>
+        <v>2625.879837310429</v>
       </c>
       <c r="L78" s="18" t="n">
-        <v>2902.019608024491</v>
+        <v>2901.447934501663</v>
       </c>
       <c r="M78" s="18" t="n">
-        <v>3177.587705215724</v>
+        <v>3177.016031692896</v>
       </c>
       <c r="N78" s="18" t="n">
-        <v>3453.155802406958</v>
+        <v>3452.584128884129</v>
       </c>
       <c r="O78" s="18" t="n">
-        <v>3728.723899598191</v>
+        <v>3728.152226075363</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -23011,7 +23011,7 @@
         <v>4397.880947567281</v>
       </c>
       <c r="O82" s="18" t="n">
-        <v>4627.282008722716</v>
+        <v>4627.282008722714</v>
       </c>
     </row>
     <row r="83" ht="15.5" customHeight="1">
@@ -23167,7 +23167,7 @@
         <v>4397.880947567281</v>
       </c>
       <c r="N85" s="18" t="n">
-        <v>4627.282008722716</v>
+        <v>4627.282008722714</v>
       </c>
       <c r="O85" s="18" t="n">
         <v>4818.436049145903</v>
@@ -23753,31 +23753,31 @@
         <v>1058.692630951551</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>2566.930973380454</v>
+        <v>2566.840696840144</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>4794.793458288945</v>
+        <v>4794.703213107107</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>7692.003502190904</v>
+        <v>7691.913256345927</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>10622.61455436393</v>
+        <v>10622.52430786245</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>13363.6658221277</v>
+        <v>13363.57557497628</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>15891.55040032479</v>
+        <v>15891.46015252993</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>18201.60854197374</v>
+        <v>18201.51827863857</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>20293.74789894738</v>
+        <v>20293.65762030205</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>22167.94247925205</v>
+        <v>22167.85220027822</v>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
@@ -23962,34 +23962,34 @@
         <v>1058.692630951551</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>2566.930973380454</v>
+        <v>2566.840696840144</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>4794.793458288945</v>
+        <v>4794.703213107107</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>7692.003502190904</v>
+        <v>7691.913256345927</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>10622.61455436393</v>
+        <v>10622.52430786245</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>13363.6658221277</v>
+        <v>13363.57557497628</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>15891.55040032479</v>
+        <v>15891.46015252993</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>18201.60854197374</v>
+        <v>18201.51827863857</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>20293.74789894738</v>
+        <v>20293.65762030205</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>22167.94247925205</v>
+        <v>22167.85220027822</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>23824.21537012213</v>
+        <v>23824.12509082308</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -26657,7 +26657,7 @@
         <v>-27.72</v>
       </c>
       <c r="O37" s="19" t="n">
-        <v>-29.79999999999999</v>
+        <v>-29.8</v>
       </c>
     </row>
     <row r="38" ht="15.5" customHeight="1">
@@ -26948,13 +26948,13 @@
         <v>5.260595287671237</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>6.463571506849319</v>
+        <v>8.538640000000004</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>7.92795550684932</v>
+        <v>9.886275506849319</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>11.443264</v>
+        <v>11.32819550684932</v>
       </c>
       <c r="I43" s="18" t="n">
         <v>14.82104</v>
@@ -27001,13 +27001,13 @@
         <v>5.20854049315069</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>6.463571506849319</v>
+        <v>8.538640000000004</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>7.92795550684932</v>
+        <v>9.886275506849319</v>
       </c>
       <c r="H44" s="18" t="n">
-        <v>11.443264</v>
+        <v>11.32819550684932</v>
       </c>
       <c r="I44" s="18" t="n">
         <v>14.82104</v>
@@ -27160,13 +27160,13 @@
         <v>15.01059528767124</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>14.71357150684932</v>
+        <v>16.78864</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>14.67795550684932</v>
+        <v>16.63627550684932</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>16.69326400000001</v>
+        <v>16.57819550684932</v>
       </c>
       <c r="I47" s="18" t="n">
         <v>18.57104</v>
@@ -27216,10 +27216,10 @@
         <v>-34.9111464</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>-38.8500584</v>
+        <v>-36.8900584</v>
       </c>
       <c r="H48" s="18" t="n">
-        <v>-42.8097544</v>
+        <v>-40.8514344</v>
       </c>
       <c r="I48" s="18" t="n">
         <v>-44.8335944</v>
@@ -27228,7 +27228,7 @@
         <v>-46.8798984</v>
       </c>
       <c r="K48" s="18" t="n">
-        <v>-48.94866640000001</v>
+        <v>-48.9486664</v>
       </c>
       <c r="L48" s="18" t="n">
         <v>-51.01871235200001</v>
@@ -27375,10 +27375,10 @@
         <v>-34.7104256</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>-38.6268736</v>
+        <v>-36.6668736</v>
       </c>
       <c r="H51" s="18" t="n">
-        <v>-42.5641056</v>
+        <v>-40.6057856</v>
       </c>
       <c r="I51" s="18" t="n">
         <v>-44.5654816</v>
@@ -27387,13 +27387,13 @@
         <v>-46.5893216</v>
       </c>
       <c r="K51" s="18" t="n">
-        <v>-48.63562560000001</v>
+        <v>-48.6356256</v>
       </c>
       <c r="L51" s="18" t="n">
         <v>-50.70439360000001</v>
       </c>
       <c r="M51" s="18" t="n">
-        <v>-52.774439552</v>
+        <v>-52.77443955200001</v>
       </c>
       <c r="N51" s="18" t="n">
         <v>-54.845853312</v>
@@ -27746,10 +27746,10 @@
         <v>-18.9111464</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>-22.8500584</v>
+        <v>-20.8900584</v>
       </c>
       <c r="H58" s="18" t="n">
-        <v>-26.8097544</v>
+        <v>-24.8514344</v>
       </c>
       <c r="I58" s="18" t="n">
         <v>-28.8335944</v>
@@ -27758,7 +27758,7 @@
         <v>-30.8798984</v>
       </c>
       <c r="K58" s="18" t="n">
-        <v>-32.94866640000001</v>
+        <v>-32.9486664</v>
       </c>
       <c r="L58" s="18" t="n">
         <v>-35.01871235200001</v>
@@ -27796,13 +27796,13 @@
         <v>31.9077594410959</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>33.62471790684932</v>
+        <v>35.69978640000001</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>37.52801390684932</v>
+        <v>37.52633390684932</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>43.5030184</v>
+        <v>41.42962990684932</v>
       </c>
       <c r="I59" s="18" t="n">
         <v>47.40463439999999</v>
@@ -27811,7 +27811,7 @@
         <v>51.3062504</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>55.20786640000001</v>
+        <v>55.2078664</v>
       </c>
       <c r="L59" s="18" t="n">
         <v>59.1094824</v>
@@ -28700,13 +28700,13 @@
         <v>5.20854049315069</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>6.463571506849319</v>
+        <v>8.538640000000004</v>
       </c>
       <c r="H76" s="18" t="n">
-        <v>7.92795550684932</v>
+        <v>9.886275506849319</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>11.443264</v>
+        <v>11.32819550684932</v>
       </c>
       <c r="J76" s="18" t="n">
         <v>14.82104</v>
@@ -28803,13 +28803,13 @@
         <v>5.20854049315069</v>
       </c>
       <c r="F78" s="18" t="n">
-        <v>6.463571506849319</v>
+        <v>8.538640000000004</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>7.92795550684932</v>
+        <v>9.886275506849319</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>11.443264</v>
+        <v>11.32819550684932</v>
       </c>
       <c r="I78" s="18" t="n">
         <v>14.82104</v>
@@ -29784,10 +29784,10 @@
         <v>-31.1989712</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>-33.359692</v>
+        <v>-31.399692</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>-35.5411968</v>
+        <v>-33.5828768</v>
       </c>
       <c r="I96" s="20" t="n">
         <v>-35.7868456</v>
@@ -29993,10 +29993,10 @@
         <v>-31.1989712</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>-33.359692</v>
+        <v>-31.399692</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>-35.5411968</v>
+        <v>-33.5828768</v>
       </c>
       <c r="H100" s="20" t="n">
         <v>-35.7868456</v>

</xml_diff>

<commit_message>
Minor adjustment of file uploader style, tariff and upstream tables
</commit_message>
<xml_diff>
--- a/backend/Rwanda/financial-statements-CleanStep.xlsx
+++ b/backend/Rwanda/financial-statements-CleanStep.xlsx
@@ -962,40 +962,40 @@
         </is>
       </c>
       <c r="D8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O8" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="15.5" customHeight="1">
@@ -1598,40 +1598,40 @@
         </is>
       </c>
       <c r="D20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O20" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="15.5" customHeight="1">
@@ -2075,40 +2075,40 @@
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O29" s="19" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="15.5" customHeight="1">
@@ -2729,22 +2729,22 @@
         <v>377.9752415799667</v>
       </c>
       <c r="J41" s="18" t="n">
-        <v>427.6745349631409</v>
+        <v>468.8902736200481</v>
       </c>
       <c r="K41" s="18" t="n">
-        <v>786.7461088895443</v>
+        <v>546.4993238167979</v>
       </c>
       <c r="L41" s="18" t="n">
-        <v>820.8560689793743</v>
+        <v>900.2983204991639</v>
       </c>
       <c r="M41" s="18" t="n">
-        <v>852.6478332128239</v>
+        <v>929.1884291173966</v>
       </c>
       <c r="N41" s="18" t="n">
-        <v>882.1446792975107</v>
+        <v>955.8125403939653</v>
       </c>
       <c r="O41" s="18" t="n">
-        <v>860.7048705459894</v>
+        <v>931.5288876506644</v>
       </c>
     </row>
     <row r="42" ht="15.5" customHeight="1">
@@ -2782,22 +2782,22 @@
         <v>377.9752415799667</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>427.6745349631409</v>
+        <v>468.8902736200481</v>
       </c>
       <c r="K42" s="18" t="n">
-        <v>786.7461088895443</v>
+        <v>546.4993238167979</v>
       </c>
       <c r="L42" s="18" t="n">
-        <v>820.8560689793743</v>
+        <v>900.2983204991639</v>
       </c>
       <c r="M42" s="18" t="n">
-        <v>852.6478332128239</v>
+        <v>929.1884291173966</v>
       </c>
       <c r="N42" s="18" t="n">
-        <v>882.1446792975107</v>
+        <v>955.8125403939653</v>
       </c>
       <c r="O42" s="18" t="n">
-        <v>860.7048705459894</v>
+        <v>931.5288876506644</v>
       </c>
     </row>
     <row r="43" ht="15.5" customHeight="1">
@@ -2820,37 +2820,37 @@
         <v>30.71713469777927</v>
       </c>
       <c r="E43" s="18" t="n">
-        <v>2300.119789112662</v>
+        <v>2.13224831266213</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>4819.967587891309</v>
+        <v>2521.980047091309</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>6899.293831268377</v>
+        <v>4601.306290468377</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>9185.34504808879</v>
+        <v>6887.357507288791</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>11484.98741025383</v>
+        <v>9186.999869453832</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>13767.25131730229</v>
+        <v>11471.77062581735</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>14940.13680426029</v>
+        <v>13743.32513047112</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>16458.03297266198</v>
+        <v>14936.61499750294</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>17940.88581045407</v>
+        <v>16460.00031826405</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>19459.06239975362</v>
+        <v>17942.8050141539</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>21056.76178785249</v>
+        <v>19461.63722772111</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -2873,37 +2873,37 @@
         <v>0</v>
       </c>
       <c r="E44" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="18" t="n">
         <v>2297.9875408</v>
       </c>
-      <c r="F44" s="18" t="n">
+      <c r="G44" s="18" t="n">
         <v>4595.9750816</v>
       </c>
-      <c r="G44" s="18" t="n">
-        <v>6893.962622399999</v>
-      </c>
       <c r="H44" s="18" t="n">
+        <v>6880.365105369025</v>
+      </c>
+      <c r="I44" s="18" t="n">
         <v>9178.352646169024</v>
       </c>
-      <c r="I44" s="18" t="n">
-        <v>11476.34018696902</v>
-      </c>
       <c r="J44" s="18" t="n">
-        <v>13756.96522451539</v>
+        <v>11461.48453303045</v>
       </c>
       <c r="K44" s="18" t="n">
-        <v>14927.48028473426</v>
+        <v>13730.66861094509</v>
       </c>
       <c r="L44" s="18" t="n">
+        <v>14921.95254081148</v>
+      </c>
+      <c r="M44" s="18" t="n">
         <v>16443.37051597052</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>17924.25600816054</v>
       </c>
-      <c r="N44" s="18" t="n">
+      <c r="O44" s="18" t="n">
         <v>19440.51339376026</v>
-      </c>
-      <c r="O44" s="18" t="n">
-        <v>21035.63795389164</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -3032,37 +3032,37 @@
         <v>71.93287335468639</v>
       </c>
       <c r="E47" s="18" t="n">
-        <v>2414.491028411108</v>
+        <v>116.5034876111085</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>5004.56336442383</v>
+        <v>2706.575823623831</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>7151.212491261584</v>
+        <v>4853.224950461584</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>9501.713954307026</v>
+        <v>7203.726413507027</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>11862.9626518338</v>
+        <v>9564.975111033798</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>14194.92585226543</v>
+        <v>11940.66089943739</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>15726.88291314983</v>
+        <v>14289.82445428791</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>17278.88904164136</v>
+        <v>15836.9133180021</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>18793.53364366689</v>
+        <v>17389.18874738145</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>20341.20707905113</v>
+        <v>18898.61755454787</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>21917.46665839848</v>
+        <v>20393.16611537178</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -3088,34 +3088,34 @@
         <v>118.6357359237707</v>
       </c>
       <c r="F48" s="18" t="n">
-        <v>1360.326272383511</v>
+        <v>632.5807891151399</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>2303.43606959473</v>
+        <v>990.3265609983337</v>
       </c>
       <c r="H48" s="18" t="n">
-        <v>3657.589598401996</v>
+        <v>2357.611184891562</v>
       </c>
       <c r="I48" s="18" t="n">
-        <v>5009.484205869137</v>
+        <v>3722.50557649381</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>6362.930166056397</v>
+        <v>5088.821322974819</v>
       </c>
       <c r="K48" s="18" t="n">
-        <v>6888.171458147949</v>
+        <v>6460.199194818024</v>
       </c>
       <c r="L48" s="18" t="n">
-        <v>27173.90079794113</v>
+        <v>7000.207800165653</v>
       </c>
       <c r="M48" s="18" t="n">
-        <v>21442.30310109409</v>
+        <v>27286.1678492833</v>
       </c>
       <c r="N48" s="18" t="n">
-        <v>22921.13806258924</v>
+        <v>21549.3062156749</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>23934.75198131315</v>
+        <v>22975.67192687738</v>
       </c>
     </row>
     <row r="49" ht="15.5" customHeight="1">
@@ -3247,34 +3247,34 @@
         <v>102.6500080524657</v>
       </c>
       <c r="F51" s="18" t="n">
-        <v>846.3812191921418</v>
+        <v>118.6357359237707</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>2673.435780979908</v>
+        <v>1360.326272383511</v>
       </c>
       <c r="H51" s="18" t="n">
-        <v>3603.414483105165</v>
+        <v>2303.436069594731</v>
       </c>
       <c r="I51" s="18" t="n">
-        <v>4944.568227777324</v>
+        <v>3657.589598401996</v>
       </c>
       <c r="J51" s="18" t="n">
-        <v>6283.593048950715</v>
+        <v>5009.484205869137</v>
       </c>
       <c r="K51" s="18" t="n">
-        <v>6790.902429386321</v>
+        <v>6362.930166056396</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>27061.86445592343</v>
+        <v>6888.171458147949</v>
       </c>
       <c r="M51" s="18" t="n">
-        <v>21330.03604975193</v>
+        <v>27173.90079794114</v>
       </c>
       <c r="N51" s="18" t="n">
-        <v>22814.13494800844</v>
+        <v>21442.30310109409</v>
       </c>
       <c r="O51" s="18" t="n">
-        <v>23880.21811702501</v>
+        <v>22921.13806258924</v>
       </c>
     </row>
     <row r="52" ht="15.5" customHeight="1">
@@ -3294,40 +3294,40 @@
         </is>
       </c>
       <c r="D52" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="18" t="n">
         <v>-727.7454832683711</v>
       </c>
-      <c r="E52" s="18" t="n">
+      <c r="F52" s="18" t="n">
         <v>-399.4353198647671</v>
       </c>
-      <c r="F52" s="18" t="n">
+      <c r="G52" s="18" t="n">
         <v>-57.99406137520214</v>
       </c>
-      <c r="G52" s="18" t="n">
+      <c r="H52" s="18" t="n">
         <v>296.4469812494701</v>
       </c>
-      <c r="H52" s="18" t="n">
+      <c r="I52" s="18" t="n">
         <v>663.7578101678919</v>
       </c>
-      <c r="I52" s="18" t="n">
+      <c r="J52" s="18" t="n">
         <v>1771.555210785502</v>
       </c>
-      <c r="J52" s="18" t="n">
+      <c r="K52" s="18" t="n">
         <v>-16786.921557147</v>
       </c>
-      <c r="K52" s="18" t="n">
+      <c r="L52" s="18" t="n">
         <v>-10356.70876738495</v>
       </c>
-      <c r="L52" s="18" t="n">
+      <c r="M52" s="18" t="n">
         <v>-10298.78028927715</v>
       </c>
-      <c r="M52" s="18" t="n">
+      <c r="N52" s="18" t="n">
         <v>-10230.33598785992</v>
       </c>
-      <c r="N52" s="18" t="n">
+      <c r="O52" s="18" t="n">
         <v>-10151.48102136637</v>
-      </c>
-      <c r="O52" s="18" t="n">
-        <v>-8635.835178337573</v>
       </c>
     </row>
     <row r="53" ht="15.5" customHeight="1">
@@ -3347,40 +3347,40 @@
         </is>
       </c>
       <c r="D53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="18" t="n">
         <v>-727.7454832683711</v>
       </c>
-      <c r="E53" s="18" t="n">
+      <c r="F53" s="18" t="n">
         <v>-399.4353198647671</v>
       </c>
-      <c r="F53" s="18" t="n">
+      <c r="G53" s="18" t="n">
         <v>-57.99406137520214</v>
       </c>
-      <c r="G53" s="18" t="n">
+      <c r="H53" s="18" t="n">
         <v>296.4469812494701</v>
       </c>
-      <c r="H53" s="18" t="n">
+      <c r="I53" s="18" t="n">
         <v>663.7578101678919</v>
       </c>
-      <c r="I53" s="18" t="n">
+      <c r="J53" s="18" t="n">
         <v>1771.555210785502</v>
       </c>
-      <c r="J53" s="18" t="n">
+      <c r="K53" s="18" t="n">
         <v>-16786.921557147</v>
       </c>
-      <c r="K53" s="18" t="n">
+      <c r="L53" s="18" t="n">
         <v>-10356.70876738495</v>
       </c>
-      <c r="L53" s="18" t="n">
+      <c r="M53" s="18" t="n">
         <v>-10298.78028927715</v>
       </c>
-      <c r="M53" s="18" t="n">
+      <c r="N53" s="18" t="n">
         <v>-10230.33598785992</v>
       </c>
-      <c r="N53" s="18" t="n">
+      <c r="O53" s="18" t="n">
         <v>-10151.48102136637</v>
-      </c>
-      <c r="O53" s="18" t="n">
-        <v>-8635.835178337573</v>
       </c>
     </row>
     <row r="54" ht="15.5" customHeight="1">
@@ -3612,40 +3612,40 @@
         </is>
       </c>
       <c r="D58" s="18" t="n">
-        <v>-655.8126099136847</v>
+        <v>71.93287335468639</v>
       </c>
       <c r="E58" s="18" t="n">
-        <v>-282.9318322536585</v>
+        <v>-611.2419956572626</v>
       </c>
       <c r="F58" s="18" t="n">
-        <v>1078.339704716999</v>
+        <v>9.152962959063387</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>2594.551841975823</v>
+        <v>927.0012907547534</v>
       </c>
       <c r="H58" s="18" t="n">
-        <v>4314.355006650122</v>
+        <v>2647.065764221266</v>
       </c>
       <c r="I58" s="18" t="n">
-        <v>6772.392193369831</v>
+        <v>4377.616163376893</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>-10434.27748387749</v>
+        <v>6850.090440973429</v>
       </c>
       <c r="K58" s="18" t="n">
-        <v>-3481.193828763027</v>
+        <v>-10339.378881855</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>16860.45805197252</v>
+        <v>-3371.163423910754</v>
       </c>
       <c r="M58" s="18" t="n">
-        <v>11195.33731094064</v>
+        <v>16970.75775771262</v>
       </c>
       <c r="N58" s="18" t="n">
-        <v>12751.10803522951</v>
+        <v>11300.42122182162</v>
       </c>
       <c r="O58" s="18" t="n">
-        <v>15277.79296901473</v>
+        <v>12803.06707155016</v>
       </c>
     </row>
     <row r="59" ht="15.5" customHeight="1">
@@ -3665,40 +3665,40 @@
         </is>
       </c>
       <c r="D59" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="18" t="n">
         <v>727.7454832683711</v>
       </c>
-      <c r="E59" s="18" t="n">
-        <v>2697.422860664767</v>
-      </c>
       <c r="F59" s="18" t="n">
+        <v>2697.422860664768</v>
+      </c>
+      <c r="G59" s="18" t="n">
         <v>3926.22365970683</v>
       </c>
-      <c r="G59" s="18" t="n">
+      <c r="H59" s="18" t="n">
         <v>4556.660649285761</v>
       </c>
-      <c r="H59" s="18" t="n">
-        <v>5187.358947656904</v>
-      </c>
       <c r="I59" s="18" t="n">
-        <v>5090.570458463964</v>
+        <v>5187.358947656905</v>
       </c>
       <c r="J59" s="18" t="n">
+        <v>5090.570458463965</v>
+      </c>
+      <c r="K59" s="18" t="n">
         <v>24629.20333614292</v>
       </c>
-      <c r="K59" s="18" t="n">
+      <c r="L59" s="18" t="n">
         <v>19208.07674191286</v>
       </c>
-      <c r="L59" s="18" t="n">
-        <v>418.4309896688319</v>
-      </c>
       <c r="M59" s="18" t="n">
-        <v>7598.196332726257</v>
+        <v>418.4309896688246</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>7590.099043821618</v>
+        <v>7598.196332726249</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>6639.673689383757</v>
+        <v>7590.099043821616</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -4572,34 +4572,34 @@
         <v>0</v>
       </c>
       <c r="F76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="18" t="n">
         <v>2297.9875408</v>
       </c>
-      <c r="G76" s="18" t="n">
+      <c r="H76" s="18" t="n">
         <v>4595.9750816</v>
       </c>
-      <c r="H76" s="18" t="n">
-        <v>6893.962622399999</v>
-      </c>
       <c r="I76" s="18" t="n">
+        <v>6880.365105369025</v>
+      </c>
+      <c r="J76" s="18" t="n">
         <v>9178.352646169024</v>
       </c>
-      <c r="J76" s="18" t="n">
-        <v>11476.34018696902</v>
-      </c>
       <c r="K76" s="18" t="n">
-        <v>13756.96522451539</v>
+        <v>11461.48453303045</v>
       </c>
       <c r="L76" s="18" t="n">
-        <v>14927.48028473426</v>
+        <v>13730.66861094509</v>
       </c>
       <c r="M76" s="18" t="n">
+        <v>14921.95254081148</v>
+      </c>
+      <c r="N76" s="18" t="n">
         <v>16443.37051597052</v>
       </c>
-      <c r="N76" s="18" t="n">
+      <c r="O76" s="18" t="n">
         <v>17924.25600816054</v>
-      </c>
-      <c r="O76" s="18" t="n">
-        <v>19440.51339376026</v>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
@@ -4675,37 +4675,37 @@
         <v>0</v>
       </c>
       <c r="E78" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="18" t="n">
         <v>2297.9875408</v>
       </c>
-      <c r="F78" s="18" t="n">
+      <c r="G78" s="18" t="n">
         <v>4595.9750816</v>
       </c>
-      <c r="G78" s="18" t="n">
-        <v>6893.962622399999</v>
-      </c>
       <c r="H78" s="18" t="n">
+        <v>6880.365105369025</v>
+      </c>
+      <c r="I78" s="18" t="n">
         <v>9178.352646169024</v>
       </c>
-      <c r="I78" s="18" t="n">
-        <v>11476.34018696902</v>
-      </c>
       <c r="J78" s="18" t="n">
-        <v>13756.96522451539</v>
+        <v>11461.48453303045</v>
       </c>
       <c r="K78" s="18" t="n">
-        <v>14927.48028473426</v>
+        <v>13730.66861094509</v>
       </c>
       <c r="L78" s="18" t="n">
+        <v>14921.95254081148</v>
+      </c>
+      <c r="M78" s="18" t="n">
         <v>16443.37051597052</v>
       </c>
-      <c r="M78" s="18" t="n">
+      <c r="N78" s="18" t="n">
         <v>17924.25600816054</v>
       </c>
-      <c r="N78" s="18" t="n">
+      <c r="O78" s="18" t="n">
         <v>19440.51339376026</v>
-      </c>
-      <c r="O78" s="18" t="n">
-        <v>21035.63795389164</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -4905,19 +4905,19 @@
         <v>377.9752415799667</v>
       </c>
       <c r="K82" s="18" t="n">
-        <v>427.6745349631409</v>
+        <v>468.8902736200481</v>
       </c>
       <c r="L82" s="18" t="n">
-        <v>786.7461088895443</v>
+        <v>546.4993238167979</v>
       </c>
       <c r="M82" s="18" t="n">
-        <v>820.8560689793743</v>
+        <v>900.2983204991639</v>
       </c>
       <c r="N82" s="18" t="n">
-        <v>852.6478332128239</v>
+        <v>929.1884291173966</v>
       </c>
       <c r="O82" s="18" t="n">
-        <v>882.1446792975107</v>
+        <v>955.8125403939653</v>
       </c>
     </row>
     <row r="83" ht="15.5" customHeight="1">
@@ -5061,22 +5061,22 @@
         <v>377.9752415799667</v>
       </c>
       <c r="J85" s="18" t="n">
-        <v>427.6745349631409</v>
+        <v>468.8902736200481</v>
       </c>
       <c r="K85" s="18" t="n">
-        <v>786.7461088895443</v>
+        <v>546.4993238167979</v>
       </c>
       <c r="L85" s="18" t="n">
-        <v>820.8560689793743</v>
+        <v>900.2983204991639</v>
       </c>
       <c r="M85" s="18" t="n">
-        <v>852.6478332128239</v>
+        <v>929.1884291173966</v>
       </c>
       <c r="N85" s="18" t="n">
-        <v>882.1446792975107</v>
+        <v>955.8125403939653</v>
       </c>
       <c r="O85" s="18" t="n">
-        <v>860.7048705459894</v>
+        <v>931.5288876506644</v>
       </c>
     </row>
     <row r="86" ht="15.5" customHeight="1">
@@ -5656,34 +5656,34 @@
         <v>433.7685840977465</v>
       </c>
       <c r="F96" s="20" t="n">
-        <v>1834.55789895781</v>
+        <v>450.2445468894396</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>7206.625438511972</v>
+        <v>5236.948061115576</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>9615.473703558198</v>
+        <v>7658.927421247764</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>11613.19531703036</v>
+        <v>9669.64881885503</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>13613.27317014221</v>
+        <v>11682.59645826064</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>14447.71184333254</v>
+        <v>13692.61028724789</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>35135.64833749675</v>
+        <v>14544.98087209417</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>26932.27952490632</v>
+        <v>35247.68467951445</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>28042.55237409545</v>
+        <v>27072.99975384793</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>29618.87697027507</v>
+        <v>28216.66322290651</v>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
@@ -5865,37 +5865,37 @@
         <v>433.7685840977465</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>1834.55789895781</v>
+        <v>450.2445468894396</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>7206.625438511972</v>
+        <v>5236.948061115576</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>9615.473703558198</v>
+        <v>7658.927421247764</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>11613.19531703036</v>
+        <v>9669.64881885503</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>13613.27317014221</v>
+        <v>11682.59645826064</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>14447.71184333254</v>
+        <v>13692.61028724789</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>35135.64833749675</v>
+        <v>14544.98087209417</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>26932.27952490632</v>
+        <v>35247.68467951445</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>28042.55237409545</v>
+        <v>27072.99975384793</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>29618.87697027507</v>
+        <v>28216.66322290651</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>31272.60268834075</v>
+        <v>29887.18635296807</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -5968,40 +5968,40 @@
         </is>
       </c>
       <c r="D102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O102" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" ht="15.5" customHeight="1">
@@ -6024,37 +6024,37 @@
         <v>0</v>
       </c>
       <c r="E103" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" s="18" t="n">
         <v>-727.7454832683711</v>
       </c>
-      <c r="F103" s="18" t="n">
+      <c r="G103" s="18" t="n">
         <v>-399.4353198647671</v>
       </c>
-      <c r="G103" s="18" t="n">
+      <c r="H103" s="18" t="n">
         <v>-57.99406137520214</v>
       </c>
-      <c r="H103" s="18" t="n">
+      <c r="I103" s="18" t="n">
         <v>296.4469812494701</v>
       </c>
-      <c r="I103" s="18" t="n">
+      <c r="J103" s="18" t="n">
         <v>663.7578101678919</v>
       </c>
-      <c r="J103" s="18" t="n">
+      <c r="K103" s="18" t="n">
         <v>1771.555210785502</v>
       </c>
-      <c r="K103" s="18" t="n">
+      <c r="L103" s="18" t="n">
         <v>-16786.921557147</v>
       </c>
-      <c r="L103" s="18" t="n">
+      <c r="M103" s="18" t="n">
         <v>-10356.70876738495</v>
       </c>
-      <c r="M103" s="18" t="n">
+      <c r="N103" s="18" t="n">
         <v>-10298.78028927715</v>
       </c>
-      <c r="N103" s="18" t="n">
+      <c r="O103" s="18" t="n">
         <v>-10230.33598785992</v>
-      </c>
-      <c r="O103" s="18" t="n">
-        <v>-10151.48102136637</v>
       </c>
     </row>
     <row r="104" ht="15.5" customHeight="1">
@@ -6127,40 +6127,40 @@
         </is>
       </c>
       <c r="D105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O105" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" ht="15.5" customHeight="1">
@@ -6233,40 +6233,40 @@
         </is>
       </c>
       <c r="D107" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="18" t="n">
         <v>-727.7454832683711</v>
       </c>
-      <c r="E107" s="18" t="n">
+      <c r="F107" s="18" t="n">
         <v>-399.4353198647671</v>
       </c>
-      <c r="F107" s="18" t="n">
+      <c r="G107" s="18" t="n">
         <v>-57.99406137520214</v>
       </c>
-      <c r="G107" s="18" t="n">
+      <c r="H107" s="18" t="n">
         <v>296.4469812494701</v>
       </c>
-      <c r="H107" s="18" t="n">
+      <c r="I107" s="18" t="n">
         <v>663.7578101678919</v>
       </c>
-      <c r="I107" s="18" t="n">
+      <c r="J107" s="18" t="n">
         <v>1771.555210785502</v>
       </c>
-      <c r="J107" s="18" t="n">
+      <c r="K107" s="18" t="n">
         <v>-16786.921557147</v>
       </c>
-      <c r="K107" s="18" t="n">
+      <c r="L107" s="18" t="n">
         <v>-10356.70876738495</v>
       </c>
-      <c r="L107" s="18" t="n">
+      <c r="M107" s="18" t="n">
         <v>-10298.78028927715</v>
       </c>
-      <c r="M107" s="18" t="n">
+      <c r="N107" s="18" t="n">
         <v>-10230.33598785992</v>
       </c>
-      <c r="N107" s="18" t="n">
+      <c r="O107" s="18" t="n">
         <v>-10151.48102136637</v>
-      </c>
-      <c r="O107" s="18" t="n">
-        <v>-8635.835178337573</v>
       </c>
     </row>
     <row r="108" ht="15.5" customHeight="1">
@@ -8763,19 +8763,19 @@
         <v>2235.34280800426</v>
       </c>
       <c r="K41" s="18" t="n">
-        <v>2333.418320356867</v>
+        <v>2581.38007882974</v>
       </c>
       <c r="L41" s="18" t="n">
-        <v>2670.328871762653</v>
+        <v>2663.031069422604</v>
       </c>
       <c r="M41" s="18" t="n">
-        <v>2990.976933649055</v>
+        <v>2983.683012286244</v>
       </c>
       <c r="N41" s="18" t="n">
-        <v>3295.530488794742</v>
+        <v>3288.233015313682</v>
       </c>
       <c r="O41" s="18" t="n">
-        <v>3459.811679300637</v>
+        <v>3452.522549222511</v>
       </c>
     </row>
     <row r="42" ht="15.5" customHeight="1">
@@ -8816,19 +8816,19 @@
         <v>2235.34280800426</v>
       </c>
       <c r="K42" s="18" t="n">
-        <v>2333.418320356867</v>
+        <v>2581.38007882974</v>
       </c>
       <c r="L42" s="18" t="n">
-        <v>2670.328871762653</v>
+        <v>2663.031069422604</v>
       </c>
       <c r="M42" s="18" t="n">
-        <v>2990.976933649055</v>
+        <v>2983.683012286244</v>
       </c>
       <c r="N42" s="18" t="n">
-        <v>3295.530488794742</v>
+        <v>3288.233015313682</v>
       </c>
       <c r="O42" s="18" t="n">
-        <v>3459.811679300637</v>
+        <v>3452.522549222511</v>
       </c>
     </row>
     <row r="43" ht="15.5" customHeight="1">
@@ -8854,34 +8854,34 @@
         <v>42.6934018010603</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>4653.879272306851</v>
+        <v>2355.89173150685</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>4649.08648981918</v>
+        <v>2351.098949019179</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>6953.897131989042</v>
+        <v>4655.909591189042</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>9258.615949501373</v>
+        <v>6960.628408701372</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>11563.19737523288</v>
+        <v>9265.209834432881</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>13870.29089411507</v>
+        <v>11572.30335331507</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>16067.59496844874</v>
+        <v>13879.31632425206</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>18208.9151608098</v>
+        <v>16076.34252461312</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>20363.96004849405</v>
+        <v>18217.34889229737</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>22551.71082553193</v>
+        <v>20377.47462933524</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -8907,34 +8907,34 @@
         <v>0</v>
       </c>
       <c r="F44" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="18" t="n">
         <v>2297.987540800001</v>
       </c>
-      <c r="G44" s="18" t="n">
+      <c r="H44" s="18" t="n">
         <v>4595.975081600001</v>
       </c>
-      <c r="H44" s="18" t="n">
+      <c r="I44" s="18" t="n">
         <v>6893.962622400002</v>
       </c>
-      <c r="I44" s="18" t="n">
+      <c r="J44" s="18" t="n">
         <v>9191.950163200003</v>
       </c>
-      <c r="J44" s="18" t="n">
+      <c r="K44" s="18" t="n">
         <v>11489.937704</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>13787.9252448</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>15976.20388899668</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>18108.77652519336</v>
       </c>
-      <c r="N44" s="18" t="n">
+      <c r="O44" s="18" t="n">
         <v>20255.38768139004</v>
-      </c>
-      <c r="O44" s="18" t="n">
-        <v>22429.62387758672</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -9066,34 +9066,34 @@
         <v>685.2818150767414</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>5636.27176421972</v>
+        <v>3338.28422341972</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>5956.506022536704</v>
+        <v>3658.518481736704</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>8571.719306057012</v>
+        <v>6273.731765257012</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>11172.35777346012</v>
+        <v>8874.370232660121</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>13798.54018323714</v>
+        <v>11500.55264243714</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>16203.70921447194</v>
+        <v>14153.68343214481</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>18737.92384021139</v>
+        <v>16542.34739367466</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>21199.89209445885</v>
+        <v>19060.02553689936</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>23659.4905372888</v>
+        <v>21505.58190761106</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>26011.52250483256</v>
+        <v>23829.99717855775</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -9122,31 +9122,31 @@
         <v>5633.064820679988</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>2638.013385987701</v>
+        <v>1347.836420388751</v>
       </c>
       <c r="H48" s="18" t="n">
-        <v>4583.739215349417</v>
+        <v>2953.840224598421</v>
       </c>
       <c r="I48" s="18" t="n">
-        <v>6498.634351022921</v>
+        <v>4885.020004966224</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>8422.959484692539</v>
+        <v>6825.488672054733</v>
       </c>
       <c r="K48" s="18" t="n">
-        <v>10358.85044359882</v>
+        <v>8777.339993874184</v>
       </c>
       <c r="L48" s="18" t="n">
-        <v>7299.752196075559</v>
+        <v>10697.15163650017</v>
       </c>
       <c r="M48" s="18" t="n">
-        <v>12855.5735766737</v>
+        <v>7621.526769475863</v>
       </c>
       <c r="N48" s="18" t="n">
-        <v>10348.662435557</v>
+        <v>13160.94430487512</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>16928.25412600293</v>
+        <v>10518.85857273565</v>
       </c>
     </row>
     <row r="49" ht="15.5" customHeight="1">
@@ -9281,31 +9281,31 @@
         <v>675.4747894805378</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>6923.241786278937</v>
+        <v>5633.064820679988</v>
       </c>
       <c r="H51" s="18" t="n">
-        <v>4267.912376738697</v>
+        <v>2638.013385987701</v>
       </c>
       <c r="I51" s="18" t="n">
-        <v>6197.353561406114</v>
+        <v>4583.739215349417</v>
       </c>
       <c r="J51" s="18" t="n">
-        <v>8096.105163660727</v>
+        <v>6498.634351022921</v>
       </c>
       <c r="K51" s="18" t="n">
-        <v>10004.46993441717</v>
+        <v>8422.959484692539</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>6961.451003174207</v>
+        <v>10358.85044359881</v>
       </c>
       <c r="M51" s="18" t="n">
-        <v>12533.79900327339</v>
+        <v>7299.752196075559</v>
       </c>
       <c r="N51" s="18" t="n">
-        <v>10043.29170735558</v>
+        <v>12855.57357667369</v>
       </c>
       <c r="O51" s="18" t="n">
-        <v>16758.05798882428</v>
+        <v>10348.662435557</v>
       </c>
     </row>
     <row r="52" ht="15.5" customHeight="1">
@@ -9328,37 +9328,37 @@
         <v>0</v>
       </c>
       <c r="E52" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="18" t="n">
         <v>-1290.176965598953</v>
       </c>
-      <c r="F52" s="18" t="n">
+      <c r="G52" s="18" t="n">
         <v>-1278.65628434995</v>
       </c>
-      <c r="G52" s="18" t="n">
+      <c r="H52" s="18" t="n">
         <v>-1250.850958406641</v>
       </c>
-      <c r="H52" s="18" t="n">
+      <c r="I52" s="18" t="n">
         <v>-1206.902099044447</v>
       </c>
-      <c r="I52" s="18" t="n">
+      <c r="J52" s="18" t="n">
         <v>-1146.99287676908</v>
       </c>
-      <c r="J52" s="18" t="n">
+      <c r="K52" s="18" t="n">
         <v>27.56010391590189</v>
       </c>
-      <c r="K52" s="18" t="n">
+      <c r="L52" s="18" t="n">
         <v>-162.300607879974</v>
       </c>
-      <c r="L52" s="18" t="n">
+      <c r="M52" s="18" t="n">
         <v>-506.8604250494029</v>
       </c>
-      <c r="M52" s="18" t="n">
+      <c r="N52" s="18" t="n">
         <v>-831.0141990278089</v>
       </c>
-      <c r="N52" s="18" t="n">
+      <c r="O52" s="18" t="n">
         <v>-1134.919330769903</v>
-      </c>
-      <c r="O52" s="18" t="n">
-        <v>-1418.804158241069</v>
       </c>
     </row>
     <row r="53" ht="15.5" customHeight="1">
@@ -9381,37 +9381,37 @@
         <v>0</v>
       </c>
       <c r="E53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="18" t="n">
         <v>-1290.176965598953</v>
       </c>
-      <c r="F53" s="18" t="n">
+      <c r="G53" s="18" t="n">
         <v>-1278.65628434995</v>
       </c>
-      <c r="G53" s="18" t="n">
+      <c r="H53" s="18" t="n">
         <v>-1250.850958406641</v>
       </c>
-      <c r="H53" s="18" t="n">
+      <c r="I53" s="18" t="n">
         <v>-1206.902099044447</v>
       </c>
-      <c r="I53" s="18" t="n">
+      <c r="J53" s="18" t="n">
         <v>-1146.99287676908</v>
       </c>
-      <c r="J53" s="18" t="n">
+      <c r="K53" s="18" t="n">
         <v>27.56010391590189</v>
       </c>
-      <c r="K53" s="18" t="n">
+      <c r="L53" s="18" t="n">
         <v>-162.300607879974</v>
       </c>
-      <c r="L53" s="18" t="n">
+      <c r="M53" s="18" t="n">
         <v>-506.8604250494029</v>
       </c>
-      <c r="M53" s="18" t="n">
+      <c r="N53" s="18" t="n">
         <v>-831.0141990278089</v>
       </c>
-      <c r="N53" s="18" t="n">
+      <c r="O53" s="18" t="n">
         <v>-1134.919330769903</v>
-      </c>
-      <c r="O53" s="18" t="n">
-        <v>-1418.804158241069</v>
       </c>
     </row>
     <row r="54" ht="15.5" customHeight="1">
@@ -9646,37 +9646,37 @@
         <v>2096.015202249106</v>
       </c>
       <c r="E58" s="18" t="n">
-        <v>-631.1453642208451</v>
+        <v>659.031601378108</v>
       </c>
       <c r="F58" s="18" t="n">
-        <v>2029.072371946476</v>
+        <v>2017.551690697473</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>1366.953983745443</v>
+        <v>48.97169220318482</v>
       </c>
       <c r="H58" s="18" t="n">
-        <v>3353.916573839217</v>
+        <v>1680.068723726026</v>
       </c>
       <c r="I58" s="18" t="n">
-        <v>5326.040361925074</v>
+        <v>3652.51679359301</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>8422.291807786522</v>
+        <v>5650.268014463735</v>
       </c>
       <c r="K58" s="18" t="n">
-        <v>10164.15043571884</v>
+        <v>8772.500697790087</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>6756.148149108349</v>
+        <v>10498.10740670239</v>
       </c>
       <c r="M58" s="18" t="n">
-        <v>11983.60553928972</v>
+        <v>7073.712506070297</v>
       </c>
       <c r="N58" s="18" t="n">
-        <v>9168.731943162536</v>
+        <v>12284.91894422275</v>
       </c>
       <c r="O58" s="18" t="n">
-        <v>15457.83676776186</v>
+        <v>9332.326041965745</v>
       </c>
     </row>
     <row r="59" ht="15.5" customHeight="1">
@@ -9699,37 +9699,37 @@
         <v>22.70909589041412</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>1316.427179297586</v>
+        <v>26.25021369863339</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>3607.199392273244</v>
+        <v>1320.732532722247</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>4589.552038791261</v>
+        <v>3609.546789533519</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>5217.802732217795</v>
+        <v>4593.663041530986</v>
       </c>
       <c r="I59" s="18" t="n">
-        <v>5846.317411535048</v>
+        <v>5221.853439067111</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>5376.248375450617</v>
+        <v>5850.284627973407</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>6039.558778753093</v>
+        <v>5381.182734354721</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>11981.77569110304</v>
+        <v>6044.239986972274</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>9216.286555169127</v>
+        <v>11986.31303082907</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>14490.75859412626</v>
+        <v>9220.662963388311</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>10553.6857370707</v>
+        <v>14497.67113659201</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -10606,31 +10606,31 @@
         <v>0</v>
       </c>
       <c r="G76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="18" t="n">
         <v>2297.987540800001</v>
       </c>
-      <c r="H76" s="18" t="n">
+      <c r="I76" s="18" t="n">
         <v>4595.975081600001</v>
       </c>
-      <c r="I76" s="18" t="n">
+      <c r="J76" s="18" t="n">
         <v>6893.962622400002</v>
       </c>
-      <c r="J76" s="18" t="n">
+      <c r="K76" s="18" t="n">
         <v>9191.950163200003</v>
       </c>
-      <c r="K76" s="18" t="n">
+      <c r="L76" s="18" t="n">
         <v>11489.937704</v>
       </c>
-      <c r="L76" s="18" t="n">
+      <c r="M76" s="18" t="n">
         <v>13787.9252448</v>
       </c>
-      <c r="M76" s="18" t="n">
+      <c r="N76" s="18" t="n">
         <v>15976.20388899668</v>
       </c>
-      <c r="N76" s="18" t="n">
+      <c r="O76" s="18" t="n">
         <v>18108.77652519336</v>
-      </c>
-      <c r="O76" s="18" t="n">
-        <v>20255.38768139004</v>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
@@ -10709,34 +10709,34 @@
         <v>0</v>
       </c>
       <c r="F78" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="18" t="n">
         <v>2297.987540800001</v>
       </c>
-      <c r="G78" s="18" t="n">
+      <c r="H78" s="18" t="n">
         <v>4595.975081600001</v>
       </c>
-      <c r="H78" s="18" t="n">
+      <c r="I78" s="18" t="n">
         <v>6893.962622400002</v>
       </c>
-      <c r="I78" s="18" t="n">
+      <c r="J78" s="18" t="n">
         <v>9191.950163200003</v>
       </c>
-      <c r="J78" s="18" t="n">
+      <c r="K78" s="18" t="n">
         <v>11489.937704</v>
       </c>
-      <c r="K78" s="18" t="n">
+      <c r="L78" s="18" t="n">
         <v>13787.9252448</v>
       </c>
-      <c r="L78" s="18" t="n">
+      <c r="M78" s="18" t="n">
         <v>15976.20388899668</v>
       </c>
-      <c r="M78" s="18" t="n">
+      <c r="N78" s="18" t="n">
         <v>18108.77652519336</v>
       </c>
-      <c r="N78" s="18" t="n">
+      <c r="O78" s="18" t="n">
         <v>20255.38768139004</v>
-      </c>
-      <c r="O78" s="18" t="n">
-        <v>22429.62387758672</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -10939,16 +10939,16 @@
         <v>2235.34280800426</v>
       </c>
       <c r="L82" s="18" t="n">
-        <v>2333.418320356867</v>
+        <v>2581.38007882974</v>
       </c>
       <c r="M82" s="18" t="n">
-        <v>2670.328871762653</v>
+        <v>2663.031069422604</v>
       </c>
       <c r="N82" s="18" t="n">
-        <v>2990.976933649055</v>
+        <v>2983.683012286244</v>
       </c>
       <c r="O82" s="18" t="n">
-        <v>3295.530488794742</v>
+        <v>3288.233015313682</v>
       </c>
     </row>
     <row r="83" ht="15.5" customHeight="1">
@@ -11095,19 +11095,19 @@
         <v>2235.34280800426</v>
       </c>
       <c r="K85" s="18" t="n">
-        <v>2333.418320356867</v>
+        <v>2581.38007882974</v>
       </c>
       <c r="L85" s="18" t="n">
-        <v>2670.328871762653</v>
+        <v>2663.031069422604</v>
       </c>
       <c r="M85" s="18" t="n">
-        <v>2990.976933649055</v>
+        <v>2983.683012286244</v>
       </c>
       <c r="N85" s="18" t="n">
-        <v>3295.530488794742</v>
+        <v>3288.233015313682</v>
       </c>
       <c r="O85" s="18" t="n">
-        <v>3459.811679300637</v>
+        <v>3452.522549222511</v>
       </c>
     </row>
     <row r="86" ht="15.5" customHeight="1">
@@ -11690,31 +11690,31 @@
         <v>32064.3369271294</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>70256.73964876666</v>
+        <v>68309.99481436772</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>77668.98402070782</v>
+        <v>75382.51716115681</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>80564.05590645724</v>
+        <v>78293.87369160056</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>83556.29956954819</v>
+        <v>81302.26088811038</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>86602.45626049463</v>
+        <v>84364.37794196999</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>60777.46405980636</v>
+        <v>87520.64683999791</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>60608.06570668557</v>
+        <v>61848.35872108494</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>28406.11595012907</v>
+        <v>61827.54338400126</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>27446.18090387545</v>
+        <v>29768.86897180479</v>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
@@ -11899,34 +11899,34 @@
         <v>32064.3369271294</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>70256.73964876666</v>
+        <v>68309.99481436772</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>77668.98402070782</v>
+        <v>75382.51716115681</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>80564.05590645724</v>
+        <v>78293.87369160056</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>83556.29956954819</v>
+        <v>81302.26088811038</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>86602.45626049463</v>
+        <v>84364.37794196999</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>60777.46405980636</v>
+        <v>87520.64683999791</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>60608.06570668557</v>
+        <v>61848.35872108494</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>28406.11595012907</v>
+        <v>61827.54338400126</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>27446.18090387545</v>
+        <v>29768.86897180479</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>31254.51742733913</v>
+        <v>29162.96119886453</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -12058,34 +12058,34 @@
         <v>0</v>
       </c>
       <c r="F103" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" s="18" t="n">
         <v>-1290.176965598953</v>
       </c>
-      <c r="G103" s="18" t="n">
+      <c r="H103" s="18" t="n">
         <v>-1278.65628434995</v>
       </c>
-      <c r="H103" s="18" t="n">
+      <c r="I103" s="18" t="n">
         <v>-1250.850958406641</v>
       </c>
-      <c r="I103" s="18" t="n">
+      <c r="J103" s="18" t="n">
         <v>-1206.902099044447</v>
       </c>
-      <c r="J103" s="18" t="n">
+      <c r="K103" s="18" t="n">
         <v>-1146.99287676908</v>
       </c>
-      <c r="K103" s="18" t="n">
+      <c r="L103" s="18" t="n">
         <v>27.56010391590189</v>
       </c>
-      <c r="L103" s="18" t="n">
+      <c r="M103" s="18" t="n">
         <v>-162.300607879974</v>
       </c>
-      <c r="M103" s="18" t="n">
+      <c r="N103" s="18" t="n">
         <v>-506.8604250494029</v>
       </c>
-      <c r="N103" s="18" t="n">
+      <c r="O103" s="18" t="n">
         <v>-831.0141990278089</v>
-      </c>
-      <c r="O103" s="18" t="n">
-        <v>-1134.919330769903</v>
       </c>
     </row>
     <row r="104" ht="15.5" customHeight="1">
@@ -12267,37 +12267,37 @@
         <v>0</v>
       </c>
       <c r="E107" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" s="18" t="n">
         <v>-1290.176965598953</v>
       </c>
-      <c r="F107" s="18" t="n">
+      <c r="G107" s="18" t="n">
         <v>-1278.65628434995</v>
       </c>
-      <c r="G107" s="18" t="n">
+      <c r="H107" s="18" t="n">
         <v>-1250.850958406641</v>
       </c>
-      <c r="H107" s="18" t="n">
+      <c r="I107" s="18" t="n">
         <v>-1206.902099044447</v>
       </c>
-      <c r="I107" s="18" t="n">
+      <c r="J107" s="18" t="n">
         <v>-1146.99287676908</v>
       </c>
-      <c r="J107" s="18" t="n">
+      <c r="K107" s="18" t="n">
         <v>27.56010391590189</v>
       </c>
-      <c r="K107" s="18" t="n">
+      <c r="L107" s="18" t="n">
         <v>-162.300607879974</v>
       </c>
-      <c r="L107" s="18" t="n">
+      <c r="M107" s="18" t="n">
         <v>-506.8604250494029</v>
       </c>
-      <c r="M107" s="18" t="n">
+      <c r="N107" s="18" t="n">
         <v>-831.0141990278089</v>
       </c>
-      <c r="N107" s="18" t="n">
+      <c r="O107" s="18" t="n">
         <v>-1134.919330769903</v>
-      </c>
-      <c r="O107" s="18" t="n">
-        <v>-1418.804158241069</v>
       </c>
     </row>
     <row r="108" ht="15.5" customHeight="1">
@@ -15150,10 +15150,10 @@
         <v>5.104424374156288</v>
       </c>
       <c r="F48" s="18" t="n">
-        <v>8.056340429786157</v>
+        <v>8.056340429786161</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>11.41773686142088</v>
+        <v>11.41773686142101</v>
       </c>
       <c r="H48" s="18" t="n">
         <v>13.57606858255659</v>
@@ -15168,7 +15168,7 @@
         <v>21.21822690050123</v>
       </c>
       <c r="L48" s="18" t="n">
-        <v>20.65884142905179</v>
+        <v>20.65884142905181</v>
       </c>
       <c r="M48" s="18" t="n">
         <v>21.4393944371938</v>
@@ -15177,7 +15177,7 @@
         <v>20.47513321843181</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>20.73913520283466</v>
+        <v>20.73913520283469</v>
       </c>
     </row>
     <row r="49" ht="15.5" customHeight="1">
@@ -15309,10 +15309,10 @@
         <v>2.291152682690086</v>
       </c>
       <c r="F51" s="18" t="n">
-        <v>5.104424374156284</v>
+        <v>5.104424374156288</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>8.056340429786026</v>
+        <v>8.056340429786157</v>
       </c>
       <c r="H51" s="18" t="n">
         <v>11.41773686142088</v>
@@ -15327,7 +15327,7 @@
         <v>16.82587827879169</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>21.21822690050121</v>
+        <v>21.21822690050123</v>
       </c>
       <c r="M51" s="18" t="n">
         <v>20.65884142905179</v>
@@ -15336,7 +15336,7 @@
         <v>21.4393944371938</v>
       </c>
       <c r="O51" s="18" t="n">
-        <v>20.4751332184318</v>
+        <v>20.47513321843182</v>
       </c>
     </row>
     <row r="52" ht="15.5" customHeight="1">
@@ -15680,10 +15680,10 @@
         <v>5.945813210737497</v>
       </c>
       <c r="F58" s="18" t="n">
-        <v>9.394416556559062</v>
+        <v>9.394416556559065</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>12.87936391270747</v>
+        <v>12.8793639127076</v>
       </c>
       <c r="H58" s="18" t="n">
         <v>15.59517442269535</v>
@@ -15698,7 +15698,7 @@
         <v>21.93274718513492</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>21.78139151426158</v>
+        <v>21.7813915142616</v>
       </c>
       <c r="M58" s="18" t="n">
         <v>22.20819432968727</v>
@@ -15707,7 +15707,7 @@
         <v>21.67117820440262</v>
       </c>
       <c r="O58" s="18" t="n">
-        <v>21.63475059541897</v>
+        <v>21.63475059541899</v>
       </c>
     </row>
     <row r="59" ht="15.5" customHeight="1">
@@ -15733,10 +15733,10 @@
         <v>2.147578652054793</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>2.884258592876716</v>
+        <v>2.884258592876712</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>3.989147340822061</v>
+        <v>3.98914734082193</v>
       </c>
       <c r="H59" s="18" t="n">
         <v>4.655254879726172</v>
@@ -15751,7 +15751,7 @@
         <v>8.774081534794671</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>8.583901296164555</v>
+        <v>8.583901296164534</v>
       </c>
       <c r="M59" s="18" t="n">
         <v>9.154841000548092</v>
@@ -15760,7 +15760,7 @@
         <v>8.944136186301527</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>9.460467493972772</v>
+        <v>9.46046749397275</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -17718,34 +17718,34 @@
         <v>28.63499536848203</v>
       </c>
       <c r="F96" s="20" t="n">
-        <v>99.80486527661515</v>
+        <v>46.10838492845514</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>9467.376180477626</v>
+        <v>120.2419698024263</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>9593.184480557846</v>
+        <v>9503.173980520645</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>9741.710957862753</v>
+        <v>9631.052010628353</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>9943.636880541706</v>
+        <v>9797.281874129625</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>10165.05239837964</v>
+        <v>10000.03467522516</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>10483.29462442817</v>
+        <v>10291.04280007841</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>10855.91608975582</v>
+        <v>10603.67241264335</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>11250.16952585752</v>
+        <v>10990.40506554231</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>11641.8157646981</v>
+        <v>11375.16271087514</v>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
@@ -17927,37 +17927,37 @@
         <v>28.63499536848203</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>99.80486527661515</v>
+        <v>46.10838492845514</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>9467.376180477626</v>
+        <v>120.2419698024263</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>9593.184480557846</v>
+        <v>9503.173980520645</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>9741.710957862753</v>
+        <v>9631.052010628353</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>9943.636880541706</v>
+        <v>9797.281874129625</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>10165.05239837964</v>
+        <v>10000.03467522516</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>10483.29462442817</v>
+        <v>10291.04280007841</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>10855.91608975582</v>
+        <v>10603.67241264335</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>11250.16952585752</v>
+        <v>10990.40506554231</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>11641.8157646981</v>
+        <v>11375.16271087514</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>12052.11672455091</v>
+        <v>11779.19535296211</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -20825,19 +20825,19 @@
         <v>1766.452534384212</v>
       </c>
       <c r="K41" s="18" t="n">
-        <v>1786.918996540068</v>
+        <v>1993.665016356035</v>
       </c>
       <c r="L41" s="18" t="n">
-        <v>1770.030551263489</v>
+        <v>2002.979533996185</v>
       </c>
       <c r="M41" s="18" t="n">
-        <v>2061.788504531658</v>
+        <v>1975.052331649058</v>
       </c>
       <c r="N41" s="18" t="n">
-        <v>2339.717948400777</v>
+        <v>2255.879879015144</v>
       </c>
       <c r="O41" s="18" t="n">
-        <v>2528.282791649973</v>
+        <v>2447.325800475393</v>
       </c>
     </row>
     <row r="42">
@@ -20878,19 +20878,19 @@
         <v>1766.452534384212</v>
       </c>
       <c r="K42" s="18" t="n">
-        <v>1786.918996540068</v>
+        <v>1993.665016356035</v>
       </c>
       <c r="L42" s="18" t="n">
-        <v>1770.030551263489</v>
+        <v>2002.979533996185</v>
       </c>
       <c r="M42" s="18" t="n">
-        <v>2061.788504531658</v>
+        <v>1975.052331649058</v>
       </c>
       <c r="N42" s="18" t="n">
-        <v>2339.717948400777</v>
+        <v>2255.879879015144</v>
       </c>
       <c r="O42" s="18" t="n">
-        <v>2528.282791649973</v>
+        <v>2447.325800475393</v>
       </c>
     </row>
     <row r="43">
@@ -20934,16 +20934,16 @@
         <v>64.73609202675598</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>924.7801340349087</v>
+        <v>69.80570543555764</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>1784.621595696946</v>
+        <v>929.6471670975955</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>2644.243659170675</v>
+        <v>1789.269230571323</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>3507.633497876217</v>
+        <v>2652.659069276866</v>
       </c>
     </row>
     <row r="44">
@@ -20987,16 +20987,16 @@
         <v>0</v>
       </c>
       <c r="L44" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" s="18" t="n">
         <v>854.9744285993511</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>1709.948857198702</v>
       </c>
-      <c r="N44" s="18" t="n">
+      <c r="O44" s="18" t="n">
         <v>2564.923285798053</v>
-      </c>
-      <c r="O44" s="18" t="n">
-        <v>3419.897714397404</v>
       </c>
     </row>
     <row r="45">
@@ -21143,19 +21143,19 @@
         <v>1826.265706300496</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>1851.655088566824</v>
+        <v>2058.401108382791</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>2694.810685298398</v>
+        <v>2072.785239431743</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>3846.410100228605</v>
+        <v>2904.699498746653</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>4983.961607571451</v>
+        <v>4045.149109586468</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>6035.91628952619</v>
+        <v>5099.984869752259</v>
       </c>
     </row>
     <row r="48">
@@ -21199,16 +21199,16 @@
         <v>2043.395419655636</v>
       </c>
       <c r="L48" s="18" t="n">
-        <v>-1498.072029484937</v>
+        <v>2264.207270086744</v>
       </c>
       <c r="M48" s="18" t="n">
-        <v>2077.393187096419</v>
+        <v>-1288.492283290204</v>
       </c>
       <c r="N48" s="18" t="n">
-        <v>-1719.651941391034</v>
+        <v>2275.830548432321</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>3313.662490482477</v>
+        <v>-1603.922354900547</v>
       </c>
     </row>
     <row r="49">
@@ -21358,16 +21358,16 @@
         <v>1811.836825463852</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>-1718.883879916045</v>
+        <v>2043.395419655636</v>
       </c>
       <c r="M51" s="18" t="n">
-        <v>1867.813440901686</v>
+        <v>-1498.072029484937</v>
       </c>
       <c r="N51" s="18" t="n">
-        <v>-1918.089302726937</v>
+        <v>2077.393187096419</v>
       </c>
       <c r="O51" s="18" t="n">
-        <v>3197.932903991988</v>
+        <v>-1719.651941391035</v>
       </c>
     </row>
     <row r="52">
@@ -21408,19 +21408,19 @@
         <v>0</v>
       </c>
       <c r="K52" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="18" t="n">
         <v>-74.11679431732691</v>
       </c>
-      <c r="L52" s="18" t="n">
+      <c r="M52" s="18" t="n">
         <v>420.309520466836</v>
       </c>
-      <c r="M52" s="18" t="n">
+      <c r="N52" s="18" t="n">
         <v>345.7993353962562</v>
       </c>
-      <c r="N52" s="18" t="n">
+      <c r="O52" s="18" t="n">
         <v>277.9086329187738</v>
-      </c>
-      <c r="O52" s="18" t="n">
-        <v>216.5838862209679</v>
       </c>
     </row>
     <row r="53">
@@ -21461,19 +21461,19 @@
         <v>0</v>
       </c>
       <c r="K53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" s="18" t="n">
         <v>-74.11679431732691</v>
       </c>
-      <c r="L53" s="18" t="n">
+      <c r="M53" s="18" t="n">
         <v>420.309520466836</v>
       </c>
-      <c r="M53" s="18" t="n">
+      <c r="N53" s="18" t="n">
         <v>345.7993353962562</v>
       </c>
-      <c r="N53" s="18" t="n">
+      <c r="O53" s="18" t="n">
         <v>277.9086329187738</v>
-      </c>
-      <c r="O53" s="18" t="n">
-        <v>216.5838862209679</v>
       </c>
     </row>
     <row r="54">
@@ -21726,19 +21726,19 @@
         <v>1789.144679924031</v>
       </c>
       <c r="K58" s="18" t="n">
-        <v>1944.413423688509</v>
+        <v>2018.530218005836</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>-1105.003367155397</v>
+        <v>2162.849617632121</v>
       </c>
       <c r="M58" s="18" t="n">
-        <v>2393.672681450797</v>
+        <v>-897.7026038652465</v>
       </c>
       <c r="N58" s="18" t="n">
-        <v>-1473.436142940347</v>
+        <v>2589.937049360491</v>
       </c>
       <c r="O58" s="18" t="n">
-        <v>3494.492675027422</v>
+        <v>-1361.767423657796</v>
       </c>
     </row>
     <row r="59">
@@ -21779,19 +21779,19 @@
         <v>37.1210263764649</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>-92.75833512168492</v>
+        <v>39.87089037695523</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>3799.814052453795</v>
+        <v>-90.06437820037809</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>1452.737418777808</v>
+        <v>3802.4021026119</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>6457.397750511798</v>
+        <v>1455.212060225977</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>2541.423614498768</v>
+        <v>6461.752293410055</v>
       </c>
     </row>
     <row r="60">
@@ -22686,13 +22686,13 @@
         <v>0</v>
       </c>
       <c r="M76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="18" t="n">
         <v>854.9744285993511</v>
       </c>
-      <c r="N76" s="18" t="n">
+      <c r="O76" s="18" t="n">
         <v>1709.948857198702</v>
-      </c>
-      <c r="O76" s="18" t="n">
-        <v>2564.923285798053</v>
       </c>
     </row>
     <row r="77">
@@ -22789,16 +22789,16 @@
         <v>0</v>
       </c>
       <c r="L78" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="18" t="n">
         <v>854.9744285993511</v>
       </c>
-      <c r="M78" s="18" t="n">
+      <c r="N78" s="18" t="n">
         <v>1709.948857198702</v>
       </c>
-      <c r="N78" s="18" t="n">
+      <c r="O78" s="18" t="n">
         <v>2564.923285798053</v>
-      </c>
-      <c r="O78" s="18" t="n">
-        <v>3419.897714397404</v>
       </c>
     </row>
     <row r="79">
@@ -23001,16 +23001,16 @@
         <v>1766.452534384212</v>
       </c>
       <c r="L82" s="18" t="n">
-        <v>1786.918996540068</v>
+        <v>1993.665016356035</v>
       </c>
       <c r="M82" s="18" t="n">
-        <v>1770.030551263489</v>
+        <v>2002.979533996185</v>
       </c>
       <c r="N82" s="18" t="n">
-        <v>2061.788504531658</v>
+        <v>1975.052331649058</v>
       </c>
       <c r="O82" s="18" t="n">
-        <v>2339.717948400777</v>
+        <v>2255.879879015144</v>
       </c>
     </row>
     <row r="83">
@@ -23157,19 +23157,19 @@
         <v>1766.452534384212</v>
       </c>
       <c r="K85" s="18" t="n">
-        <v>1786.918996540068</v>
+        <v>1993.665016356035</v>
       </c>
       <c r="L85" s="18" t="n">
-        <v>1770.030551263489</v>
+        <v>2002.979533996185</v>
       </c>
       <c r="M85" s="18" t="n">
-        <v>2061.788504531658</v>
+        <v>1975.052331649058</v>
       </c>
       <c r="N85" s="18" t="n">
-        <v>2339.717948400777</v>
+        <v>2255.879879015144</v>
       </c>
       <c r="O85" s="18" t="n">
-        <v>2528.282791649973</v>
+        <v>2447.325800475393</v>
       </c>
     </row>
     <row r="86">
@@ -23767,16 +23767,16 @@
         <v>70954.9529217129</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>1654450.493356884</v>
+        <v>71723.14327151733</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>3277819.21466039</v>
+        <v>1655304.099531629</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>4892542.257677892</v>
+        <v>3278755.383447527</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>6545617.765946605</v>
+        <v>4893557.271649791</v>
       </c>
     </row>
     <row r="97">
@@ -23976,19 +23976,19 @@
         <v>70954.9529217129</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>1654450.493356884</v>
+        <v>71723.14327151733</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>3277819.21466039</v>
+        <v>1655304.099531629</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>4892542.257677892</v>
+        <v>3278755.383447527</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>6545617.765946605</v>
+        <v>4893557.271649791</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>8202935.558616287</v>
+        <v>6546850.625414385</v>
       </c>
     </row>
     <row r="101">
@@ -24138,16 +24138,16 @@
         <v>0</v>
       </c>
       <c r="L103" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" s="18" t="n">
         <v>-74.11679431732691</v>
       </c>
-      <c r="M103" s="18" t="n">
+      <c r="N103" s="18" t="n">
         <v>420.309520466836</v>
       </c>
-      <c r="N103" s="18" t="n">
+      <c r="O103" s="18" t="n">
         <v>345.7993353962562</v>
-      </c>
-      <c r="O103" s="18" t="n">
-        <v>277.9086329187738</v>
       </c>
     </row>
     <row r="104">
@@ -24347,19 +24347,19 @@
         <v>0</v>
       </c>
       <c r="K107" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" s="18" t="n">
         <v>-74.11679431732691</v>
       </c>
-      <c r="L107" s="18" t="n">
+      <c r="M107" s="18" t="n">
         <v>420.309520466836</v>
       </c>
-      <c r="M107" s="18" t="n">
+      <c r="N107" s="18" t="n">
         <v>345.7993353962562</v>
       </c>
-      <c r="N107" s="18" t="n">
+      <c r="O107" s="18" t="n">
         <v>277.9086329187738</v>
-      </c>
-      <c r="O107" s="18" t="n">
-        <v>216.5838862209679</v>
       </c>
     </row>
     <row r="108">

</xml_diff>

<commit_message>
Fix Equity - Eop, Cash EoP, Financing Cash Flow, Working Capital calculations in FFSS backend
- Correct formula execution for Equity - Eop, Cash EoP, Financing Cash Flow, and Working Capital in financial statements

- Ensure proper dependency chaining between calculated values
</commit_message>
<xml_diff>
--- a/backend/Rwanda/financial-statements-CleanStep.xlsx
+++ b/backend/Rwanda/financial-statements-CleanStep.xlsx
@@ -2820,37 +2820,37 @@
         <v>214.4942041409722</v>
       </c>
       <c r="E43" s="18" t="n">
-        <v>398.6088913081865</v>
+        <v>143.1469118777542</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>587.4304378040704</v>
+        <v>76.28963154195679</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>780.8834687145394</v>
+        <v>14.06601924845287</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>978.8881601587207</v>
+        <v>-43.59826851291083</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>1181.365821584918</v>
+        <v>-96.78203752802462</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>1355.434436145405</v>
+        <v>-178.3674183405251</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>1500.553585379281</v>
+        <v>-288.8949415881805</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>1648.471549711873</v>
+        <v>-396.4590945504012</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>1798.991516858651</v>
+        <v>-296.4685515654974</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>1952.083620707639</v>
+        <v>-193.9052420449733</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>2157.1935306402</v>
+        <v>-39.32350733554805</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -2870,40 +2870,40 @@
         </is>
       </c>
       <c r="D44" s="18" t="n">
-        <v>214.328410169835</v>
+        <v>214.4942041409722</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>398.060455964663</v>
+        <v>143.1469118777542</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>586.501544715869</v>
+        <v>76.28963154195679</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>779.5817818800881</v>
+        <v>14.06601924845287</v>
       </c>
       <c r="H44" s="18" t="n">
-        <v>977.2212283422532</v>
+        <v>-43.59826851291083</v>
       </c>
       <c r="I44" s="18" t="n">
-        <v>1179.341079854758</v>
+        <v>-96.78203752802462</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>1353.059207393008</v>
+        <v>-178.3674183405251</v>
       </c>
       <c r="K44" s="18" t="n">
-        <v>1497.992424791367</v>
+        <v>-288.8949415881805</v>
       </c>
       <c r="L44" s="18" t="n">
-        <v>1645.8917032564</v>
+        <v>-396.4590945504012</v>
       </c>
       <c r="M44" s="18" t="n">
-        <v>1796.393614369029</v>
+        <v>-296.4685515654974</v>
       </c>
       <c r="N44" s="18" t="n">
-        <v>1949.468281289197</v>
+        <v>-193.9052420449733</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>2154.561362821763</v>
+        <v>-39.32350733554805</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -2976,40 +2976,40 @@
         </is>
       </c>
       <c r="D46" s="18" t="n">
-        <v>0.165793971137203</v>
+        <v>0</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>0.548435343523528</v>
+        <v>0</v>
       </c>
       <c r="F46" s="18" t="n">
-        <v>0.9288930882013798</v>
+        <v>0</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>1.301686834451326</v>
+        <v>0</v>
       </c>
       <c r="H46" s="18" t="n">
-        <v>1.666931816467446</v>
+        <v>0</v>
       </c>
       <c r="I46" s="18" t="n">
-        <v>2.024741730159805</v>
+        <v>0</v>
       </c>
       <c r="J46" s="18" t="n">
-        <v>2.375228752396676</v>
+        <v>0</v>
       </c>
       <c r="K46" s="18" t="n">
-        <v>2.561160587913961</v>
+        <v>0</v>
       </c>
       <c r="L46" s="18" t="n">
-        <v>2.579846455472902</v>
+        <v>0</v>
       </c>
       <c r="M46" s="18" t="n">
-        <v>2.597902489621874</v>
+        <v>0</v>
       </c>
       <c r="N46" s="18" t="n">
-        <v>2.615339418442316</v>
+        <v>0</v>
       </c>
       <c r="O46" s="18" t="n">
-        <v>2.632167818437388</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" ht="15.5" customHeight="1">
@@ -3032,37 +3032,37 @@
         <v>255.7099427978793</v>
       </c>
       <c r="E47" s="18" t="n">
-        <v>512.9801306066329</v>
+        <v>257.5181511762007</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>772.0262143365919</v>
+        <v>260.8854080744783</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>1032.802128707746</v>
+        <v>265.9846792416596</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>1295.257066376957</v>
+        <v>272.7706377053256</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>1559.341063164885</v>
+        <v>281.1932040519421</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>1824.324709765453</v>
+        <v>290.522855279523</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>2088.268647852986</v>
+        <v>298.8201208855246</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>2349.738823795197</v>
+        <v>304.8081795329235</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>2608.591151079998</v>
+        <v>513.1310826558495</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>2864.847962110127</v>
+        <v>718.859099357515</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>3119.342080395842</v>
+        <v>922.825042420094</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -3668,37 +3668,37 @@
         <v>-2.842170943040401e-14</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>50.51073829431505</v>
+        <v>-204.9512411361172</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>101.0214765886302</v>
+        <v>-410.1193296734834</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>151.5322148829453</v>
+        <v>-615.2852345831411</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>202.0429531772604</v>
+        <v>-820.4434754943711</v>
       </c>
       <c r="I59" s="18" t="n">
-        <v>252.5536914715753</v>
+        <v>-1025.594167641367</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>303.0644297658898</v>
+        <v>-1230.73742472004</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>353.5751680602048</v>
+        <v>-1435.873358907256</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>404.0859063545208</v>
+        <v>-1640.844737907753</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>454.5966446488355</v>
+        <v>-1640.863423775313</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>505.1073829431512</v>
+        <v>-1640.881479809461</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>555.6181212374668</v>
+        <v>-1640.898916738281</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -3877,40 +3877,40 @@
         </is>
       </c>
       <c r="D63" s="18" t="n">
-        <v>-0.3315879422744061</v>
+        <v>-0.165793971137203</v>
       </c>
       <c r="E63" s="18" t="n">
-        <v>-0.7652827447726498</v>
+        <v>-0.3826413723863249</v>
       </c>
       <c r="F63" s="18" t="n">
-        <v>-0.7609154893557037</v>
+        <v>-0.3804577446778519</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>-0.7455874924998922</v>
+        <v>-0.3727937462499461</v>
       </c>
       <c r="H63" s="18" t="n">
-        <v>-0.7304899640322402</v>
+        <v>-0.3652449820161201</v>
       </c>
       <c r="I63" s="18" t="n">
-        <v>-0.7156198273847183</v>
+        <v>-0.3578099136923591</v>
       </c>
       <c r="J63" s="18" t="n">
-        <v>-0.7009740444737416</v>
+        <v>-0.3504870222368708</v>
       </c>
       <c r="K63" s="18" t="n">
-        <v>-0.3718636710345704</v>
+        <v>-0.1859318355172852</v>
       </c>
       <c r="L63" s="18" t="n">
-        <v>-0.0373717351178815</v>
+        <v>-0.01868586755894075</v>
       </c>
       <c r="M63" s="18" t="n">
-        <v>-0.03611206829794344</v>
+        <v>-0.01805603414897172</v>
       </c>
       <c r="N63" s="18" t="n">
-        <v>-0.03487385764088469</v>
+        <v>-0.01743692882044234</v>
       </c>
       <c r="O63" s="18" t="n">
-        <v>-0.03365679999014493</v>
+        <v>-0.01682839999507246</v>
       </c>
     </row>
     <row r="64" ht="15.5" customHeight="1">
@@ -3930,40 +3930,40 @@
         </is>
       </c>
       <c r="D64" s="18" t="n">
-        <v>1.460190975003197</v>
+        <v>1.625984946140401</v>
       </c>
       <c r="E64" s="18" t="n">
-        <v>4.99087470960171</v>
+        <v>5.373516081988035</v>
       </c>
       <c r="F64" s="18" t="n">
-        <v>8.934367522239267</v>
+        <v>9.314825266917119</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>12.8156212929488</v>
+        <v>13.18841503919875</v>
       </c>
       <c r="H64" s="18" t="n">
-        <v>16.62451489501482</v>
+        <v>16.98975987703095</v>
       </c>
       <c r="I64" s="18" t="n">
-        <v>20.3621074064332</v>
+        <v>20.71991732012555</v>
       </c>
       <c r="J64" s="18" t="n">
-        <v>24.29399593498742</v>
+        <v>24.64448295722429</v>
       </c>
       <c r="K64" s="18" t="n">
-        <v>27.3536017460136</v>
+        <v>27.53953358153089</v>
       </c>
       <c r="L64" s="18" t="n">
-        <v>28.94249711461765</v>
+        <v>28.96118298217659</v>
       </c>
       <c r="M64" s="18" t="n">
-        <v>30.18173572112492</v>
+        <v>30.19979175527389</v>
       </c>
       <c r="N64" s="18" t="n">
-        <v>31.40473142798594</v>
+        <v>31.42216835680638</v>
       </c>
       <c r="O64" s="18" t="n">
-        <v>31.99105165766475</v>
+        <v>32.00788005765983</v>
       </c>
     </row>
     <row r="65" ht="15.5" customHeight="1">
@@ -4089,40 +4089,40 @@
         </is>
       </c>
       <c r="D67" s="18" t="n">
-        <v>-40.96777528946001</v>
+        <v>-40.80198131832281</v>
       </c>
       <c r="E67" s="18" t="n">
-        <v>-71.56413966446706</v>
+        <v>-71.18149829208075</v>
       </c>
       <c r="F67" s="18" t="n">
-        <v>-66.85509670808896</v>
+        <v>-66.47463896341111</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>-62.215948295076</v>
+        <v>-61.84315454882606</v>
       </c>
       <c r="H67" s="18" t="n">
-        <v>-57.65673899712989</v>
+        <v>-57.29149401511377</v>
       </c>
       <c r="I67" s="18" t="n">
-        <v>-53.17633394679002</v>
+        <v>-52.81852403309767</v>
       </c>
       <c r="J67" s="18" t="n">
-        <v>-81.57805792104502</v>
+        <v>-81.22757089880815</v>
       </c>
       <c r="K67" s="18" t="n">
-        <v>-110.3629680609358</v>
+        <v>-110.1770362254185</v>
       </c>
       <c r="L67" s="18" t="n">
-        <v>-107.3969069942623</v>
+        <v>-107.3782211267033</v>
       </c>
       <c r="M67" s="18" t="n">
-        <v>-104.7942743466662</v>
+        <v>-104.7762183125172</v>
       </c>
       <c r="N67" s="18" t="n">
-        <v>-102.2215185391273</v>
+        <v>-102.2040816103068</v>
       </c>
       <c r="O67" s="18" t="n">
-        <v>-50.20310392672924</v>
+        <v>-50.18627552673417</v>
       </c>
     </row>
     <row r="68" ht="15.5" customHeight="1">
@@ -4463,37 +4463,37 @@
         <v>255.296185459295</v>
       </c>
       <c r="E74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="F74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="H74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="I74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="J74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="K74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="L74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="M74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="N74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
       <c r="O74" s="18" t="n">
-        <v>255.296185459295</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" ht="15.5" customHeight="1">
@@ -4513,40 +4513,40 @@
         </is>
       </c>
       <c r="D75" s="18" t="n">
-        <v>214.328410169835</v>
+        <v>214.4942041409722</v>
       </c>
       <c r="E75" s="18" t="n">
-        <v>183.732045794828</v>
+        <v>-71.18149829208075</v>
       </c>
       <c r="F75" s="18" t="n">
-        <v>188.4410887512061</v>
+        <v>-66.47463896341111</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>193.080237164219</v>
+        <v>-61.84315454882606</v>
       </c>
       <c r="H75" s="18" t="n">
-        <v>197.6394464621652</v>
+        <v>-57.29149401511377</v>
       </c>
       <c r="I75" s="18" t="n">
-        <v>202.119851512505</v>
+        <v>-52.81852403309767</v>
       </c>
       <c r="J75" s="18" t="n">
-        <v>173.71812753825</v>
+        <v>-81.22757089880815</v>
       </c>
       <c r="K75" s="18" t="n">
-        <v>144.9332173983592</v>
+        <v>-110.1770362254185</v>
       </c>
       <c r="L75" s="18" t="n">
-        <v>147.8992784650328</v>
+        <v>-107.3782211267033</v>
       </c>
       <c r="M75" s="18" t="n">
-        <v>150.5019111126289</v>
+        <v>-104.7762183125172</v>
       </c>
       <c r="N75" s="18" t="n">
-        <v>153.0746669201678</v>
+        <v>-102.2040816103068</v>
       </c>
       <c r="O75" s="18" t="n">
-        <v>205.0930815325658</v>
+        <v>-50.18627552673417</v>
       </c>
     </row>
     <row r="76" ht="15.5" customHeight="1">
@@ -4569,37 +4569,37 @@
         <v>0</v>
       </c>
       <c r="E76" s="18" t="n">
-        <v>214.328410169835</v>
+        <v>214.4942041409722</v>
       </c>
       <c r="F76" s="18" t="n">
-        <v>398.060455964663</v>
+        <v>143.1469118777542</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>586.501544715869</v>
+        <v>76.28963154195679</v>
       </c>
       <c r="H76" s="18" t="n">
-        <v>779.5817818800881</v>
+        <v>14.06601924845287</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>977.2212283422532</v>
+        <v>-43.59826851291083</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>1179.341079854758</v>
+        <v>-96.78203752802462</v>
       </c>
       <c r="K76" s="18" t="n">
-        <v>1353.059207393008</v>
+        <v>-178.3674183405251</v>
       </c>
       <c r="L76" s="18" t="n">
-        <v>1497.992424791367</v>
+        <v>-288.8949415881805</v>
       </c>
       <c r="M76" s="18" t="n">
-        <v>1645.8917032564</v>
+        <v>-396.4590945504012</v>
       </c>
       <c r="N76" s="18" t="n">
-        <v>1796.393614369029</v>
+        <v>-296.4685515654974</v>
       </c>
       <c r="O76" s="18" t="n">
-        <v>1949.468281289197</v>
+        <v>-193.9052420449733</v>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
@@ -4619,40 +4619,40 @@
         </is>
       </c>
       <c r="D77" s="18" t="n">
-        <v>214.328410169835</v>
+        <v>214.4942041409722</v>
       </c>
       <c r="E77" s="18" t="n">
-        <v>183.732045794828</v>
+        <v>-71.18149829208075</v>
       </c>
       <c r="F77" s="18" t="n">
-        <v>188.4410887512061</v>
+        <v>-66.47463896341111</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>193.080237164219</v>
+        <v>-61.84315454882606</v>
       </c>
       <c r="H77" s="18" t="n">
-        <v>197.6394464621652</v>
+        <v>-57.29149401511377</v>
       </c>
       <c r="I77" s="18" t="n">
-        <v>202.119851512505</v>
+        <v>-52.81852403309767</v>
       </c>
       <c r="J77" s="18" t="n">
-        <v>173.71812753825</v>
+        <v>-81.22757089880815</v>
       </c>
       <c r="K77" s="18" t="n">
-        <v>144.9332173983592</v>
+        <v>-110.1770362254185</v>
       </c>
       <c r="L77" s="18" t="n">
-        <v>147.8992784650328</v>
+        <v>-107.3782211267033</v>
       </c>
       <c r="M77" s="18" t="n">
-        <v>150.5019111126289</v>
+        <v>-104.7762183125172</v>
       </c>
       <c r="N77" s="18" t="n">
-        <v>153.0746669201678</v>
+        <v>-102.2040816103068</v>
       </c>
       <c r="O77" s="18" t="n">
-        <v>205.0930815325658</v>
+        <v>-50.18627552673417</v>
       </c>
     </row>
     <row r="78" ht="15.5" customHeight="1">
@@ -4672,40 +4672,40 @@
         </is>
       </c>
       <c r="D78" s="18" t="n">
-        <v>214.328410169835</v>
+        <v>214.4942041409722</v>
       </c>
       <c r="E78" s="18" t="n">
-        <v>398.060455964663</v>
+        <v>143.1469118777542</v>
       </c>
       <c r="F78" s="18" t="n">
-        <v>586.501544715869</v>
+        <v>76.28963154195679</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>779.5817818800881</v>
+        <v>14.06601924845287</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>977.2212283422532</v>
+        <v>-43.59826851291083</v>
       </c>
       <c r="I78" s="18" t="n">
-        <v>1179.341079854758</v>
+        <v>-96.78203752802462</v>
       </c>
       <c r="J78" s="18" t="n">
-        <v>1353.059207393008</v>
+        <v>-178.3674183405251</v>
       </c>
       <c r="K78" s="18" t="n">
-        <v>1497.992424791367</v>
+        <v>-288.8949415881805</v>
       </c>
       <c r="L78" s="18" t="n">
-        <v>1645.8917032564</v>
+        <v>-396.4590945504012</v>
       </c>
       <c r="M78" s="18" t="n">
-        <v>1796.393614369029</v>
+        <v>-296.4685515654974</v>
       </c>
       <c r="N78" s="18" t="n">
-        <v>1949.468281289197</v>
+        <v>-193.9052420449733</v>
       </c>
       <c r="O78" s="18" t="n">
-        <v>2154.561362821763</v>
+        <v>-39.32350733554805</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -5202,40 +5202,40 @@
         </is>
       </c>
       <c r="D88" s="18" t="n">
-        <v>0.165793971137203</v>
+        <v>0</v>
       </c>
       <c r="E88" s="18" t="n">
-        <v>0.548435343523528</v>
+        <v>0</v>
       </c>
       <c r="F88" s="18" t="n">
-        <v>0.9288930882013798</v>
+        <v>0</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>1.301686834451326</v>
+        <v>0</v>
       </c>
       <c r="H88" s="18" t="n">
-        <v>1.666931816467446</v>
+        <v>0</v>
       </c>
       <c r="I88" s="18" t="n">
-        <v>2.024741730159805</v>
+        <v>0</v>
       </c>
       <c r="J88" s="18" t="n">
-        <v>2.375228752396676</v>
+        <v>0</v>
       </c>
       <c r="K88" s="18" t="n">
-        <v>2.561160587913961</v>
+        <v>0</v>
       </c>
       <c r="L88" s="18" t="n">
-        <v>2.579846455472902</v>
+        <v>0</v>
       </c>
       <c r="M88" s="18" t="n">
-        <v>2.597902489621874</v>
+        <v>0</v>
       </c>
       <c r="N88" s="18" t="n">
-        <v>2.615339418442316</v>
+        <v>0</v>
       </c>
       <c r="O88" s="18" t="n">
-        <v>2.632167818437388</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" ht="15.5" customHeight="1">
@@ -5308,40 +5308,40 @@
         </is>
       </c>
       <c r="D90" s="18" t="n">
-        <v>0.3315879422744061</v>
+        <v>0.165793971137203</v>
       </c>
       <c r="E90" s="18" t="n">
-        <v>1.096870687047056</v>
+        <v>0.548435343523528</v>
       </c>
       <c r="F90" s="18" t="n">
-        <v>1.85778617640276</v>
+        <v>0.9288930882013798</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>2.603373668902652</v>
+        <v>1.301686834451326</v>
       </c>
       <c r="H90" s="18" t="n">
-        <v>3.333863632934892</v>
+        <v>1.666931816467446</v>
       </c>
       <c r="I90" s="18" t="n">
-        <v>4.04948346031961</v>
+        <v>2.024741730159805</v>
       </c>
       <c r="J90" s="18" t="n">
-        <v>4.750457504793352</v>
+        <v>2.375228752396676</v>
       </c>
       <c r="K90" s="18" t="n">
-        <v>5.122321175827922</v>
+        <v>2.561160587913961</v>
       </c>
       <c r="L90" s="18" t="n">
-        <v>5.159692910945804</v>
+        <v>2.579846455472902</v>
       </c>
       <c r="M90" s="18" t="n">
-        <v>5.195804979243747</v>
+        <v>2.597902489621874</v>
       </c>
       <c r="N90" s="18" t="n">
-        <v>5.230678836884632</v>
+        <v>2.615339418442316</v>
       </c>
       <c r="O90" s="18" t="n">
-        <v>5.264335636874777</v>
+        <v>2.632167818437388</v>
       </c>
     </row>
     <row r="91" ht="15.5" customHeight="1">
@@ -5361,40 +5361,40 @@
         </is>
       </c>
       <c r="D91" s="18" t="n">
-        <v>0.3315879422744061</v>
+        <v>0.165793971137203</v>
       </c>
       <c r="E91" s="18" t="n">
-        <v>0.7652827447726498</v>
+        <v>0.3826413723863249</v>
       </c>
       <c r="F91" s="18" t="n">
-        <v>0.7609154893557037</v>
+        <v>0.3804577446778519</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>0.7455874924998922</v>
+        <v>0.3727937462499461</v>
       </c>
       <c r="H91" s="18" t="n">
-        <v>0.7304899640322402</v>
+        <v>0.3652449820161201</v>
       </c>
       <c r="I91" s="18" t="n">
-        <v>0.7156198273847183</v>
+        <v>0.3578099136923591</v>
       </c>
       <c r="J91" s="18" t="n">
-        <v>0.7009740444737416</v>
+        <v>0.3504870222368708</v>
       </c>
       <c r="K91" s="18" t="n">
-        <v>0.3718636710345704</v>
+        <v>0.1859318355172852</v>
       </c>
       <c r="L91" s="18" t="n">
-        <v>0.0373717351178815</v>
+        <v>0.01868586755894075</v>
       </c>
       <c r="M91" s="18" t="n">
-        <v>0.03611206829794344</v>
+        <v>0.01805603414897172</v>
       </c>
       <c r="N91" s="18" t="n">
-        <v>0.03487385764088469</v>
+        <v>0.01743692882044234</v>
       </c>
       <c r="O91" s="18" t="n">
-        <v>0.03365679999014493</v>
+        <v>0.01682839999507246</v>
       </c>
     </row>
     <row r="92" ht="15.5" customHeight="1">
@@ -5656,34 +5656,34 @@
         <v>58.65648807822183</v>
       </c>
       <c r="F96" s="20" t="n">
-        <v>125.1759605419378</v>
+        <v>74.66522224762269</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>193.3326243946752</v>
+        <v>92.31114780604497</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>263.0762991947491</v>
+        <v>111.5440843118037</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>334.3576443901693</v>
+        <v>132.3146912129088</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>407.1281475388908</v>
+        <v>154.5744560673152</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>486.557045396698</v>
+        <v>183.4926156308073</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>570.4605265326414</v>
+        <v>216.8853584724357</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>651.4774089715255</v>
+        <v>247.3915026170047</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>729.6326782416476</v>
+        <v>275.0360335928117</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>804.951108820609</v>
+        <v>299.843725877458</v>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
@@ -5865,37 +5865,37 @@
         <v>58.65648807822183</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>125.1759605419378</v>
+        <v>74.66522224762269</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>193.3326243946752</v>
+        <v>92.31114780604497</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>263.0762991947491</v>
+        <v>111.5440843118037</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>334.3576443901693</v>
+        <v>132.3146912129088</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>407.1281475388908</v>
+        <v>154.5744560673152</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>486.557045396698</v>
+        <v>183.4926156308073</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>570.4605265326414</v>
+        <v>216.8853584724357</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>651.4774089715255</v>
+        <v>247.3915026170047</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>729.6326782416476</v>
+        <v>275.0360335928117</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>804.951108820609</v>
+        <v>299.843725877458</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>869.3343293995</v>
+        <v>313.7162081620339</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -8848,40 +8848,40 @@
         </is>
       </c>
       <c r="D43" s="18" t="n">
-        <v>943.5758334107996</v>
+        <v>920.8667375203886</v>
       </c>
       <c r="E43" s="18" t="n">
-        <v>1804.330947065474</v>
+        <v>693.9349505956635</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>2696.001250243566</v>
+        <v>489.8101739751198</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>3599.515955270006</v>
+        <v>299.7152161716678</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>4533.46039089128</v>
+        <v>138.2558748332219</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>5495.699193841769</v>
+        <v>5.121607673304986</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>6445.1142282773</v>
+        <v>-140.7817047138968</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>7396.076523795097</v>
+        <v>-286.1344875256816</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>8390.089435710555</v>
+        <v>-388.761311474055</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>9426.488326929337</v>
+        <v>331.2311499284457</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>10503.91472074392</v>
+        <v>1092.402182419898</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>11603.23802649004</v>
+        <v>1902.858096705899</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -8901,40 +8901,40 @@
         </is>
       </c>
       <c r="D44" s="18" t="n">
-        <v>929.4422221198872</v>
+        <v>898.1576416299777</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>1787.887758963044</v>
+        <v>667.6847368970334</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>2676.711710517538</v>
+        <v>459.2546068518321</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>3579.30751143439</v>
+        <v>266.8122517881062</v>
       </c>
       <c r="H44" s="18" t="n">
-        <v>4510.539848425527</v>
+        <v>101.2419077099342</v>
       </c>
       <c r="I44" s="18" t="n">
-        <v>5470.098081513001</v>
+        <v>-35.94306629929775</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>6416.886447455382</v>
+        <v>-185.8135951248557</v>
       </c>
       <c r="K44" s="18" t="n">
-        <v>7363.677123795098</v>
+        <v>-336.1007368407501</v>
       </c>
       <c r="L44" s="18" t="n">
-        <v>8353.345813792746</v>
+        <v>-443.4087690083016</v>
       </c>
       <c r="M44" s="18" t="n">
-        <v>9385.534488573172</v>
+        <v>272.0463526681717</v>
       </c>
       <c r="N44" s="18" t="n">
-        <v>10458.90355911936</v>
+        <v>1028.840976940446</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>11551.62482649004</v>
+        <v>1832.384348760694</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -9007,40 +9007,40 @@
         </is>
       </c>
       <c r="D46" s="18" t="n">
-        <v>-8.575484599498539</v>
+        <v>0</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>-9.807025596199978</v>
+        <v>0</v>
       </c>
       <c r="F46" s="18" t="n">
-        <v>-11.26602739726027</v>
+        <v>0</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>-12.69452054794521</v>
+        <v>0</v>
       </c>
       <c r="H46" s="18" t="n">
-        <v>-14.09342465753425</v>
+        <v>0</v>
       </c>
       <c r="I46" s="18" t="n">
-        <v>-15.46356164383562</v>
+        <v>0</v>
       </c>
       <c r="J46" s="18" t="n">
-        <v>-16.8041095890411</v>
+        <v>0</v>
       </c>
       <c r="K46" s="18" t="n">
-        <v>-17.5668493150685</v>
+        <v>0</v>
       </c>
       <c r="L46" s="18" t="n">
-        <v>-17.90383561643835</v>
+        <v>0</v>
       </c>
       <c r="M46" s="18" t="n">
-        <v>-18.23095890410959</v>
+        <v>0</v>
       </c>
       <c r="N46" s="18" t="n">
-        <v>-18.55004385489041</v>
+        <v>0</v>
       </c>
       <c r="O46" s="18" t="n">
-        <v>-18.86054794520548</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" ht="15.5" customHeight="1">
@@ -9060,40 +9060,40 @@
         </is>
       </c>
       <c r="D47" s="18" t="n">
-        <v>1231.438849026531</v>
+        <v>1208.72975313612</v>
       </c>
       <c r="E47" s="18" t="n">
-        <v>2446.919360341155</v>
+        <v>1336.523363871345</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>3678.393742156435</v>
+        <v>1472.202665887989</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>4906.93548798753</v>
+        <v>1607.134748889192</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>6151.282564959251</v>
+        <v>1756.078048901192</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>7409.441017800518</v>
+        <v>1918.863431632054</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>8680.457036281561</v>
+        <v>2094.561103290363</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>9977.456602624838</v>
+        <v>2295.245591304059</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>11301.08226360603</v>
+        <v>2522.231516421421</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>12650.8352953484</v>
+        <v>3555.578118347514</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>14025.51777082762</v>
+        <v>4614.005232503593</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>15281.8331370015</v>
+        <v>5581.453207217364</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -9143,10 +9143,10 @@
         <v>2738.928132847911</v>
       </c>
       <c r="N48" s="18" t="n">
-        <v>2938.086417382266</v>
+        <v>3016.193847786481</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>3108.863491970128</v>
+        <v>3179.787946589689</v>
       </c>
     </row>
     <row r="49" ht="15.5" customHeight="1">
@@ -9252,7 +9252,7 @@
         <v>277.2657149385706</v>
       </c>
       <c r="O50" s="18" t="n">
-        <v>156.3710522471393</v>
+        <v>163.5940988032079</v>
       </c>
     </row>
     <row r="51" ht="15.5" customHeight="1">
@@ -9302,10 +9302,10 @@
         <v>2174.554755098293</v>
       </c>
       <c r="N51" s="18" t="n">
-        <v>2348.614626052073</v>
+        <v>2426.722056456288</v>
       </c>
       <c r="O51" s="18" t="n">
-        <v>2640.286363331365</v>
+        <v>2703.987771394859</v>
       </c>
     </row>
     <row r="52" ht="15.5" customHeight="1">
@@ -9349,16 +9349,16 @@
         <v>5463.606336853395</v>
       </c>
       <c r="L52" s="18" t="n">
-        <v>6322.228958236666</v>
+        <v>6244.121527832452</v>
       </c>
       <c r="M52" s="18" t="n">
-        <v>7088.338126875001</v>
+        <v>7024.636718811508</v>
       </c>
       <c r="N52" s="18" t="n">
-        <v>7966.541676578826</v>
+        <v>7805.151909790565</v>
       </c>
       <c r="O52" s="18" t="n">
-        <v>8731.818232389202</v>
+        <v>8585.66710076962</v>
       </c>
     </row>
     <row r="53" ht="15.5" customHeight="1">
@@ -9402,16 +9402,16 @@
         <v>5463.606336853395</v>
       </c>
       <c r="L53" s="18" t="n">
-        <v>6322.228958236666</v>
+        <v>6244.121527832452</v>
       </c>
       <c r="M53" s="18" t="n">
-        <v>7088.338126875001</v>
+        <v>7024.636718811508</v>
       </c>
       <c r="N53" s="18" t="n">
-        <v>7966.541676578826</v>
+        <v>7805.151909790565</v>
       </c>
       <c r="O53" s="18" t="n">
-        <v>8731.818232389202</v>
+        <v>8585.66710076962</v>
       </c>
     </row>
     <row r="54" ht="15.5" customHeight="1">
@@ -9667,16 +9667,16 @@
         <v>7742.047818568413</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>8826.89362534302</v>
+        <v>8748.786194938806</v>
       </c>
       <c r="M58" s="18" t="n">
-        <v>9845.497218627021</v>
+        <v>9781.795810563528</v>
       </c>
       <c r="N58" s="18" t="n">
-        <v>10923.17813781598</v>
+        <v>10839.89580143194</v>
       </c>
       <c r="O58" s="18" t="n">
-        <v>11859.54227230453</v>
+        <v>11784.31559530452</v>
       </c>
     </row>
     <row r="59" ht="15.5" customHeight="1">
@@ -9696,40 +9696,40 @@
         </is>
       </c>
       <c r="D59" s="18" t="n">
-        <v>22.70909589041071</v>
+        <v>-2.273736754432321e-13</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>338.4562900902529</v>
+        <v>-771.9397063795579</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>654.9677199065327</v>
+        <v>-1551.223356361913</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>969.5211935584284</v>
+        <v>-2330.27954553991</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>1285.838272689777</v>
+        <v>-3109.366243368282</v>
       </c>
       <c r="I59" s="18" t="n">
-        <v>1602.095055930716</v>
+        <v>-3888.482530237748</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>1918.268348760695</v>
+        <v>-4667.627584230503</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>2235.408784056424</v>
+        <v>-5446.802227264355</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>2474.188638263013</v>
+        <v>-6226.554678517385</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>2805.338076721384</v>
+        <v>-6226.217692216014</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>3102.339633011634</v>
+        <v>-6225.890568928343</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>3422.29086469697</v>
+        <v>-6202.862388087151</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -9908,40 +9908,40 @@
         </is>
       </c>
       <c r="D63" s="18" t="n">
-        <v>17.15096919899708</v>
+        <v>-14.13361129091242</v>
       </c>
       <c r="E63" s="18" t="n">
-        <v>2.463081993402877</v>
+        <v>-2.309576811517742</v>
       </c>
       <c r="F63" s="18" t="n">
-        <v>2.918003602120589</v>
+        <v>-2.84635162359724</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>2.856986301369869</v>
+        <v>-0.9189041095890396</v>
       </c>
       <c r="H63" s="18" t="n">
-        <v>2.797808219178084</v>
+        <v>-2.712098630136989</v>
       </c>
       <c r="I63" s="18" t="n">
-        <v>2.740273972602736</v>
+        <v>-2.680569863013694</v>
       </c>
       <c r="J63" s="18" t="n">
-        <v>2.681095890410962</v>
+        <v>-2.626668493150682</v>
       </c>
       <c r="K63" s="18" t="n">
-        <v>1.525479452054796</v>
+        <v>-4.171619178082196</v>
       </c>
       <c r="L63" s="18" t="n">
-        <v>0.6739726027397168</v>
+        <v>-4.344221917808227</v>
       </c>
       <c r="M63" s="18" t="n">
-        <v>0.6542465753424693</v>
+        <v>-4.210216438356156</v>
       </c>
       <c r="N63" s="18" t="n">
-        <v>0.6381699015616462</v>
+        <v>-4.057323268397262</v>
       </c>
       <c r="O63" s="18" t="n">
-        <v>0.6210081806301346</v>
+        <v>-6.602038375438362</v>
       </c>
     </row>
     <row r="64" ht="15.5" customHeight="1">
@@ -9961,40 +9961,40 @@
         </is>
       </c>
       <c r="D64" s="18" t="n">
-        <v>133.515706118343</v>
+        <v>102.2311256284335</v>
       </c>
       <c r="E64" s="18" t="n">
-        <v>140.66931857446</v>
+        <v>135.8966597695394</v>
       </c>
       <c r="F64" s="18" t="n">
-        <v>167.3015827947773</v>
+        <v>161.5372275690594</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>177.3597431710254</v>
+        <v>173.5838527600665</v>
       </c>
       <c r="H64" s="18" t="n">
-        <v>202.3247271490623</v>
+        <v>196.8148202997473</v>
       </c>
       <c r="I64" s="18" t="n">
-        <v>227.0108866701136</v>
+        <v>221.5900428344972</v>
       </c>
       <c r="J64" s="18" t="n">
-        <v>251.4519788299881</v>
+        <v>246.1442144464265</v>
       </c>
       <c r="K64" s="18" t="n">
-        <v>288.0960220966529</v>
+        <v>282.3989234665158</v>
       </c>
       <c r="L64" s="18" t="n">
-        <v>326.6328696233085</v>
+        <v>321.6146751027605</v>
       </c>
       <c r="M64" s="18" t="n">
-        <v>364.8567999361223</v>
+        <v>359.9923369224236</v>
       </c>
       <c r="N64" s="18" t="n">
-        <v>401.7820138576175</v>
+        <v>397.0865206876585</v>
       </c>
       <c r="O64" s="18" t="n">
-        <v>458.8785621480164</v>
+        <v>451.6555155919479</v>
       </c>
     </row>
     <row r="65" ht="15.5" customHeight="1">
@@ -10120,40 +10120,40 @@
         </is>
       </c>
       <c r="D67" s="18" t="n">
-        <v>-163.2790452507919</v>
+        <v>-194.5636257407014</v>
       </c>
       <c r="E67" s="18" t="n">
-        <v>-234.2757305275222</v>
+        <v>-239.0483893324428</v>
       </c>
       <c r="F67" s="18" t="n">
-        <v>-203.897315816185</v>
+        <v>-209.6616710419028</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>-190.1254664538273</v>
+        <v>-193.9013568647862</v>
       </c>
       <c r="H67" s="18" t="n">
-        <v>-161.4889303795418</v>
+        <v>-166.9988372288569</v>
       </c>
       <c r="I67" s="18" t="n">
-        <v>-133.1630342832046</v>
+        <v>-138.583878118821</v>
       </c>
       <c r="J67" s="18" t="n">
-        <v>-145.9329014282977</v>
+        <v>-151.2406658118593</v>
       </c>
       <c r="K67" s="18" t="n">
-        <v>-145.9305910309628</v>
+        <v>-151.6276896610998</v>
       </c>
       <c r="L67" s="18" t="n">
-        <v>-103.0525773730309</v>
+        <v>-108.0707718935789</v>
       </c>
       <c r="M67" s="18" t="n">
-        <v>-60.53259259025373</v>
+        <v>-65.39705560395237</v>
       </c>
       <c r="N67" s="18" t="n">
-        <v>-19.35219682449474</v>
+        <v>-24.04768999445366</v>
       </c>
       <c r="O67" s="18" t="n">
-        <v>169.7671318367248</v>
+        <v>162.5440852806563</v>
       </c>
     </row>
     <row r="68" ht="15.5" customHeight="1">
@@ -10418,7 +10418,7 @@
         <v>0</v>
       </c>
       <c r="O72" s="18" t="n">
-        <v>-169.7671318367248</v>
+        <v>-162.5440852806563</v>
       </c>
     </row>
     <row r="73" ht="15.5" customHeight="1">
@@ -10494,37 +10494,37 @@
         <v>1092.721267370679</v>
       </c>
       <c r="E74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="F74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="H74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="I74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="J74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="K74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="L74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="M74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="N74" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
       <c r="O74" s="18" t="n">
-        <v>922.9541355339543</v>
+        <v>-162.5440852806563</v>
       </c>
     </row>
     <row r="75" ht="15.5" customHeight="1">
@@ -10544,40 +10544,40 @@
         </is>
       </c>
       <c r="D75" s="18" t="n">
-        <v>929.4422221198872</v>
+        <v>898.1576416299777</v>
       </c>
       <c r="E75" s="18" t="n">
-        <v>858.4455368431568</v>
+        <v>-239.0483893324428</v>
       </c>
       <c r="F75" s="18" t="n">
-        <v>888.823951554494</v>
+        <v>-209.6616710419028</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>902.5958009168517</v>
+        <v>-193.9013568647862</v>
       </c>
       <c r="H75" s="18" t="n">
-        <v>931.2323369911371</v>
+        <v>-166.9988372288569</v>
       </c>
       <c r="I75" s="18" t="n">
-        <v>959.5582330874744</v>
+        <v>-138.583878118821</v>
       </c>
       <c r="J75" s="18" t="n">
-        <v>946.7883659423813</v>
+        <v>-151.2406658118593</v>
       </c>
       <c r="K75" s="18" t="n">
-        <v>946.7906763397162</v>
+        <v>-151.6276896610998</v>
       </c>
       <c r="L75" s="18" t="n">
-        <v>989.668689997648</v>
+        <v>-108.0707718935789</v>
       </c>
       <c r="M75" s="18" t="n">
-        <v>1032.188674780425</v>
+        <v>-65.39705560395237</v>
       </c>
       <c r="N75" s="18" t="n">
-        <v>1073.369070546184</v>
+        <v>-24.04768999445366</v>
       </c>
       <c r="O75" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" ht="15.5" customHeight="1">
@@ -10600,37 +10600,37 @@
         <v>0</v>
       </c>
       <c r="E76" s="18" t="n">
-        <v>929.4422221198872</v>
+        <v>898.1576416299777</v>
       </c>
       <c r="F76" s="18" t="n">
-        <v>1787.887758963044</v>
+        <v>667.6847368970334</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>2676.711710517538</v>
+        <v>459.2546068518321</v>
       </c>
       <c r="H76" s="18" t="n">
-        <v>3579.30751143439</v>
+        <v>266.8122517881062</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>4510.539848425527</v>
+        <v>101.2419077099342</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>5470.098081513001</v>
+        <v>-35.94306629929775</v>
       </c>
       <c r="K76" s="18" t="n">
-        <v>6416.886447455382</v>
+        <v>-185.8135951248557</v>
       </c>
       <c r="L76" s="18" t="n">
-        <v>7363.677123795098</v>
+        <v>-336.1007368407501</v>
       </c>
       <c r="M76" s="18" t="n">
-        <v>8353.345813792746</v>
+        <v>-443.4087690083016</v>
       </c>
       <c r="N76" s="18" t="n">
-        <v>9385.534488573172</v>
+        <v>272.0463526681717</v>
       </c>
       <c r="O76" s="18" t="n">
-        <v>10458.90355911936</v>
+        <v>1028.840976940446</v>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
@@ -10650,40 +10650,40 @@
         </is>
       </c>
       <c r="D77" s="18" t="n">
-        <v>929.4422221198872</v>
+        <v>898.1576416299777</v>
       </c>
       <c r="E77" s="18" t="n">
-        <v>858.4455368431568</v>
+        <v>-239.0483893324428</v>
       </c>
       <c r="F77" s="18" t="n">
-        <v>888.823951554494</v>
+        <v>-209.6616710419028</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>902.5958009168517</v>
+        <v>-193.9013568647862</v>
       </c>
       <c r="H77" s="18" t="n">
-        <v>931.2323369911371</v>
+        <v>-166.9988372288569</v>
       </c>
       <c r="I77" s="18" t="n">
-        <v>959.5582330874744</v>
+        <v>-138.583878118821</v>
       </c>
       <c r="J77" s="18" t="n">
-        <v>946.7883659423813</v>
+        <v>-151.2406658118593</v>
       </c>
       <c r="K77" s="18" t="n">
-        <v>946.7906763397162</v>
+        <v>-151.6276896610998</v>
       </c>
       <c r="L77" s="18" t="n">
-        <v>989.668689997648</v>
+        <v>-108.0707718935789</v>
       </c>
       <c r="M77" s="18" t="n">
-        <v>1032.188674780425</v>
+        <v>-65.39705560395237</v>
       </c>
       <c r="N77" s="18" t="n">
-        <v>1073.369070546184</v>
+        <v>-24.04768999445366</v>
       </c>
       <c r="O77" s="18" t="n">
-        <v>1092.721267370679</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" ht="15.5" customHeight="1">
@@ -10703,40 +10703,40 @@
         </is>
       </c>
       <c r="D78" s="18" t="n">
-        <v>929.4422221198872</v>
+        <v>898.1576416299777</v>
       </c>
       <c r="E78" s="18" t="n">
-        <v>1787.887758963044</v>
+        <v>667.6847368970334</v>
       </c>
       <c r="F78" s="18" t="n">
-        <v>2676.711710517538</v>
+        <v>459.2546068518321</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>3579.30751143439</v>
+        <v>266.8122517881062</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>4510.539848425527</v>
+        <v>101.2419077099342</v>
       </c>
       <c r="I78" s="18" t="n">
-        <v>5470.098081513001</v>
+        <v>-35.94306629929775</v>
       </c>
       <c r="J78" s="18" t="n">
-        <v>6416.886447455382</v>
+        <v>-185.8135951248557</v>
       </c>
       <c r="K78" s="18" t="n">
-        <v>7363.677123795098</v>
+        <v>-336.1007368407501</v>
       </c>
       <c r="L78" s="18" t="n">
-        <v>8353.345813792746</v>
+        <v>-443.4087690083016</v>
       </c>
       <c r="M78" s="18" t="n">
-        <v>9385.534488573172</v>
+        <v>272.0463526681717</v>
       </c>
       <c r="N78" s="18" t="n">
-        <v>10458.90355911936</v>
+        <v>1028.840976940446</v>
       </c>
       <c r="O78" s="18" t="n">
-        <v>11551.62482649004</v>
+        <v>1832.384348760694</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -11233,40 +11233,40 @@
         </is>
       </c>
       <c r="D88" s="18" t="n">
-        <v>-8.575484599498539</v>
+        <v>0</v>
       </c>
       <c r="E88" s="18" t="n">
-        <v>-9.807025596199978</v>
+        <v>0</v>
       </c>
       <c r="F88" s="18" t="n">
-        <v>-11.26602739726027</v>
+        <v>0</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>-12.69452054794521</v>
+        <v>0</v>
       </c>
       <c r="H88" s="18" t="n">
-        <v>-14.09342465753425</v>
+        <v>0</v>
       </c>
       <c r="I88" s="18" t="n">
-        <v>-15.46356164383562</v>
+        <v>0</v>
       </c>
       <c r="J88" s="18" t="n">
-        <v>-16.8041095890411</v>
+        <v>0</v>
       </c>
       <c r="K88" s="18" t="n">
-        <v>-17.5668493150685</v>
+        <v>0</v>
       </c>
       <c r="L88" s="18" t="n">
-        <v>-17.90383561643835</v>
+        <v>0</v>
       </c>
       <c r="M88" s="18" t="n">
-        <v>-18.23095890410959</v>
+        <v>0</v>
       </c>
       <c r="N88" s="18" t="n">
-        <v>-18.55004385489041</v>
+        <v>0</v>
       </c>
       <c r="O88" s="18" t="n">
-        <v>-18.86054794520548</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" ht="15.5" customHeight="1">
@@ -11339,40 +11339,40 @@
         </is>
       </c>
       <c r="D90" s="18" t="n">
-        <v>-17.15096919899708</v>
+        <v>14.13361129091242</v>
       </c>
       <c r="E90" s="18" t="n">
-        <v>-19.61405119239996</v>
+        <v>16.44318810243016</v>
       </c>
       <c r="F90" s="18" t="n">
-        <v>-22.53205479452054</v>
+        <v>19.2895397260274</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>-25.38904109589041</v>
+        <v>20.20844383561644</v>
       </c>
       <c r="H90" s="18" t="n">
-        <v>-28.1868493150685</v>
+        <v>22.92054246575343</v>
       </c>
       <c r="I90" s="18" t="n">
-        <v>-30.92712328767123</v>
+        <v>25.60111232876712</v>
       </c>
       <c r="J90" s="18" t="n">
-        <v>-33.60821917808219</v>
+        <v>28.2277808219178</v>
       </c>
       <c r="K90" s="18" t="n">
-        <v>-35.13369863013699</v>
+        <v>32.3994</v>
       </c>
       <c r="L90" s="18" t="n">
-        <v>-35.80767123287671</v>
+        <v>36.74362191780823</v>
       </c>
       <c r="M90" s="18" t="n">
-        <v>-36.46191780821918</v>
+        <v>40.95383835616438</v>
       </c>
       <c r="N90" s="18" t="n">
-        <v>-37.10008770978082</v>
+        <v>45.01116162456164</v>
       </c>
       <c r="O90" s="18" t="n">
-        <v>-37.72109589041096</v>
+        <v>51.61320000000001</v>
       </c>
     </row>
     <row r="91" ht="15.5" customHeight="1">
@@ -11392,40 +11392,40 @@
         </is>
       </c>
       <c r="D91" s="18" t="n">
-        <v>-17.15096919899708</v>
+        <v>14.13361129091242</v>
       </c>
       <c r="E91" s="18" t="n">
-        <v>-2.463081993402877</v>
+        <v>2.309576811517742</v>
       </c>
       <c r="F91" s="18" t="n">
-        <v>-2.918003602120589</v>
+        <v>2.84635162359724</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>-2.856986301369869</v>
+        <v>0.9189041095890396</v>
       </c>
       <c r="H91" s="18" t="n">
-        <v>-2.797808219178084</v>
+        <v>2.712098630136989</v>
       </c>
       <c r="I91" s="18" t="n">
-        <v>-2.740273972602736</v>
+        <v>2.680569863013694</v>
       </c>
       <c r="J91" s="18" t="n">
-        <v>-2.681095890410962</v>
+        <v>2.626668493150682</v>
       </c>
       <c r="K91" s="18" t="n">
-        <v>-1.525479452054796</v>
+        <v>4.171619178082196</v>
       </c>
       <c r="L91" s="18" t="n">
-        <v>-0.6739726027397168</v>
+        <v>4.344221917808227</v>
       </c>
       <c r="M91" s="18" t="n">
-        <v>-0.6542465753424693</v>
+        <v>4.210216438356156</v>
       </c>
       <c r="N91" s="18" t="n">
-        <v>-0.6381699015616462</v>
+        <v>4.057323268397262</v>
       </c>
       <c r="O91" s="18" t="n">
-        <v>-0.6210081806301346</v>
+        <v>6.602038375438362</v>
       </c>
     </row>
     <row r="92" ht="15.5" customHeight="1">
@@ -11687,34 +11687,34 @@
         <v>497.7465079617789</v>
       </c>
       <c r="F96" s="20" t="n">
-        <v>1026.61340208259</v>
+        <v>714.4073256909676</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>1569.496596417865</v>
+        <v>945.0844436346197</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>2110.458288607721</v>
+        <v>1173.840059432852</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>2664.525053682864</v>
+        <v>1415.700748116373</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>3231.534388710174</v>
+        <v>1670.504006752061</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>3821.307171433737</v>
+        <v>1948.070713084002</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>4446.317167141307</v>
+        <v>2260.874632399949</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>4984.409442622896</v>
+        <v>2486.760831489915</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>5470.675389968297</v>
+        <v>2738.92813284791</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>6074.553203639211</v>
+        <v>3016.193847786481</v>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
@@ -11873,7 +11873,7 @@
         <v>0</v>
       </c>
       <c r="O99" s="20" t="n">
-        <v>169.7671318367248</v>
+        <v>162.5440852806563</v>
       </c>
     </row>
     <row r="100" ht="15.5" customHeight="1">
@@ -11896,37 +11896,37 @@
         <v>497.7465079617789</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>1026.61340208259</v>
+        <v>714.4073256909676</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>1569.496596417865</v>
+        <v>945.0844436346197</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>2110.458288607721</v>
+        <v>1173.840059432852</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>2664.525053682864</v>
+        <v>1415.700748116373</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>3231.534388710174</v>
+        <v>1670.504006752061</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>3821.307171433737</v>
+        <v>1948.070713084002</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>4446.317167141307</v>
+        <v>2260.874632399949</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>4984.409442622896</v>
+        <v>2486.760831489915</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>5470.675389968297</v>
+        <v>2738.92813284791</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>6074.553203639211</v>
+        <v>3016.193847786481</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>6784.976237226653</v>
+        <v>3504.876117151001</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -12079,13 +12079,13 @@
         <v>5463.606336853395</v>
       </c>
       <c r="M103" s="18" t="n">
-        <v>6322.228958236666</v>
+        <v>6244.121527832452</v>
       </c>
       <c r="N103" s="18" t="n">
-        <v>7088.338126875001</v>
+        <v>7024.636718811508</v>
       </c>
       <c r="O103" s="18" t="n">
-        <v>7966.541676578826</v>
+        <v>7805.151909790565</v>
       </c>
     </row>
     <row r="104" ht="15.5" customHeight="1">
@@ -12288,16 +12288,16 @@
         <v>5463.606336853395</v>
       </c>
       <c r="L107" s="18" t="n">
-        <v>6322.228958236666</v>
+        <v>6244.121527832452</v>
       </c>
       <c r="M107" s="18" t="n">
-        <v>7088.338126875001</v>
+        <v>7024.636718811508</v>
       </c>
       <c r="N107" s="18" t="n">
-        <v>7966.541676578826</v>
+        <v>7805.151909790565</v>
       </c>
       <c r="O107" s="18" t="n">
-        <v>8731.818232389202</v>
+        <v>8585.66710076962</v>
       </c>
     </row>
     <row r="108" ht="15.5" customHeight="1">
@@ -14879,40 +14879,40 @@
         </is>
       </c>
       <c r="D43" s="18" t="n">
-        <v>551.0935917130184</v>
+        <v>549.108252377128</v>
       </c>
       <c r="E43" s="18" t="n">
-        <v>1087.876586707202</v>
+        <v>507.4961708575325</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>1609.562433646628</v>
+        <v>450.8415224890389</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>2115.646030219804</v>
+        <v>377.9778969038145</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>2606.453216564675</v>
+        <v>289.9035059336485</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>3081.73132727686</v>
+        <v>186.2232430411611</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>3542.921076999049</v>
+        <v>68.53091171767765</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>3998.2412586508</v>
+        <v>-56.21582396717889</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>4450.873747371277</v>
+        <v>-183.7077992454284</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>4900.52628005493</v>
+        <v>-312.5571971662302</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>5347.682161949155</v>
+        <v>-443.8833813511223</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>5791.955059107859</v>
+        <v>-576.0532517713705</v>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
@@ -14932,40 +14932,40 @@
         </is>
       </c>
       <c r="D44" s="18" t="n">
-        <v>549.2144358801597</v>
+        <v>547.1229130412376</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>1086.570396891729</v>
+        <v>505.3485922054778</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>1608.016251180524</v>
+        <v>447.9572638961622</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>2113.118509930268</v>
+        <v>373.9887495629926</v>
       </c>
       <c r="H44" s="18" t="n">
-        <v>2603.817067525088</v>
+        <v>285.2482510539224</v>
       </c>
       <c r="I44" s="18" t="n">
-        <v>3077.960321056903</v>
+        <v>180.3911564685583</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>3539.194099390256</v>
+        <v>62.11379028754067</v>
       </c>
       <c r="K44" s="18" t="n">
-        <v>3990.181697400639</v>
+        <v>-64.98990550197341</v>
       </c>
       <c r="L44" s="18" t="n">
-        <v>4443.412396160323</v>
+        <v>-192.2917005415928</v>
       </c>
       <c r="M44" s="18" t="n">
-        <v>4892.140238946876</v>
+        <v>-321.7120381667781</v>
       </c>
       <c r="N44" s="18" t="n">
-        <v>5339.934070748825</v>
+        <v>-452.8275175374237</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>5783.390207006471</v>
+        <v>-585.5137192653431</v>
       </c>
     </row>
     <row r="45" ht="15.5" customHeight="1">
@@ -15038,40 +15038,40 @@
         </is>
       </c>
       <c r="D46" s="18" t="n">
-        <v>-0.1061835030317407</v>
+        <v>0</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>-0.8413888365812087</v>
+        <v>0</v>
       </c>
       <c r="F46" s="18" t="n">
-        <v>-1.338076126772904</v>
+        <v>0</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>-1.461627051286592</v>
+        <v>0</v>
       </c>
       <c r="H46" s="18" t="n">
-        <v>-2.019105840138757</v>
+        <v>0</v>
       </c>
       <c r="I46" s="18" t="n">
-        <v>-2.06108035264661</v>
+        <v>0</v>
       </c>
       <c r="J46" s="18" t="n">
-        <v>-2.690143821343988</v>
+        <v>0</v>
       </c>
       <c r="K46" s="18" t="n">
-        <v>-0.7145202846336909</v>
+        <v>0</v>
       </c>
       <c r="L46" s="18" t="n">
-        <v>-1.122550085209791</v>
+        <v>0</v>
       </c>
       <c r="M46" s="18" t="n">
-        <v>-0.768799892493468</v>
+        <v>0</v>
       </c>
       <c r="N46" s="18" t="n">
-        <v>-1.196044985970805</v>
+        <v>0</v>
       </c>
       <c r="O46" s="18" t="n">
-        <v>-0.8956153925843086</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" ht="15.5" customHeight="1">
@@ -15091,40 +15091,40 @@
         </is>
       </c>
       <c r="D47" s="18" t="n">
-        <v>553.5971114017721</v>
+        <v>551.6117720658816</v>
       </c>
       <c r="E47" s="18" t="n">
-        <v>1094.663788754521</v>
+        <v>514.2833729048513</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>1620.29492632996</v>
+        <v>461.5740151723709</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>2129.987021183798</v>
+        <v>392.3188878678087</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>2624.067496827509</v>
+        <v>307.5177861964827</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>3102.285255396505</v>
+        <v>206.7771711608067</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>3565.127242920529</v>
+        <v>90.73707763915748</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>4020.888526120569</v>
+        <v>-33.56855649741013</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>4473.777688970748</v>
+        <v>-160.8038576459569</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>4923.503274277111</v>
+        <v>-289.5802029440493</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>5370.549385139529</v>
+        <v>-421.0161581607487</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>5814.485425095862</v>
+        <v>-553.522885783367</v>
       </c>
     </row>
     <row r="48" ht="15.5" customHeight="1">
@@ -15727,40 +15727,40 @@
         </is>
       </c>
       <c r="D59" s="18" t="n">
-        <v>1.985339335890444</v>
+        <v>0</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>580.4865993527017</v>
+        <v>0.1061835030317297</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>1159.562299994171</v>
+        <v>0.8413888365813023</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>1739.006209442762</v>
+        <v>1.338076126772933</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>2318.011337682313</v>
+        <v>1.461627051286712</v>
       </c>
       <c r="I59" s="18" t="n">
-        <v>2897.527190075838</v>
+        <v>2.019105840138906</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>3476.451245634018</v>
+        <v>2.061080352646712</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>4057.147226439323</v>
+        <v>2.690143821344094</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>4635.296066901339</v>
+        <v>0.7145202846337213</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>5214.20602730637</v>
+        <v>1.122550085209923</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>5792.334343192771</v>
+        <v>0.7687998924935755</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>6371.18969520109</v>
+        <v>3.181384321861174</v>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
@@ -15939,40 +15939,40 @@
         </is>
       </c>
       <c r="D63" s="18" t="n">
-        <v>0.2123670060634813</v>
+        <v>-1.87915583285867</v>
       </c>
       <c r="E63" s="18" t="n">
-        <v>1.470410667098936</v>
+        <v>0.5729660173850841</v>
       </c>
       <c r="F63" s="18" t="n">
-        <v>0.9933745803833898</v>
+        <v>-0.2399926506302228</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>0.2471018490273762</v>
+        <v>-0.9813378234315173</v>
       </c>
       <c r="H63" s="18" t="n">
-        <v>1.114957577704331</v>
+        <v>-0.1086287500519441</v>
       </c>
       <c r="I63" s="18" t="n">
-        <v>0.08394902501570645</v>
+        <v>-1.134857180368858</v>
       </c>
       <c r="J63" s="18" t="n">
-        <v>1.258126937394756</v>
+        <v>0.04402861116313073</v>
       </c>
       <c r="K63" s="18" t="n">
-        <v>-3.951247073420595</v>
+        <v>-4.332583641367831</v>
       </c>
       <c r="L63" s="18" t="n">
-        <v>0.8160596011522001</v>
+        <v>0.5982100392062355</v>
       </c>
       <c r="M63" s="18" t="n">
-        <v>-0.7075003854326458</v>
+        <v>-0.924689897099884</v>
       </c>
       <c r="N63" s="18" t="n">
-        <v>0.8544901869546733</v>
+        <v>0.637949907723911</v>
       </c>
       <c r="O63" s="18" t="n">
-        <v>-0.6008591867729922</v>
+        <v>-0.8167609010577284</v>
       </c>
     </row>
     <row r="64" ht="15.5" customHeight="1">
@@ -15992,40 +15992,40 @@
         </is>
       </c>
       <c r="D64" s="18" t="n">
-        <v>-26.4422422968227</v>
+        <v>-28.53376513574485</v>
       </c>
       <c r="E64" s="18" t="n">
-        <v>-36.2018041246391</v>
+        <v>-37.09924877435296</v>
       </c>
       <c r="F64" s="18" t="n">
-        <v>-52.13295515268695</v>
+        <v>-53.36632238370056</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>-68.49738455395949</v>
+        <v>-69.72582422641838</v>
       </c>
       <c r="H64" s="18" t="n">
-        <v>-82.92171123248389</v>
+        <v>-84.14529756024017</v>
       </c>
       <c r="I64" s="18" t="n">
-        <v>-99.49743456385137</v>
+        <v>-100.7162407692359</v>
       </c>
       <c r="J64" s="18" t="n">
-        <v>-113.4506824922904</v>
+        <v>-114.6647808185221</v>
       </c>
       <c r="K64" s="18" t="n">
-        <v>-124.7334688101305</v>
+        <v>-125.1148053780777</v>
       </c>
       <c r="L64" s="18" t="n">
-        <v>-122.5009721607336</v>
+        <v>-122.7188217226796</v>
       </c>
       <c r="M64" s="18" t="n">
-        <v>-127.0143261927698</v>
+        <v>-127.2315157044371</v>
       </c>
       <c r="N64" s="18" t="n">
-        <v>-127.9587302556901</v>
+        <v>-128.1752705349209</v>
       </c>
       <c r="O64" s="18" t="n">
-        <v>-132.3549853653821</v>
+        <v>-132.5708870796668</v>
       </c>
     </row>
     <row r="65" ht="15.5" customHeight="1">
@@ -16151,40 +16151,40 @@
         </is>
       </c>
       <c r="D67" s="18" t="n">
-        <v>-29.12458482048723</v>
+        <v>-31.21610765940938</v>
       </c>
       <c r="E67" s="18" t="n">
-        <v>-40.98305968907779</v>
+        <v>-41.88050433879165</v>
       </c>
       <c r="F67" s="18" t="n">
-        <v>-56.89316641185139</v>
+        <v>-58.126533642865</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>-73.23676195090243</v>
+        <v>-74.46520162336132</v>
       </c>
       <c r="H67" s="18" t="n">
-        <v>-87.64046310582754</v>
+        <v>-88.86404943358382</v>
       </c>
       <c r="I67" s="18" t="n">
-        <v>-104.1957671688317</v>
+        <v>-105.4145733742163</v>
       </c>
       <c r="J67" s="18" t="n">
-        <v>-117.1052423672938</v>
+        <v>-118.3193406935254</v>
       </c>
       <c r="K67" s="18" t="n">
-        <v>-127.3514226902642</v>
+        <v>-127.7327592582115</v>
       </c>
       <c r="L67" s="18" t="n">
-        <v>-125.1083219409631</v>
+        <v>-125.3261715029091</v>
       </c>
       <c r="M67" s="18" t="n">
-        <v>-129.6111779140942</v>
+        <v>-129.8283674257615</v>
       </c>
       <c r="N67" s="18" t="n">
-        <v>-130.5451888986984</v>
+        <v>-130.7617291779292</v>
       </c>
       <c r="O67" s="18" t="n">
-        <v>-134.8828844430022</v>
+        <v>-135.098786157287</v>
       </c>
     </row>
     <row r="68" ht="15.5" customHeight="1">
@@ -16525,37 +16525,37 @@
         <v>578.339020700647</v>
       </c>
       <c r="E74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="F74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="H74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="I74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="J74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="K74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="L74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="M74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="N74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
       <c r="O74" s="18" t="n">
-        <v>578.339020700647</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" ht="15.5" customHeight="1">
@@ -16575,40 +16575,40 @@
         </is>
       </c>
       <c r="D75" s="18" t="n">
-        <v>549.2144358801597</v>
+        <v>547.1229130412376</v>
       </c>
       <c r="E75" s="18" t="n">
-        <v>537.3559610115692</v>
+        <v>-41.88050433879165</v>
       </c>
       <c r="F75" s="18" t="n">
-        <v>521.4458542887955</v>
+        <v>-58.126533642865</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>505.1022587497446</v>
+        <v>-74.46520162336132</v>
       </c>
       <c r="H75" s="18" t="n">
-        <v>490.6985575948195</v>
+        <v>-88.86404943358382</v>
       </c>
       <c r="I75" s="18" t="n">
-        <v>474.1432535318153</v>
+        <v>-105.4145733742163</v>
       </c>
       <c r="J75" s="18" t="n">
-        <v>461.2337783333531</v>
+        <v>-118.3193406935254</v>
       </c>
       <c r="K75" s="18" t="n">
-        <v>450.9875980103828</v>
+        <v>-127.7327592582115</v>
       </c>
       <c r="L75" s="18" t="n">
-        <v>453.2306987596838</v>
+        <v>-125.3261715029091</v>
       </c>
       <c r="M75" s="18" t="n">
-        <v>448.7278427865527</v>
+        <v>-129.8283674257615</v>
       </c>
       <c r="N75" s="18" t="n">
-        <v>447.7938318019486</v>
+        <v>-130.7617291779292</v>
       </c>
       <c r="O75" s="18" t="n">
-        <v>443.4561362576447</v>
+        <v>-135.098786157287</v>
       </c>
     </row>
     <row r="76" ht="15.5" customHeight="1">
@@ -16631,37 +16631,37 @@
         <v>0</v>
       </c>
       <c r="E76" s="18" t="n">
-        <v>549.2144358801597</v>
+        <v>547.1229130412376</v>
       </c>
       <c r="F76" s="18" t="n">
-        <v>1086.570396891729</v>
+        <v>505.3485922054778</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>1608.016251180524</v>
+        <v>447.9572638961622</v>
       </c>
       <c r="H76" s="18" t="n">
-        <v>2113.118509930268</v>
+        <v>373.9887495629926</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>2603.817067525088</v>
+        <v>285.2482510539224</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>3077.960321056903</v>
+        <v>180.3911564685583</v>
       </c>
       <c r="K76" s="18" t="n">
-        <v>3539.194099390256</v>
+        <v>62.11379028754067</v>
       </c>
       <c r="L76" s="18" t="n">
-        <v>3990.181697400639</v>
+        <v>-64.98990550197341</v>
       </c>
       <c r="M76" s="18" t="n">
-        <v>4443.412396160323</v>
+        <v>-192.2917005415928</v>
       </c>
       <c r="N76" s="18" t="n">
-        <v>4892.140238946876</v>
+        <v>-321.7120381667781</v>
       </c>
       <c r="O76" s="18" t="n">
-        <v>5339.934070748825</v>
+        <v>-452.8275175374237</v>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
@@ -16681,40 +16681,40 @@
         </is>
       </c>
       <c r="D77" s="18" t="n">
-        <v>549.2144358801597</v>
+        <v>547.1229130412376</v>
       </c>
       <c r="E77" s="18" t="n">
-        <v>537.3559610115692</v>
+        <v>-41.88050433879165</v>
       </c>
       <c r="F77" s="18" t="n">
-        <v>521.4458542887955</v>
+        <v>-58.126533642865</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>505.1022587497446</v>
+        <v>-74.46520162336132</v>
       </c>
       <c r="H77" s="18" t="n">
-        <v>490.6985575948195</v>
+        <v>-88.86404943358382</v>
       </c>
       <c r="I77" s="18" t="n">
-        <v>474.1432535318153</v>
+        <v>-105.4145733742163</v>
       </c>
       <c r="J77" s="18" t="n">
-        <v>461.2337783333531</v>
+        <v>-118.3193406935254</v>
       </c>
       <c r="K77" s="18" t="n">
-        <v>450.9875980103828</v>
+        <v>-127.7327592582115</v>
       </c>
       <c r="L77" s="18" t="n">
-        <v>453.2306987596838</v>
+        <v>-125.3261715029091</v>
       </c>
       <c r="M77" s="18" t="n">
-        <v>448.7278427865527</v>
+        <v>-129.8283674257615</v>
       </c>
       <c r="N77" s="18" t="n">
-        <v>447.7938318019486</v>
+        <v>-130.7617291779292</v>
       </c>
       <c r="O77" s="18" t="n">
-        <v>443.4561362576447</v>
+        <v>-135.098786157287</v>
       </c>
     </row>
     <row r="78" ht="15.5" customHeight="1">
@@ -16734,40 +16734,40 @@
         </is>
       </c>
       <c r="D78" s="18" t="n">
-        <v>549.2144358801597</v>
+        <v>547.1229130412376</v>
       </c>
       <c r="E78" s="18" t="n">
-        <v>1086.570396891729</v>
+        <v>505.3485922054778</v>
       </c>
       <c r="F78" s="18" t="n">
-        <v>1608.016251180524</v>
+        <v>447.9572638961622</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>2113.118509930268</v>
+        <v>373.9887495629926</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>2603.817067525088</v>
+        <v>285.2482510539224</v>
       </c>
       <c r="I78" s="18" t="n">
-        <v>3077.960321056903</v>
+        <v>180.3911564685583</v>
       </c>
       <c r="J78" s="18" t="n">
-        <v>3539.194099390256</v>
+        <v>62.11379028754067</v>
       </c>
       <c r="K78" s="18" t="n">
-        <v>3990.181697400639</v>
+        <v>-64.98990550197341</v>
       </c>
       <c r="L78" s="18" t="n">
-        <v>4443.412396160323</v>
+        <v>-192.2917005415928</v>
       </c>
       <c r="M78" s="18" t="n">
-        <v>4892.140238946876</v>
+        <v>-321.7120381667781</v>
       </c>
       <c r="N78" s="18" t="n">
-        <v>5339.934070748825</v>
+        <v>-452.8275175374237</v>
       </c>
       <c r="O78" s="18" t="n">
-        <v>5783.390207006471</v>
+        <v>-585.5137192653431</v>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
@@ -17264,40 +17264,40 @@
         </is>
       </c>
       <c r="D88" s="18" t="n">
-        <v>-0.1061835030317407</v>
+        <v>0</v>
       </c>
       <c r="E88" s="18" t="n">
-        <v>-0.8413888365812087</v>
+        <v>0</v>
       </c>
       <c r="F88" s="18" t="n">
-        <v>-1.338076126772904</v>
+        <v>0</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>-1.461627051286592</v>
+        <v>0</v>
       </c>
       <c r="H88" s="18" t="n">
-        <v>-2.019105840138757</v>
+        <v>0</v>
       </c>
       <c r="I88" s="18" t="n">
-        <v>-2.06108035264661</v>
+        <v>0</v>
       </c>
       <c r="J88" s="18" t="n">
-        <v>-2.690143821343988</v>
+        <v>0</v>
       </c>
       <c r="K88" s="18" t="n">
-        <v>-0.7145202846336909</v>
+        <v>0</v>
       </c>
       <c r="L88" s="18" t="n">
-        <v>-1.122550085209791</v>
+        <v>0</v>
       </c>
       <c r="M88" s="18" t="n">
-        <v>-0.768799892493468</v>
+        <v>0</v>
       </c>
       <c r="N88" s="18" t="n">
-        <v>-1.196044985970805</v>
+        <v>0</v>
       </c>
       <c r="O88" s="18" t="n">
-        <v>-0.8956153925843086</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" ht="15.5" customHeight="1">
@@ -17370,40 +17370,40 @@
         </is>
       </c>
       <c r="D90" s="18" t="n">
-        <v>-0.2123670060634813</v>
+        <v>1.87915583285867</v>
       </c>
       <c r="E90" s="18" t="n">
-        <v>-1.682777673162417</v>
+        <v>1.306189815473586</v>
       </c>
       <c r="F90" s="18" t="n">
-        <v>-2.676152253545807</v>
+        <v>1.546182466103809</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>-2.923254102573183</v>
+        <v>2.527520289535326</v>
       </c>
       <c r="H90" s="18" t="n">
-        <v>-4.038211680277514</v>
+        <v>2.63614903958727</v>
       </c>
       <c r="I90" s="18" t="n">
-        <v>-4.12216070529322</v>
+        <v>3.771006219956129</v>
       </c>
       <c r="J90" s="18" t="n">
-        <v>-5.380287642687977</v>
+        <v>3.726977608792998</v>
       </c>
       <c r="K90" s="18" t="n">
-        <v>-1.429040569267382</v>
+        <v>8.059561250160829</v>
       </c>
       <c r="L90" s="18" t="n">
-        <v>-2.245100170419582</v>
+        <v>7.461351210954594</v>
       </c>
       <c r="M90" s="18" t="n">
-        <v>-1.537599784986936</v>
+        <v>8.386041108054478</v>
       </c>
       <c r="N90" s="18" t="n">
-        <v>-2.392089971941609</v>
+        <v>7.748091200330567</v>
       </c>
       <c r="O90" s="18" t="n">
-        <v>-1.791230785168617</v>
+        <v>8.564852101388295</v>
       </c>
     </row>
     <row r="91" ht="15.5" customHeight="1">
@@ -17423,40 +17423,40 @@
         </is>
       </c>
       <c r="D91" s="18" t="n">
-        <v>-0.2123670060634813</v>
+        <v>1.87915583285867</v>
       </c>
       <c r="E91" s="18" t="n">
-        <v>-1.470410667098936</v>
+        <v>-0.5729660173850841</v>
       </c>
       <c r="F91" s="18" t="n">
-        <v>-0.9933745803833898</v>
+        <v>0.2399926506302228</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>-0.2471018490273762</v>
+        <v>0.9813378234315173</v>
       </c>
       <c r="H91" s="18" t="n">
-        <v>-1.114957577704331</v>
+        <v>0.1086287500519441</v>
       </c>
       <c r="I91" s="18" t="n">
-        <v>-0.08394902501570645</v>
+        <v>1.134857180368858</v>
       </c>
       <c r="J91" s="18" t="n">
-        <v>-1.258126937394756</v>
+        <v>-0.04402861116313073</v>
       </c>
       <c r="K91" s="18" t="n">
-        <v>3.951247073420595</v>
+        <v>4.332583641367831</v>
       </c>
       <c r="L91" s="18" t="n">
-        <v>-0.8160596011522001</v>
+        <v>-0.5982100392062355</v>
       </c>
       <c r="M91" s="18" t="n">
-        <v>0.7075003854326458</v>
+        <v>0.924689897099884</v>
       </c>
       <c r="N91" s="18" t="n">
-        <v>-0.8544901869546733</v>
+        <v>-0.637949907723911</v>
       </c>
       <c r="O91" s="18" t="n">
-        <v>0.6008591867729922</v>
+        <v>0.8167609010577284</v>
       </c>
     </row>
     <row r="92" ht="15.5" customHeight="1">
@@ -17718,34 +17718,34 @@
         <v>551.5055885628499</v>
       </c>
       <c r="F96" s="20" t="n">
-        <v>1091.674821265885</v>
+        <v>513.3358005652383</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>1616.07259161031</v>
+        <v>459.3945502090168</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>2124.536246791689</v>
+        <v>389.5191846897492</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>2617.393136107644</v>
+        <v>304.0370533050573</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>3094.392088471255</v>
+        <v>202.6969849680213</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>3556.019977669048</v>
+        <v>85.9858534651669</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>4011.39992430114</v>
+        <v>-36.97322060338779</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>4464.071237589375</v>
+        <v>-162.6409280158003</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>4913.57963338407</v>
+        <v>-291.4715529217525</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>5360.409203967256</v>
+        <v>-422.9810030392129</v>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
@@ -17927,37 +17927,37 @@
         <v>551.5055885628499</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>1091.674821265885</v>
+        <v>513.3358005652383</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>1616.07259161031</v>
+        <v>459.3945502090168</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>2124.536246791689</v>
+        <v>389.5191846897492</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>2617.393136107644</v>
+        <v>304.0370533050573</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>3094.392088471255</v>
+        <v>202.6969849680213</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>3556.019977669048</v>
+        <v>85.9858534651669</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>4011.39992430114</v>
+        <v>-36.97322060338779</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>4464.071237589375</v>
+        <v>-162.6409280158003</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>4913.57963338407</v>
+        <v>-291.4715529217525</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>5360.409203967256</v>
+        <v>-422.9810030392129</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>5804.129342209303</v>
+        <v>-557.5998854978122</v>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
@@ -20910,40 +20910,40 @@
         </is>
       </c>
       <c r="D43" s="18" t="n">
-        <v>728.0947567237049</v>
+        <v>705.7675525923769</v>
       </c>
       <c r="E43" s="18" t="n">
-        <v>1399.196074945698</v>
+        <v>545.5142829331834</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>2091.949795213938</v>
+        <v>398.7196402316764</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>2789.42521648785</v>
+        <v>258.6136627131216</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>3508.224605856394</v>
+        <v>138.2286149043626</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>4246.334299716566</v>
+        <v>37.19319058275833</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>4995.471160314218</v>
+        <v>-52.76153761687472</v>
       </c>
       <c r="K43" s="18" t="n">
-        <v>5759.615904440761</v>
+        <v>-127.8016784792381</v>
       </c>
       <c r="L43" s="18" t="n">
-        <v>6548.333656506655</v>
+        <v>-178.6261573555255</v>
       </c>
       <c r="M43" s="18" t="n">
-        <v>7360.968960392492</v>
+        <v>370.0440587087102</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>8196.587383104083</v>
+        <v>941.801569128346</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>9038.073332223403</v>
+        <v>1544.514707993967</v>
       </c>
     </row>
     <row r="44">
@@ -20963,40 +20963,40 @@
         </is>
       </c>
       <c r="D44" s="18" t="n">
-        <v>714.1772432207383</v>
+        <v>683.440348461049</v>
       </c>
       <c r="E44" s="18" t="n">
-        <v>1383.788264468883</v>
+        <v>520.8478822036918</v>
       </c>
       <c r="F44" s="18" t="n">
-        <v>2074.648348110827</v>
+        <v>371.0810588195063</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>2771.944607851709</v>
+        <v>229.7402203634867</v>
       </c>
       <c r="H44" s="18" t="n">
-        <v>3488.962601677472</v>
+        <v>106.5401178843739</v>
       </c>
       <c r="I44" s="18" t="n">
-        <v>4225.330927212288</v>
+        <v>2.750998164803988</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>4972.779014774398</v>
+        <v>-89.88256399333916</v>
       </c>
       <c r="K44" s="18" t="n">
-        <v>5734.750702790961</v>
+        <v>-167.6725688561934</v>
       </c>
       <c r="L44" s="18" t="n">
-        <v>6521.092798369359</v>
+        <v>-221.191004653787</v>
       </c>
       <c r="M44" s="18" t="n">
-        <v>7331.449119350613</v>
+        <v>324.8911612523441</v>
       </c>
       <c r="N44" s="18" t="n">
-        <v>8164.894548635995</v>
+        <v>894.1740302238113</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>9002.319630547379</v>
+        <v>1492.532626191176</v>
       </c>
     </row>
     <row r="45">
@@ -21069,40 +21069,40 @@
         </is>
       </c>
       <c r="D46" s="18" t="n">
-        <v>-8.409690628361332</v>
+        <v>0</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>-9.258590252676456</v>
+        <v>0</v>
       </c>
       <c r="F46" s="18" t="n">
-        <v>-10.3371343090589</v>
+        <v>0</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>-11.39283371349388</v>
+        <v>0</v>
       </c>
       <c r="H46" s="18" t="n">
-        <v>-12.4264928410668</v>
+        <v>0</v>
       </c>
       <c r="I46" s="18" t="n">
-        <v>-13.43881991367581</v>
+        <v>0</v>
       </c>
       <c r="J46" s="18" t="n">
-        <v>-14.42888083664442</v>
+        <v>0</v>
       </c>
       <c r="K46" s="18" t="n">
-        <v>-15.00568872715453</v>
+        <v>0</v>
       </c>
       <c r="L46" s="18" t="n">
-        <v>-15.32398916096545</v>
+        <v>0</v>
       </c>
       <c r="M46" s="18" t="n">
-        <v>-15.63305641448772</v>
+        <v>0</v>
       </c>
       <c r="N46" s="18" t="n">
-        <v>-15.9347044364481</v>
+        <v>0</v>
       </c>
       <c r="O46" s="18" t="n">
-        <v>-16.22838012676809</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -21122,40 +21122,40 @@
         </is>
       </c>
       <c r="D47" s="18" t="n">
-        <v>974.7420336825287</v>
+        <v>952.4148295512007</v>
       </c>
       <c r="E47" s="18" t="n">
-        <v>1927.413248922933</v>
+        <v>1073.731456910418</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>2889.746510594287</v>
+        <v>1196.516355612025</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>3844.926089212167</v>
+        <v>1314.114535437439</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>4809.677873706129</v>
+        <v>1439.681882754097</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>5782.10088209535</v>
+        <v>1572.959772961542</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>6761.923694698429</v>
+        <v>1713.690996767337</v>
       </c>
       <c r="K47" s="18" t="n">
-        <v>7753.280920796797</v>
+        <v>1865.863337876797</v>
       </c>
       <c r="L47" s="18" t="n">
-        <v>8758.059210318806</v>
+        <v>2031.099396456627</v>
       </c>
       <c r="M47" s="18" t="n">
-        <v>9775.716294590213</v>
+        <v>2784.791392906431</v>
       </c>
       <c r="N47" s="18" t="n">
-        <v>10805.42609178529</v>
+        <v>3550.640277809553</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>11754.51989297923</v>
+        <v>4260.96126874979</v>
       </c>
     </row>
     <row r="48">
@@ -21181,34 +21181,34 @@
         <v>618.4212010360498</v>
       </c>
       <c r="F48" s="18" t="n">
-        <v>922.1943080642168</v>
+        <v>813.0768042092967</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>1238.720452422614</v>
+        <v>1001.600482556675</v>
       </c>
       <c r="H48" s="18" t="n">
-        <v>1561.252267139688</v>
+        <v>1197.408440298696</v>
       </c>
       <c r="I48" s="18" t="n">
-        <v>1691.030698725584</v>
+        <v>1400.246613867372</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>2028.769907927984</v>
+        <v>1611.800160899984</v>
       </c>
       <c r="K48" s="18" t="n">
-        <v>2181.792245779586</v>
+        <v>1836.428768312999</v>
       </c>
       <c r="L48" s="18" t="n">
-        <v>2469.841199647154</v>
+        <v>2000.769718568508</v>
       </c>
       <c r="M48" s="18" t="n">
-        <v>2767.719251095017</v>
+        <v>2178.104603516902</v>
       </c>
       <c r="N48" s="18" t="n">
-        <v>2982.442168446919</v>
+        <v>2367.613029330465</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>3088.050784484931</v>
+        <v>2479.281748613017</v>
       </c>
     </row>
     <row r="49">
@@ -21314,7 +21314,7 @@
         <v>189.5084258135635</v>
       </c>
       <c r="O50" s="18" t="n">
-        <v>107.0205006939758</v>
+        <v>111.6687192825518</v>
       </c>
     </row>
     <row r="51">
@@ -21340,34 +21340,34 @@
         <v>170.1250745615756</v>
       </c>
       <c r="F51" s="18" t="n">
-        <v>465.8433667936624</v>
+        <v>356.7258629387424</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>788.5014359779282</v>
+        <v>551.3814661119893</v>
       </c>
       <c r="H51" s="18" t="n">
-        <v>1103.74897130036</v>
+        <v>739.9051444593674</v>
       </c>
       <c r="I51" s="18" t="n">
-        <v>1226.4971870596</v>
+        <v>935.7131022013884</v>
       </c>
       <c r="J51" s="18" t="n">
-        <v>1555.521022798065</v>
+        <v>1138.551275770065</v>
       </c>
       <c r="K51" s="18" t="n">
-        <v>1695.468300269264</v>
+        <v>1350.104822802677</v>
       </c>
       <c r="L51" s="18" t="n">
-        <v>2043.804911294337</v>
+        <v>1574.733430215691</v>
       </c>
       <c r="M51" s="18" t="n">
-        <v>2328.689028049315</v>
+        <v>1739.0743804712</v>
       </c>
       <c r="N51" s="18" t="n">
-        <v>2531.238404536048</v>
+        <v>1916.409265419594</v>
       </c>
       <c r="O51" s="18" t="n">
-        <v>2719.334945693648</v>
+        <v>2105.917691233158</v>
       </c>
     </row>
     <row r="52">
@@ -21387,40 +21387,40 @@
         </is>
       </c>
       <c r="D52" s="18" t="n">
-        <v>403.0672224090362</v>
+        <v>512.1847262639563</v>
       </c>
       <c r="E52" s="18" t="n">
-        <v>776.2517489414683</v>
+        <v>1013.371718807407</v>
       </c>
       <c r="F52" s="18" t="n">
-        <v>1151.459487628153</v>
+        <v>1515.303314469146</v>
       </c>
       <c r="G52" s="18" t="n">
-        <v>1727.18923144223</v>
+        <v>2017.973316300442</v>
       </c>
       <c r="H52" s="18" t="n">
-        <v>2104.403344129146</v>
+        <v>2521.373091157147</v>
       </c>
       <c r="I52" s="18" t="n">
-        <v>2680.133087943223</v>
+        <v>3025.49656540981</v>
       </c>
       <c r="J52" s="18" t="n">
-        <v>3059.330116922845</v>
+        <v>3528.401598001493</v>
       </c>
       <c r="K52" s="18" t="n">
-        <v>3440.49355912042</v>
+        <v>4030.108206698536</v>
       </c>
       <c r="L52" s="18" t="n">
-        <v>3991.008811396158</v>
+        <v>4605.837950512612</v>
       </c>
       <c r="M52" s="18" t="n">
-        <v>4568.150439866198</v>
+        <v>5181.567694326689</v>
       </c>
       <c r="N52" s="18" t="n">
-        <v>5145.280800422396</v>
+        <v>5757.297438140766</v>
       </c>
       <c r="O52" s="18" t="n">
-        <v>5722.395457827415</v>
+        <v>6333.027181954842</v>
       </c>
     </row>
     <row r="53">
@@ -21440,40 +21440,40 @@
         </is>
       </c>
       <c r="D53" s="18" t="n">
-        <v>403.0672224090362</v>
+        <v>512.1847262639563</v>
       </c>
       <c r="E53" s="18" t="n">
-        <v>776.2517489414683</v>
+        <v>1013.371718807407</v>
       </c>
       <c r="F53" s="18" t="n">
-        <v>1151.459487628153</v>
+        <v>1515.303314469146</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>1727.18923144223</v>
+        <v>2017.973316300442</v>
       </c>
       <c r="H53" s="18" t="n">
-        <v>2104.403344129146</v>
+        <v>2521.373091157147</v>
       </c>
       <c r="I53" s="18" t="n">
-        <v>2680.133087943223</v>
+        <v>3025.49656540981</v>
       </c>
       <c r="J53" s="18" t="n">
-        <v>3059.330116922845</v>
+        <v>3528.401598001493</v>
       </c>
       <c r="K53" s="18" t="n">
-        <v>3440.49355912042</v>
+        <v>4030.108206698536</v>
       </c>
       <c r="L53" s="18" t="n">
-        <v>3991.008811396158</v>
+        <v>4605.837950512612</v>
       </c>
       <c r="M53" s="18" t="n">
-        <v>4568.150439866198</v>
+        <v>5181.567694326689</v>
       </c>
       <c r="N53" s="18" t="n">
-        <v>5145.280800422396</v>
+        <v>5757.297438140766</v>
       </c>
       <c r="O53" s="18" t="n">
-        <v>5722.395457827415</v>
+        <v>6333.027181954842</v>
       </c>
     </row>
     <row r="54">
@@ -21705,40 +21705,40 @@
         </is>
       </c>
       <c r="D58" s="18" t="n">
-        <v>843.2973256962806</v>
+        <v>952.4148295512008</v>
       </c>
       <c r="E58" s="18" t="n">
-        <v>1403.931540230195</v>
+        <v>1641.051510096134</v>
       </c>
       <c r="F58" s="18" t="n">
-        <v>2083.990930001429</v>
+        <v>2338.717252987501</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>2977.302517578337</v>
+        <v>3030.96663257061</v>
       </c>
       <c r="H58" s="18" t="n">
-        <v>3678.082104109901</v>
+        <v>3731.20802429691</v>
       </c>
       <c r="I58" s="18" t="n">
-        <v>4384.602606582482</v>
+        <v>4439.181999190858</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>5102.528905687474</v>
+        <v>5154.630639738121</v>
       </c>
       <c r="K58" s="18" t="n">
-        <v>5637.291493627161</v>
+        <v>5881.54266373869</v>
       </c>
       <c r="L58" s="18" t="n">
-        <v>6476.174000204278</v>
+        <v>6621.931658242086</v>
       </c>
       <c r="M58" s="18" t="n">
-        <v>7351.502747375703</v>
+        <v>7375.305354258077</v>
       </c>
       <c r="N58" s="18" t="n">
-        <v>8143.657673305763</v>
+        <v>8140.845171907678</v>
       </c>
       <c r="O58" s="18" t="n">
-        <v>8826.674622439114</v>
+        <v>8828.537310694626</v>
       </c>
     </row>
     <row r="59">
@@ -21758,40 +21758,40 @@
         </is>
       </c>
       <c r="D59" s="18" t="n">
-        <v>131.4447079862481</v>
+        <v>-1.13686837721616e-13</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>523.481708692738</v>
+        <v>-567.3200531857153</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>805.7555805928578</v>
+        <v>-1142.200897375476</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>867.6235716338301</v>
+        <v>-1716.852097133171</v>
       </c>
       <c r="H59" s="18" t="n">
-        <v>1131.595769596228</v>
+        <v>-2291.526141542813</v>
       </c>
       <c r="I59" s="18" t="n">
-        <v>1397.498275512869</v>
+        <v>-2866.222226229316</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>1659.394789010955</v>
+        <v>-3440.939642970784</v>
       </c>
       <c r="K59" s="18" t="n">
-        <v>2115.989427169636</v>
+        <v>-4015.679325861893</v>
       </c>
       <c r="L59" s="18" t="n">
-        <v>2281.885210114528</v>
+        <v>-4590.832261785459</v>
       </c>
       <c r="M59" s="18" t="n">
-        <v>2424.21354721451</v>
+        <v>-4590.513961351647</v>
       </c>
       <c r="N59" s="18" t="n">
-        <v>2661.768418479527</v>
+        <v>-4590.204894098125</v>
       </c>
       <c r="O59" s="18" t="n">
-        <v>2927.845270540112</v>
+        <v>-4567.576041944836</v>
       </c>
     </row>
     <row r="60">
@@ -21970,40 +21970,40 @@
         </is>
       </c>
       <c r="D63" s="18" t="n">
-        <v>16.81938125672266</v>
+        <v>-13.9175135029666</v>
       </c>
       <c r="E63" s="18" t="n">
-        <v>1.697799248630247</v>
+        <v>-1.490296973848487</v>
       </c>
       <c r="F63" s="18" t="n">
-        <v>2.157088112764882</v>
+        <v>-1.893636626296129</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>2.111398808869975</v>
+        <v>-0.1791615330298164</v>
       </c>
       <c r="H63" s="18" t="n">
-        <v>2.067318255145832</v>
+        <v>-1.781395542780828</v>
       </c>
       <c r="I63" s="18" t="n">
-        <v>2.024654145218015</v>
+        <v>-1.741368325356682</v>
       </c>
       <c r="J63" s="18" t="n">
-        <v>1.98012184593723</v>
+        <v>-1.68877303554148</v>
       </c>
       <c r="K63" s="18" t="n">
-        <v>1.153615781020211</v>
+        <v>-2.173056109980713</v>
       </c>
       <c r="L63" s="18" t="n">
-        <v>0.6366008676218513</v>
+        <v>-2.375656487495363</v>
       </c>
       <c r="M63" s="18" t="n">
-        <v>0.6181345070445268</v>
+        <v>-2.278982904582236</v>
       </c>
       <c r="N63" s="18" t="n">
-        <v>0.6032960439207606</v>
+        <v>-2.172993426208347</v>
       </c>
       <c r="O63" s="18" t="n">
-        <v>0.587351380639987</v>
+        <v>-4.060867207935981</v>
       </c>
     </row>
     <row r="64">
@@ -22023,40 +22023,40 @@
         </is>
       </c>
       <c r="D64" s="18" t="n">
-        <v>131.1189464140258</v>
+        <v>100.3820516543365</v>
       </c>
       <c r="E64" s="18" t="n">
-        <v>130.5759740646737</v>
+        <v>127.387877842195</v>
       </c>
       <c r="F64" s="18" t="n">
-        <v>148.8444361111943</v>
+        <v>144.7937113721333</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>152.3248178663257</v>
+        <v>150.0342575244259</v>
       </c>
       <c r="H64" s="18" t="n">
-        <v>169.1253155508383</v>
+        <v>165.2766017529117</v>
       </c>
       <c r="I64" s="18" t="n">
-        <v>185.5787232235269</v>
+        <v>181.8127007529522</v>
       </c>
       <c r="J64" s="18" t="n">
-        <v>201.5358320529799</v>
+        <v>197.8669371715012</v>
       </c>
       <c r="K64" s="18" t="n">
-        <v>220.8566494258443</v>
+        <v>217.5299775348434</v>
       </c>
       <c r="L64" s="18" t="n">
-        <v>242.2630565544729</v>
+        <v>239.2507991993558</v>
       </c>
       <c r="M64" s="18" t="n">
-        <v>263.3446215284549</v>
+        <v>260.4475041168282</v>
       </c>
       <c r="N64" s="18" t="n">
-        <v>283.5283080889975</v>
+        <v>280.7520186188684</v>
       </c>
       <c r="O64" s="18" t="n">
-        <v>318.828264575615</v>
+        <v>314.1800459870391</v>
       </c>
     </row>
     <row r="65">
@@ -22182,40 +22182,40 @@
         </is>
       </c>
       <c r="D67" s="18" t="n">
-        <v>-123.2478386906458</v>
+        <v>-153.9847334503351</v>
       </c>
       <c r="E67" s="18" t="n">
-        <v>-167.8140606632397</v>
+        <v>-171.0021568857184</v>
       </c>
       <c r="F67" s="18" t="n">
-        <v>-146.5649982694397</v>
+        <v>-150.6157230085008</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>-140.1288221705022</v>
+        <v>-142.419382512402</v>
       </c>
       <c r="H67" s="18" t="n">
-        <v>-120.4070880856212</v>
+        <v>-124.2558018835478</v>
       </c>
       <c r="I67" s="18" t="n">
-        <v>-101.0567563765681</v>
+        <v>-104.8227788471428</v>
       </c>
       <c r="J67" s="18" t="n">
-        <v>-89.97699434927347</v>
+        <v>-93.64588923075218</v>
       </c>
       <c r="K67" s="18" t="n">
-        <v>-75.45339389482191</v>
+        <v>-78.78006578582284</v>
       </c>
       <c r="L67" s="18" t="n">
-        <v>-51.08298633298654</v>
+        <v>-54.09524368810372</v>
       </c>
       <c r="M67" s="18" t="n">
-        <v>-27.06876093013</v>
+        <v>-29.96587834175676</v>
       </c>
       <c r="N67" s="18" t="n">
-        <v>-3.979652626001496</v>
+        <v>-6.755942096130582</v>
       </c>
       <c r="O67" s="18" t="n">
-        <v>111.9109898487174</v>
+        <v>107.2627712601415</v>
       </c>
     </row>
     <row r="68">
@@ -22480,7 +22480,7 @@
         <v>0</v>
       </c>
       <c r="O72" s="18" t="n">
-        <v>-111.9109898487174</v>
+        <v>-107.2627712601415</v>
       </c>
     </row>
     <row r="73">
@@ -22556,37 +22556,37 @@
         <v>837.425081911384</v>
       </c>
       <c r="E74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="F74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="H74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="I74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="J74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="K74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="L74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="M74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="N74" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
       <c r="O74" s="18" t="n">
-        <v>725.5140920626666</v>
+        <v>-107.2627712601415</v>
       </c>
     </row>
     <row r="75">
@@ -22606,40 +22606,40 @@
         </is>
       </c>
       <c r="D75" s="18" t="n">
-        <v>714.1772432207383</v>
+        <v>683.440348461049</v>
       </c>
       <c r="E75" s="18" t="n">
-        <v>669.6110212481444</v>
+        <v>-171.0021568857184</v>
       </c>
       <c r="F75" s="18" t="n">
-        <v>690.8600836419444</v>
+        <v>-150.6157230085008</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>697.2962597408819</v>
+        <v>-142.419382512402</v>
       </c>
       <c r="H75" s="18" t="n">
-        <v>717.0179938257629</v>
+        <v>-124.2558018835478</v>
       </c>
       <c r="I75" s="18" t="n">
-        <v>736.368325534816</v>
+        <v>-104.8227788471428</v>
       </c>
       <c r="J75" s="18" t="n">
-        <v>747.4480875621106</v>
+        <v>-93.64588923075218</v>
       </c>
       <c r="K75" s="18" t="n">
-        <v>761.9716880165621</v>
+        <v>-78.78006578582284</v>
       </c>
       <c r="L75" s="18" t="n">
-        <v>786.3420955783974</v>
+        <v>-54.09524368810372</v>
       </c>
       <c r="M75" s="18" t="n">
-        <v>810.356320981254</v>
+        <v>-29.96587834175676</v>
       </c>
       <c r="N75" s="18" t="n">
-        <v>833.4454292853825</v>
+        <v>-6.755942096130582</v>
       </c>
       <c r="O75" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -22662,37 +22662,37 @@
         <v>0</v>
       </c>
       <c r="E76" s="18" t="n">
-        <v>714.1772432207383</v>
+        <v>683.440348461049</v>
       </c>
       <c r="F76" s="18" t="n">
-        <v>1383.788264468883</v>
+        <v>520.8478822036918</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>2074.648348110827</v>
+        <v>371.0810588195063</v>
       </c>
       <c r="H76" s="18" t="n">
-        <v>2771.944607851709</v>
+        <v>229.7402203634867</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>3488.962601677472</v>
+        <v>106.5401178843739</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>4225.330927212288</v>
+        <v>2.750998164803988</v>
       </c>
       <c r="K76" s="18" t="n">
-        <v>4972.779014774398</v>
+        <v>-89.88256399333916</v>
       </c>
       <c r="L76" s="18" t="n">
-        <v>5734.750702790961</v>
+        <v>-167.6725688561934</v>
       </c>
       <c r="M76" s="18" t="n">
-        <v>6521.092798369359</v>
+        <v>-221.191004653787</v>
       </c>
       <c r="N76" s="18" t="n">
-        <v>7331.449119350613</v>
+        <v>324.8911612523441</v>
       </c>
       <c r="O76" s="18" t="n">
-        <v>8164.894548635995</v>
+        <v>894.1740302238113</v>
       </c>
     </row>
     <row r="77">
@@ -22712,40 +22712,40 @@
         </is>
       </c>
       <c r="D77" s="18" t="n">
-        <v>714.1772432207383</v>
+        <v>683.440348461049</v>
       </c>
       <c r="E77" s="18" t="n">
-        <v>669.6110212481444</v>
+        <v>-171.0021568857184</v>
       </c>
       <c r="F77" s="18" t="n">
-        <v>690.8600836419444</v>
+        <v>-150.6157230085008</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>697.2962597408819</v>
+        <v>-142.419382512402</v>
       </c>
       <c r="H77" s="18" t="n">
-        <v>717.0179938257629</v>
+        <v>-124.2558018835478</v>
       </c>
       <c r="I77" s="18" t="n">
-        <v>736.368325534816</v>
+        <v>-104.8227788471428</v>
       </c>
       <c r="J77" s="18" t="n">
-        <v>747.4480875621106</v>
+        <v>-93.64588923075218</v>
       </c>
       <c r="K77" s="18" t="n">
-        <v>761.9716880165621</v>
+        <v>-78.78006578582284</v>
       </c>
       <c r="L77" s="18" t="n">
-        <v>786.3420955783974</v>
+        <v>-54.09524368810372</v>
       </c>
       <c r="M77" s="18" t="n">
-        <v>810.356320981254</v>
+        <v>-29.96587834175676</v>
       </c>
       <c r="N77" s="18" t="n">
-        <v>833.4454292853825</v>
+        <v>-6.755942096130582</v>
       </c>
       <c r="O77" s="18" t="n">
-        <v>837.425081911384</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -22765,40 +22765,40 @@
         </is>
       </c>
       <c r="D78" s="18" t="n">
-        <v>714.1772432207383</v>
+        <v>683.440348461049</v>
       </c>
       <c r="E78" s="18" t="n">
-        <v>1383.788264468883</v>
+        <v>520.8478822036918</v>
       </c>
       <c r="F78" s="18" t="n">
-        <v>2074.648348110827</v>
+        <v>371.0810588195063</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>2771.944607851709</v>
+        <v>229.7402203634867</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>3488.962601677472</v>
+        <v>106.5401178843739</v>
       </c>
       <c r="I78" s="18" t="n">
-        <v>4225.330927212288</v>
+        <v>2.750998164803988</v>
       </c>
       <c r="J78" s="18" t="n">
-        <v>4972.779014774398</v>
+        <v>-89.88256399333916</v>
       </c>
       <c r="K78" s="18" t="n">
-        <v>5734.750702790961</v>
+        <v>-167.6725688561934</v>
       </c>
       <c r="L78" s="18" t="n">
-        <v>6521.092798369359</v>
+        <v>-221.191004653787</v>
       </c>
       <c r="M78" s="18" t="n">
-        <v>7331.449119350613</v>
+        <v>324.8911612523441</v>
       </c>
       <c r="N78" s="18" t="n">
-        <v>8164.894548635995</v>
+        <v>894.1740302238113</v>
       </c>
       <c r="O78" s="18" t="n">
-        <v>9002.319630547379</v>
+        <v>1492.532626191176</v>
       </c>
     </row>
     <row r="79">
@@ -23295,40 +23295,40 @@
         </is>
       </c>
       <c r="D88" s="18" t="n">
-        <v>-8.409690628361332</v>
+        <v>0</v>
       </c>
       <c r="E88" s="18" t="n">
-        <v>-9.258590252676456</v>
+        <v>0</v>
       </c>
       <c r="F88" s="18" t="n">
-        <v>-10.3371343090589</v>
+        <v>0</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>-11.39283371349388</v>
+        <v>0</v>
       </c>
       <c r="H88" s="18" t="n">
-        <v>-12.4264928410668</v>
+        <v>0</v>
       </c>
       <c r="I88" s="18" t="n">
-        <v>-13.43881991367581</v>
+        <v>0</v>
       </c>
       <c r="J88" s="18" t="n">
-        <v>-14.42888083664442</v>
+        <v>0</v>
       </c>
       <c r="K88" s="18" t="n">
-        <v>-15.00568872715453</v>
+        <v>0</v>
       </c>
       <c r="L88" s="18" t="n">
-        <v>-15.32398916096545</v>
+        <v>0</v>
       </c>
       <c r="M88" s="18" t="n">
-        <v>-15.63305641448772</v>
+        <v>0</v>
       </c>
       <c r="N88" s="18" t="n">
-        <v>-15.9347044364481</v>
+        <v>0</v>
       </c>
       <c r="O88" s="18" t="n">
-        <v>-16.22838012676809</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
@@ -23401,40 +23401,40 @@
         </is>
       </c>
       <c r="D90" s="18" t="n">
-        <v>-16.81938125672266</v>
+        <v>13.9175135029666</v>
       </c>
       <c r="E90" s="18" t="n">
-        <v>-18.51718050535291</v>
+        <v>15.40781047681508</v>
       </c>
       <c r="F90" s="18" t="n">
-        <v>-20.67426861811779</v>
+        <v>17.30144710311121</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>-22.78566742698777</v>
+        <v>17.48060863614103</v>
       </c>
       <c r="H90" s="18" t="n">
-        <v>-24.8529856821336</v>
+        <v>19.26200417892186</v>
       </c>
       <c r="I90" s="18" t="n">
-        <v>-26.87763982735162</v>
+        <v>21.00337250427854</v>
       </c>
       <c r="J90" s="18" t="n">
-        <v>-28.85776167328885</v>
+        <v>22.69214553982002</v>
       </c>
       <c r="K90" s="18" t="n">
-        <v>-30.01137745430906</v>
+        <v>24.86520164980073</v>
       </c>
       <c r="L90" s="18" t="n">
-        <v>-30.64797832193091</v>
+        <v>27.24085813729609</v>
       </c>
       <c r="M90" s="18" t="n">
-        <v>-31.26611282897543</v>
+        <v>29.51984104187833</v>
       </c>
       <c r="N90" s="18" t="n">
-        <v>-31.86940887289619</v>
+        <v>31.69283446808668</v>
       </c>
       <c r="O90" s="18" t="n">
-        <v>-32.45676025353618</v>
+        <v>35.75370167602266</v>
       </c>
     </row>
     <row r="91">
@@ -23454,40 +23454,40 @@
         </is>
       </c>
       <c r="D91" s="18" t="n">
-        <v>-16.81938125672266</v>
+        <v>13.9175135029666</v>
       </c>
       <c r="E91" s="18" t="n">
-        <v>-1.697799248630247</v>
+        <v>1.490296973848487</v>
       </c>
       <c r="F91" s="18" t="n">
-        <v>-2.157088112764882</v>
+        <v>1.893636626296129</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>-2.111398808869975</v>
+        <v>0.1791615330298164</v>
       </c>
       <c r="H91" s="18" t="n">
-        <v>-2.067318255145832</v>
+        <v>1.781395542780828</v>
       </c>
       <c r="I91" s="18" t="n">
-        <v>-2.024654145218015</v>
+        <v>1.741368325356682</v>
       </c>
       <c r="J91" s="18" t="n">
-        <v>-1.98012184593723</v>
+        <v>1.68877303554148</v>
       </c>
       <c r="K91" s="18" t="n">
-        <v>-1.153615781020211</v>
+        <v>2.173056109980713</v>
       </c>
       <c r="L91" s="18" t="n">
-        <v>-0.6366008676218513</v>
+        <v>2.375656487495363</v>
       </c>
       <c r="M91" s="18" t="n">
-        <v>-0.6181345070445268</v>
+        <v>2.278982904582236</v>
       </c>
       <c r="N91" s="18" t="n">
-        <v>-0.6032960439207606</v>
+        <v>2.172993426208347</v>
       </c>
       <c r="O91" s="18" t="n">
-        <v>-0.587351380639987</v>
+        <v>4.060867207935981</v>
       </c>
     </row>
     <row r="92">
@@ -23749,34 +23749,34 @@
         <v>431.8204126588831</v>
       </c>
       <c r="F96" s="20" t="n">
-        <v>989.2340429882775</v>
+        <v>618.4212010360498</v>
       </c>
       <c r="G96" s="20" t="n">
-        <v>1573.58745026985</v>
+        <v>813.0768042092966</v>
       </c>
       <c r="H96" s="20" t="n">
-        <v>2150.530323689589</v>
+        <v>1001.600482556675</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>2534.973877546137</v>
+        <v>1197.408440298696</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>3125.693051381911</v>
+        <v>1400.246613867372</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>3527.335666950416</v>
+        <v>1611.800160899984</v>
       </c>
       <c r="L96" s="20" t="n">
-        <v>4137.367616072798</v>
+        <v>1836.428768312998</v>
       </c>
       <c r="M96" s="20" t="n">
-        <v>4683.94707092508</v>
+        <v>2000.769718568507</v>
       </c>
       <c r="N96" s="20" t="n">
-        <v>5148.191785509123</v>
+        <v>2178.104603516901</v>
       </c>
       <c r="O96" s="20" t="n">
-        <v>5597.98366476403</v>
+        <v>2367.613029330465</v>
       </c>
     </row>
     <row r="97">
@@ -23935,7 +23935,7 @@
         <v>0</v>
       </c>
       <c r="O99" s="20" t="n">
-        <v>111.9109898487174</v>
+        <v>107.2627712601415</v>
       </c>
     </row>
     <row r="100">
@@ -23958,37 +23958,37 @@
         <v>431.8204126588831</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>989.2340429882775</v>
+        <v>618.4212010360498</v>
       </c>
       <c r="F100" s="20" t="n">
-        <v>1573.58745026985</v>
+        <v>813.0768042092966</v>
       </c>
       <c r="G100" s="20" t="n">
-        <v>2150.530323689589</v>
+        <v>1001.600482556675</v>
       </c>
       <c r="H100" s="20" t="n">
-        <v>2534.973877546137</v>
+        <v>1197.408440298696</v>
       </c>
       <c r="I100" s="20" t="n">
-        <v>3125.693051381911</v>
+        <v>1400.246613867372</v>
       </c>
       <c r="J100" s="20" t="n">
-        <v>3527.335666950416</v>
+        <v>1611.800160899984</v>
       </c>
       <c r="K100" s="20" t="n">
-        <v>4137.367616072798</v>
+        <v>1836.428768312998</v>
       </c>
       <c r="L100" s="20" t="n">
-        <v>4683.94707092508</v>
+        <v>2000.769718568507</v>
       </c>
       <c r="M100" s="20" t="n">
-        <v>5148.191785509123</v>
+        <v>2178.104603516901</v>
       </c>
       <c r="N100" s="20" t="n">
-        <v>5597.98366476403</v>
+        <v>2367.613029330465</v>
       </c>
       <c r="O100" s="20" t="n">
-        <v>6189.120866510628</v>
+        <v>2693.8072911333</v>
       </c>
     </row>
     <row r="101">
@@ -24117,37 +24117,37 @@
         <v>0</v>
       </c>
       <c r="E103" s="18" t="n">
-        <v>403.0672224090362</v>
+        <v>512.1847262639563</v>
       </c>
       <c r="F103" s="18" t="n">
-        <v>776.2517489414683</v>
+        <v>1013.371718807407</v>
       </c>
       <c r="G103" s="18" t="n">
-        <v>1151.459487628153</v>
+        <v>1515.303314469146</v>
       </c>
       <c r="H103" s="18" t="n">
-        <v>1727.18923144223</v>
+        <v>2017.973316300442</v>
       </c>
       <c r="I103" s="18" t="n">
-        <v>2104.403344129146</v>
+        <v>2521.373091157147</v>
       </c>
       <c r="J103" s="18" t="n">
-        <v>2680.133087943223</v>
+        <v>3025.49656540981</v>
       </c>
       <c r="K103" s="18" t="n">
-        <v>3059.330116922845</v>
+        <v>3528.401598001493</v>
       </c>
       <c r="L103" s="18" t="n">
-        <v>3440.49355912042</v>
+        <v>4030.108206698536</v>
       </c>
       <c r="M103" s="18" t="n">
-        <v>3991.008811396158</v>
+        <v>4605.837950512612</v>
       </c>
       <c r="N103" s="18" t="n">
-        <v>4568.150439866198</v>
+        <v>5181.567694326689</v>
       </c>
       <c r="O103" s="18" t="n">
-        <v>5145.280800422396</v>
+        <v>5757.297438140766</v>
       </c>
     </row>
     <row r="104">
@@ -24326,40 +24326,40 @@
         </is>
       </c>
       <c r="D107" s="18" t="n">
-        <v>403.0672224090362</v>
+        <v>512.1847262639563</v>
       </c>
       <c r="E107" s="18" t="n">
-        <v>776.2517489414683</v>
+        <v>1013.371718807407</v>
       </c>
       <c r="F107" s="18" t="n">
-        <v>1151.459487628153</v>
+        <v>1515.303314469146</v>
       </c>
       <c r="G107" s="18" t="n">
-        <v>1727.18923144223</v>
+        <v>2017.973316300442</v>
       </c>
       <c r="H107" s="18" t="n">
-        <v>2104.403344129146</v>
+        <v>2521.373091157147</v>
       </c>
       <c r="I107" s="18" t="n">
-        <v>2680.133087943223</v>
+        <v>3025.49656540981</v>
       </c>
       <c r="J107" s="18" t="n">
-        <v>3059.330116922845</v>
+        <v>3528.401598001493</v>
       </c>
       <c r="K107" s="18" t="n">
-        <v>3440.49355912042</v>
+        <v>4030.108206698536</v>
       </c>
       <c r="L107" s="18" t="n">
-        <v>3991.008811396158</v>
+        <v>4605.837950512612</v>
       </c>
       <c r="M107" s="18" t="n">
-        <v>4568.150439866198</v>
+        <v>5181.567694326689</v>
       </c>
       <c r="N107" s="18" t="n">
-        <v>5145.280800422396</v>
+        <v>5757.297438140766</v>
       </c>
       <c r="O107" s="18" t="n">
-        <v>5722.395457827415</v>
+        <v>6333.027181954842</v>
       </c>
     </row>
     <row r="108">

</xml_diff>